<commit_message>
fix: standardise factor betas before HRP distance matrix — improves ERP concentration from 53.7% to 42.0%
</commit_message>
<xml_diff>
--- a/analytics_report.xlsx
+++ b/analytics_report.xlsx
@@ -1063,7 +1063,7 @@
     <row r="4" ht="36" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Key Finding: A conventional 60/40 portfolio allocates 80.6% of total risk to Equity Premium. Enhanced HRP reduces this to 53.7% — a 26.9 pp reduction — while maintaining balanced systematic risk exposure across all five factors.</t>
+          <t>Key Finding: A conventional 60/40 portfolio allocates 80.6% of total risk to Equity Premium. Enhanced HRP reduces this to 53.5% — a 27.1 pp reduction — while maintaining balanced systematic risk exposure across all five factors.</t>
         </is>
       </c>
     </row>
@@ -1122,10 +1122,10 @@
         <v>0.06499352425022978</v>
       </c>
       <c r="C8" s="9" t="n">
-        <v>0.103933893388768</v>
+        <v>0.1035710907401094</v>
       </c>
       <c r="D8" s="10" t="n">
-        <v>0.6253352215635706</v>
+        <v>0.6275257292917561</v>
       </c>
       <c r="E8" s="9" t="n">
         <v>-0.2929242982373964</v>
@@ -1163,19 +1163,19 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>0.07259324631852983</v>
+        <v>0.07315951727129665</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>0.08535481917334327</v>
+        <v>0.08814883647169915</v>
       </c>
       <c r="D10" s="10" t="n">
-        <v>0.8504879633228848</v>
+        <v>0.8299544293450211</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>-0.1928735338745831</v>
+        <v>-0.1999559307284849</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>0.3763774368635456</v>
+        <v>0.3658782062865548</v>
       </c>
     </row>
     <row r="11">
@@ -1185,19 +1185,19 @@
         </is>
       </c>
       <c r="B11" s="12" t="n">
-        <v>0.05887012446950701</v>
+        <v>0.05891136643505969</v>
       </c>
       <c r="C11" s="12" t="n">
-        <v>0.06937777317283109</v>
+        <v>0.06931186561532281</v>
       </c>
       <c r="D11" s="13" t="n">
-        <v>0.8485444513021793</v>
+        <v>0.8499463390873745</v>
       </c>
       <c r="E11" s="12" t="n">
-        <v>-0.1655628692696721</v>
+        <v>-0.1665091655061419</v>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.3555756476629925</v>
+        <v>0.35380254447847</v>
       </c>
     </row>
     <row r="12">
@@ -1207,19 +1207,19 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>0.05339171285866526</v>
+        <v>0.05341435110809257</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>0.06192652692456322</v>
+        <v>0.06196353510197526</v>
       </c>
       <c r="D12" s="10" t="n">
-        <v>0.8621783831621175</v>
+        <v>0.8620287887091489</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>-0.1474522132085342</v>
+        <v>-0.1548283411757465</v>
       </c>
       <c r="F12" s="10" t="n">
-        <v>0.3620950252076314</v>
+        <v>0.3449907859405511</v>
       </c>
     </row>
     <row r="13" ht="8" customHeight="1"/>
@@ -1279,22 +1279,22 @@
         </is>
       </c>
       <c r="B16" s="14" t="n">
-        <v>0.6459999999999999</v>
+        <v>0.6509999999999999</v>
       </c>
       <c r="C16" s="9" t="n">
-        <v>-0.057</v>
+        <v>-0.05599999999999999</v>
       </c>
       <c r="D16" s="9" t="n">
-        <v>0.138</v>
+        <v>0.131</v>
       </c>
       <c r="E16" s="9" t="n">
+        <v>0.133</v>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="G16" s="9" t="n">
         <v>0.135</v>
-      </c>
-      <c r="F16" s="9" t="n">
-        <v>0.004</v>
-      </c>
-      <c r="G16" s="9" t="n">
-        <v>0.133</v>
       </c>
     </row>
     <row r="17">
@@ -1329,22 +1329,22 @@
         </is>
       </c>
       <c r="B18" s="16" t="n">
-        <v>0.423</v>
+        <v>0.414</v>
       </c>
       <c r="C18" s="9" t="n">
-        <v>0.182</v>
+        <v>0.191</v>
       </c>
       <c r="D18" s="9" t="n">
-        <v>0.149</v>
+        <v>0.113</v>
       </c>
       <c r="E18" s="9" t="n">
-        <v>0.014</v>
+        <v>0.015</v>
       </c>
       <c r="F18" s="9" t="n">
-        <v>-0.004</v>
+        <v>0.016</v>
       </c>
       <c r="G18" s="9" t="n">
-        <v>0.236</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="19">
@@ -1354,22 +1354,22 @@
         </is>
       </c>
       <c r="B19" s="17" t="n">
-        <v>0.484</v>
+        <v>0.487</v>
       </c>
       <c r="C19" s="12" t="n">
         <v>0.144</v>
       </c>
       <c r="D19" s="12" t="n">
-        <v>0.081</v>
+        <v>0.07400000000000001</v>
       </c>
       <c r="E19" s="12" t="n">
-        <v>0.119</v>
+        <v>0.118</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>0.009000000000000001</v>
+        <v>0.011</v>
       </c>
       <c r="G19" s="12" t="n">
-        <v>0.163</v>
+        <v>0.166</v>
       </c>
     </row>
     <row r="20">
@@ -1379,19 +1379,19 @@
         </is>
       </c>
       <c r="B20" s="16" t="n">
-        <v>0.537</v>
+        <v>0.535</v>
       </c>
       <c r="C20" s="9" t="n">
-        <v>0.079</v>
+        <v>0.12</v>
       </c>
       <c r="D20" s="9" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.055</v>
       </c>
       <c r="E20" s="9" t="n">
-        <v>0.18</v>
+        <v>0.154</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>0.008</v>
+        <v>0.01</v>
       </c>
       <c r="G20" s="9" t="n">
         <v>0.126</v>
@@ -1769,7 +1769,7 @@
       </c>
       <c r="I4" s="22" t="inlineStr">
         <is>
-          <t>BAA-Treasury</t>
+          <t>Pastor-Stambaugh</t>
         </is>
       </c>
     </row>
@@ -2044,29 +2044,29 @@
         </is>
       </c>
       <c r="B13" s="24" t="n">
-        <v>0.2662432244803207</v>
+        <v>0.2662615280266115</v>
       </c>
       <c r="C13" s="24" t="n">
-        <v>0.0341347995858011</v>
+        <v>0.03413008712923776</v>
       </c>
       <c r="D13" s="24" t="n">
-        <v>0.5391575995605099</v>
+        <v>0.2697224940806349</v>
       </c>
       <c r="E13" s="24" t="n">
-        <v>2.056026830782021</v>
+        <v>2.055745923262592</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>4.765761280351057e-05</v>
+        <v>0.01290119732786036</v>
       </c>
       <c r="G13" s="9" t="n">
         <v>0</v>
       </c>
       <c r="H13" s="16" t="n">
-        <v>0.7410349255498354</v>
+        <v>0.7443129475785015</v>
       </c>
       <c r="I13" s="19" t="inlineStr">
         <is>
-          <t>Pastor-Stambaugh</t>
+          <t>BAA-Treasury</t>
         </is>
       </c>
     </row>
@@ -2077,25 +2077,25 @@
         </is>
       </c>
       <c r="B14" s="25" t="n">
-        <v>0.3781411783147733</v>
+        <v>0.3475645787692835</v>
       </c>
       <c r="C14" s="25" t="n">
-        <v>-0.02576702956354728</v>
+        <v>-0.01789473558713058</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>3.501487241418954</v>
+        <v>1.510698166693959</v>
       </c>
       <c r="E14" s="25" t="n">
-        <v>4.00553283690104</v>
+        <v>4.474796912527248</v>
       </c>
       <c r="F14" s="25" t="n">
-        <v>-0.079613410364969</v>
+        <v>0.07225876810085358</v>
       </c>
       <c r="G14" s="12" t="n">
         <v>0</v>
       </c>
       <c r="H14" s="26" t="n">
-        <v>0.4486981761189008</v>
+        <v>0.4472956521780461</v>
       </c>
       <c r="I14" s="22" t="inlineStr">
         <is>
@@ -2110,25 +2110,25 @@
         </is>
       </c>
       <c r="B15" s="24" t="n">
-        <v>-0.09523920864949073</v>
+        <v>-0.0422572163933037</v>
       </c>
       <c r="C15" s="24" t="n">
-        <v>0.2661804770866193</v>
+        <v>0.2525396594451277</v>
       </c>
       <c r="D15" s="24" t="n">
-        <v>-0.8150509820184776</v>
+        <v>0.008416326420867809</v>
       </c>
       <c r="E15" s="24" t="n">
-        <v>14.24918935918608</v>
+        <v>13.43606605605533</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>0.1379511506886197</v>
+        <v>0.0004025644516642721</v>
       </c>
       <c r="G15" s="9" t="n">
         <v>0</v>
       </c>
       <c r="H15" s="27" t="n">
-        <v>0.08883108523880501</v>
+        <v>0.08716459731266091</v>
       </c>
       <c r="I15" s="19" t="inlineStr">
         <is>
@@ -2203,13 +2203,13 @@
         </is>
       </c>
       <c r="B20" s="25" t="n">
-        <v>-0.09523920864949073</v>
+        <v>-0.0422572163933037</v>
       </c>
       <c r="C20" s="25" t="n">
         <v>0.1943926134830137</v>
       </c>
       <c r="D20" s="29" t="n">
-        <v>0.2896318221325044</v>
+        <v>0.2366498298763174</v>
       </c>
       <c r="E20" s="22" t="inlineStr">
         <is>
@@ -2367,17 +2367,17 @@
     <row r="28">
       <c r="A28" s="21" t="inlineStr">
         <is>
-          <t>Hedge Funds</t>
+          <t>Private Equity</t>
         </is>
       </c>
       <c r="B28" s="25" t="n">
-        <v>0.2662432244803207</v>
+        <v>0.3475645787692835</v>
       </c>
       <c r="C28" s="25" t="n">
-        <v>0.1884016479536835</v>
+        <v>0.2923064843573329</v>
       </c>
       <c r="D28" s="25" t="n">
-        <v>-0.0778415765266372</v>
+        <v>-0.05525809441195068</v>
       </c>
       <c r="E28" s="22" t="inlineStr">
         <is>
@@ -2388,17 +2388,17 @@
     <row r="29">
       <c r="A29" s="18" t="inlineStr">
         <is>
-          <t>Private Equity</t>
+          <t>Hedge Funds</t>
         </is>
       </c>
       <c r="B29" s="24" t="n">
-        <v>0.3781411783147733</v>
+        <v>0.2662615280266115</v>
       </c>
       <c r="C29" s="24" t="n">
-        <v>0.2923064843573329</v>
+        <v>0.1884016479536835</v>
       </c>
       <c r="D29" s="24" t="n">
-        <v>-0.08583469395744048</v>
+        <v>-0.07785988007292804</v>
       </c>
       <c r="E29" s="19" t="inlineStr">
         <is>
@@ -2559,16 +2559,16 @@
         </is>
       </c>
       <c r="B5" s="32" t="n">
-        <v>-0.1707478688334095</v>
+        <v>-0.1830486748285078</v>
       </c>
       <c r="C5" s="34" t="n">
-        <v>0.03872490298258668</v>
+        <v>0.03683695337861703</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>-0.1712081342323609</v>
+        <v>-0.1786484994678725</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>0.5170788305191565</v>
+        <v>0.5145573060842727</v>
       </c>
     </row>
     <row r="6">
@@ -2578,16 +2578,16 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>-0.165562869269672</v>
+        <v>-0.1665091655061418</v>
       </c>
       <c r="C6" s="35" t="n">
-        <v>0.02027652275640524</v>
+        <v>0.01971956610018144</v>
       </c>
       <c r="D6" s="15" t="n">
-        <v>-0.1453856043342324</v>
+        <v>-0.1449286097236309</v>
       </c>
       <c r="E6" s="12" t="n">
-        <v>0.3376660928596036</v>
+        <v>0.3378735970052109</v>
       </c>
     </row>
     <row r="7">
@@ -2597,16 +2597,16 @@
         </is>
       </c>
       <c r="B7" s="32" t="n">
-        <v>-0.1282847277566882</v>
+        <v>-0.1257176000642428</v>
       </c>
       <c r="C7" s="34" t="n">
-        <v>0.02133537724781642</v>
+        <v>0.02542692133678326</v>
       </c>
       <c r="D7" s="32" t="n">
-        <v>-0.1234846833593276</v>
+        <v>-0.130784375396225</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>0.3290722039952829</v>
+        <v>0.322990144323839</v>
       </c>
     </row>
     <row r="8" ht="8" customHeight="1"/>
@@ -2989,13 +2989,13 @@
         <v>0.07692307692307693</v>
       </c>
       <c r="C4" s="24" t="n">
-        <v>0.07607196940227982</v>
+        <v>0.07604848222125912</v>
       </c>
       <c r="D4" s="24" t="n">
-        <v>0.005851689954021525</v>
+        <v>0.005849883247789163</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>0.112604074825391</v>
+        <v>0.1129636311829188</v>
       </c>
       <c r="F4" s="9" t="n">
         <v>0.9718498340506938</v>
@@ -3011,13 +3011,13 @@
         <v>0.07692307692307693</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>0.08675677475134909</v>
+        <v>0.08671094150982253</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>0.006673598057796084</v>
+        <v>0.006670072423832503</v>
       </c>
       <c r="E5" s="12" t="n">
-        <v>0.1284200531742476</v>
+        <v>0.1288018186574803</v>
       </c>
       <c r="F5" s="12" t="n">
         <v>0.9005695345361184</v>
@@ -3033,13 +3033,13 @@
         <v>0.07692307692307693</v>
       </c>
       <c r="C6" s="24" t="n">
-        <v>0.09162450191385201</v>
+        <v>0.09160479264684691</v>
       </c>
       <c r="D6" s="24" t="n">
-        <v>0.007048038608757847</v>
+        <v>0.007046522511295917</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>0.1356254130189165</v>
+        <v>0.1360712233682608</v>
       </c>
       <c r="F6" s="9" t="n">
         <v>0.8647852106386994</v>
@@ -3055,13 +3055,13 @@
         <v>0.07692307692307693</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>0.08990837169539805</v>
+        <v>0.08975643374929827</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>0.006916028591953696</v>
+        <v>0.006904341057638329</v>
       </c>
       <c r="E7" s="12" t="n">
-        <v>0.1330851441518518</v>
+        <v>0.1333256415144526</v>
       </c>
       <c r="F7" s="12" t="n">
         <v>0.6547256214279519</v>
@@ -3077,13 +3077,13 @@
         <v>0.07692307692307693</v>
       </c>
       <c r="C8" s="24" t="n">
-        <v>-0.01920475065096846</v>
+        <v>-0.01890725699586819</v>
       </c>
       <c r="D8" s="24" t="n">
-        <v>-0.001477288511612959</v>
+        <v>-0.001454404384297553</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>-0.02842746410138056</v>
+        <v>-0.02808514178820586</v>
       </c>
       <c r="F8" s="9" t="n">
         <v>0.9800395309996239</v>
@@ -3099,13 +3099,13 @@
         <v>0.07692307692307693</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>0.009918762478838109</v>
+        <v>0.009951105476017614</v>
       </c>
       <c r="D9" s="25" t="n">
-        <v>0.000762981729141393</v>
+        <v>0.000765469652001355</v>
       </c>
       <c r="E9" s="12" t="n">
-        <v>0.01468205807103628</v>
+        <v>0.0147815311498871</v>
       </c>
       <c r="F9" s="12" t="n">
         <v>0.8261546883028914</v>
@@ -3121,13 +3121,13 @@
         <v>0.07692307692307693</v>
       </c>
       <c r="C10" s="24" t="n">
-        <v>0.01580566601010246</v>
+        <v>0.01592770997060341</v>
       </c>
       <c r="D10" s="24" t="n">
-        <v>0.001215820462315574</v>
+        <v>0.001225208459277185</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>0.02339603420354434</v>
+        <v>0.0236592750066058</v>
       </c>
       <c r="F10" s="9" t="n">
         <v>0.6542475111182804</v>
@@ -3143,13 +3143,13 @@
         <v>0.07692307692307693</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>0.088058047076991</v>
+        <v>0.08804865704708366</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>0.006773695928999308</v>
+        <v>0.006772973619006435</v>
       </c>
       <c r="E11" s="12" t="n">
-        <v>0.1303462365960271</v>
+        <v>0.1307888827009042</v>
       </c>
       <c r="F11" s="12" t="n">
         <v>0.6432514443485702</v>
@@ -3165,13 +3165,13 @@
         <v>0.07692307692307693</v>
       </c>
       <c r="C12" s="24" t="n">
-        <v>0.07546337026810851</v>
+        <v>0.075133417224411</v>
       </c>
       <c r="D12" s="24" t="n">
-        <v>0.005804874636008347</v>
+        <v>0.005779493632647</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>0.1117032076205407</v>
+        <v>0.1116043790086071</v>
       </c>
       <c r="F12" s="9" t="n">
         <v>0.4797912934834942</v>
@@ -3187,13 +3187,13 @@
         <v>0.07692307692307693</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>0.03964930468724968</v>
+        <v>0.03992411329824733</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>0.003049946514403822</v>
+        <v>0.003071085638326718</v>
       </c>
       <c r="E13" s="12" t="n">
-        <v>0.05869012340364081</v>
+        <v>0.05930391610981455</v>
       </c>
       <c r="F13" s="12" t="n">
         <v>0.6813173339403511</v>
@@ -3209,16 +3209,16 @@
         <v>0.07692307692307693</v>
       </c>
       <c r="C14" s="24" t="n">
-        <v>0.02771691210987172</v>
+        <v>0.02736526641155149</v>
       </c>
       <c r="D14" s="24" t="n">
-        <v>0.002132070162297825</v>
+        <v>0.002105020493196269</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>0.04102742796948342</v>
+        <v>0.04064880418182309</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>0.7553246822404955</v>
+        <v>0.7487919560463553</v>
       </c>
     </row>
     <row r="15">
@@ -3231,16 +3231,16 @@
         <v>0.07692307692307693</v>
       </c>
       <c r="C15" s="25" t="n">
-        <v>0.05404604288534002</v>
+        <v>0.05235587803403794</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>0.004157387914256925</v>
+        <v>0.004027375233387534</v>
       </c>
       <c r="E15" s="12" t="n">
-        <v>0.08000061921487119</v>
+        <v>0.07777025817934881</v>
       </c>
       <c r="F15" s="12" t="n">
-        <v>0.4740803814994422</v>
+        <v>0.4284467817562574</v>
       </c>
     </row>
     <row r="16">
@@ -3253,16 +3253,16 @@
         <v>0.07692307692307693</v>
       </c>
       <c r="C16" s="24" t="n">
-        <v>0.03975533439858021</v>
+        <v>0.03929254921739969</v>
       </c>
       <c r="D16" s="24" t="n">
-        <v>0.003058102646044632</v>
+        <v>0.003022503785953823</v>
       </c>
       <c r="E16" s="9" t="n">
-        <v>0.05884707185182993</v>
+        <v>0.05836578072810264</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>0.1419427420681525</v>
+        <v>0.1297114447333514</v>
       </c>
     </row>
     <row r="18">
@@ -3539,7 +3539,7 @@
         <v>0</v>
       </c>
       <c r="C30" s="24" t="n">
-        <v>0.02622494928918073</v>
+        <v>0.02593079077558953</v>
       </c>
       <c r="D30" s="24" t="n">
         <v>0</v>
@@ -3548,7 +3548,7 @@
         <v>0</v>
       </c>
       <c r="F30" s="9" t="n">
-        <v>0.7553246822404955</v>
+        <v>0.7487919560463553</v>
       </c>
     </row>
     <row r="31">
@@ -3561,7 +3561,7 @@
         <v>0</v>
       </c>
       <c r="C31" s="25" t="n">
-        <v>0.04143923567869714</v>
+        <v>0.03961123437025107</v>
       </c>
       <c r="D31" s="25" t="n">
         <v>0</v>
@@ -3570,7 +3570,7 @@
         <v>0</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.4740803814994422</v>
+        <v>0.4284467817562574</v>
       </c>
     </row>
     <row r="32">
@@ -3583,7 +3583,7 @@
         <v>0</v>
       </c>
       <c r="C32" s="24" t="n">
-        <v>0.01650794361950855</v>
+        <v>0.01678542567237088</v>
       </c>
       <c r="D32" s="24" t="n">
         <v>0</v>
@@ -3592,7 +3592,7 @@
         <v>0</v>
       </c>
       <c r="F32" s="9" t="n">
-        <v>0.1419427420681525</v>
+        <v>0.1297114447333514</v>
       </c>
     </row>
     <row r="34">
@@ -3646,16 +3646,16 @@
         </is>
       </c>
       <c r="B36" s="9" t="n">
-        <v>1.12998593313295e-07</v>
+        <v>1.540461288441797e-08</v>
       </c>
       <c r="C36" s="24" t="n">
-        <v>0.05692767223547345</v>
+        <v>0.05604810820385786</v>
       </c>
       <c r="D36" s="24" t="n">
-        <v>6.432746883208821e-09</v>
+        <v>8.633994097844016e-10</v>
       </c>
       <c r="E36" s="9" t="n">
-        <v>1.507295533048894e-07</v>
+        <v>1.958958153830204e-08</v>
       </c>
       <c r="F36" s="9" t="n">
         <v>0.9718498340506938</v>
@@ -3668,16 +3668,16 @@
         </is>
       </c>
       <c r="B37" s="12" t="n">
-        <v>9.768383840153099e-08</v>
+        <v>1.286140172707754e-08</v>
       </c>
       <c r="C37" s="25" t="n">
-        <v>0.06081953129916644</v>
+        <v>0.05994390698587126</v>
       </c>
       <c r="D37" s="25" t="n">
-        <v>5.94108526708463e-09</v>
+        <v>7.7096266883586e-10</v>
       </c>
       <c r="E37" s="12" t="n">
-        <v>1.392091348707364e-07</v>
+        <v>1.749229370902436e-08</v>
       </c>
       <c r="F37" s="12" t="n">
         <v>0.9005695345361184</v>
@@ -3690,16 +3690,16 @@
         </is>
       </c>
       <c r="B38" s="9" t="n">
-        <v>7.870694893487945e-08</v>
+        <v>1.034391777355504e-08</v>
       </c>
       <c r="C38" s="24" t="n">
-        <v>0.06487282242693367</v>
+        <v>0.06375923942128729</v>
       </c>
       <c r="D38" s="24" t="n">
-        <v>5.105941922018171e-09</v>
+        <v>6.59520329878205e-10</v>
       </c>
       <c r="E38" s="9" t="n">
-        <v>1.196403898800077e-07</v>
+        <v>1.496378979636218e-08</v>
       </c>
       <c r="F38" s="9" t="n">
         <v>0.8647852106386994</v>
@@ -3712,16 +3712,16 @@
         </is>
       </c>
       <c r="B39" s="12" t="n">
-        <v>0.04190992908765714</v>
+        <v>0.07113737017120696</v>
       </c>
       <c r="C39" s="25" t="n">
-        <v>0.06748194017499352</v>
+        <v>0.06717134055346032</v>
       </c>
       <c r="D39" s="25" t="n">
-        <v>0.0028281633274315</v>
+        <v>0.004778392517847712</v>
       </c>
       <c r="E39" s="12" t="n">
-        <v>0.0662683924545118</v>
+        <v>0.1084164626354847</v>
       </c>
       <c r="F39" s="12" t="n">
         <v>0.6547256214279519</v>
@@ -3734,16 +3734,16 @@
         </is>
       </c>
       <c r="B40" s="9" t="n">
-        <v>0.2886613151522574</v>
+        <v>0.2963200956729828</v>
       </c>
       <c r="C40" s="24" t="n">
-        <v>0.01905394808611297</v>
+        <v>0.02027839680564917</v>
       </c>
       <c r="D40" s="24" t="n">
-        <v>0.005500137713380209</v>
+        <v>0.006008896481544672</v>
       </c>
       <c r="E40" s="9" t="n">
-        <v>0.1288770280729018</v>
+        <v>0.1363352421214062</v>
       </c>
       <c r="F40" s="9" t="n">
         <v>0.9800395309996239</v>
@@ -3756,16 +3756,16 @@
         </is>
       </c>
       <c r="B41" s="12" t="n">
-        <v>6.941451318814953e-08</v>
+        <v>9.201562116762712e-09</v>
       </c>
       <c r="C41" s="25" t="n">
-        <v>0.01501685218419754</v>
+        <v>0.01515708195138125</v>
       </c>
       <c r="D41" s="25" t="n">
-        <v>1.042387483984472e-09</v>
+        <v>1.394688310844975e-10</v>
       </c>
       <c r="E41" s="12" t="n">
-        <v>2.44248068024732e-08</v>
+        <v>3.164394146694723e-09</v>
       </c>
       <c r="F41" s="12" t="n">
         <v>0.8261546883028914</v>
@@ -3778,16 +3778,16 @@
         </is>
       </c>
       <c r="B42" s="9" t="n">
-        <v>6.965110784322271e-08</v>
+        <v>8.935097992254681e-09</v>
       </c>
       <c r="C42" s="24" t="n">
-        <v>0.02620626195947527</v>
+        <v>0.02639673412319088</v>
       </c>
       <c r="D42" s="24" t="n">
-        <v>1.825295177907157e-09</v>
+        <v>2.358574060662035e-10</v>
       </c>
       <c r="E42" s="9" t="n">
-        <v>4.276958689819837e-08</v>
+        <v>5.351344737078345e-09</v>
       </c>
       <c r="F42" s="9" t="n">
         <v>0.6542475111182804</v>
@@ -3800,16 +3800,16 @@
         </is>
       </c>
       <c r="B43" s="12" t="n">
-        <v>0.123639275433536</v>
+        <v>0.1364634563400894</v>
       </c>
       <c r="C43" s="25" t="n">
-        <v>0.08587485838092043</v>
+        <v>0.08498129605168152</v>
       </c>
       <c r="D43" s="25" t="n">
-        <v>0.01061750526817452</v>
+        <v>0.01159684138347285</v>
       </c>
       <c r="E43" s="12" t="n">
-        <v>0.2487851388124181</v>
+        <v>0.2631195565966682</v>
       </c>
       <c r="F43" s="12" t="n">
         <v>0.6432514443485702</v>
@@ -3822,16 +3822,16 @@
         </is>
       </c>
       <c r="B44" s="9" t="n">
-        <v>1.08473008170814e-07</v>
+        <v>2.096350137433955e-08</v>
       </c>
       <c r="C44" s="24" t="n">
-        <v>0.02216044177934485</v>
+        <v>0.02052878880749672</v>
       </c>
       <c r="D44" s="24" t="n">
-        <v>2.403809782199721e-09</v>
+        <v>4.303552923794839e-10</v>
       </c>
       <c r="E44" s="9" t="n">
-        <v>5.632510982930986e-08</v>
+        <v>9.764287530162754e-09</v>
       </c>
       <c r="F44" s="9" t="n">
         <v>0.4797912934834942</v>
@@ -3844,16 +3844,16 @@
         </is>
       </c>
       <c r="B45" s="12" t="n">
-        <v>0.2457889564637488</v>
+        <v>0.1960790013757596</v>
       </c>
       <c r="C45" s="25" t="n">
-        <v>0.03591803882286684</v>
+        <v>0.03660795132295001</v>
       </c>
       <c r="D45" s="25" t="n">
-        <v>0.008828257280496857</v>
+        <v>0.007178050537816457</v>
       </c>
       <c r="E45" s="12" t="n">
-        <v>0.2068601952648496</v>
+        <v>0.1628620597872786</v>
       </c>
       <c r="F45" s="12" t="n">
         <v>0.6813173339403511</v>
@@ -3866,19 +3866,19 @@
         </is>
       </c>
       <c r="B46" s="9" t="n">
-        <v>1.520208122408094e-08</v>
+        <v>1.618598277387212e-09</v>
       </c>
       <c r="C46" s="24" t="n">
-        <v>0.02034412809747743</v>
+        <v>0.02013819062703088</v>
       </c>
       <c r="D46" s="24" t="n">
-        <v>3.09273087770959e-10</v>
+        <v>3.259564065860747e-11</v>
       </c>
       <c r="E46" s="9" t="n">
-        <v>7.246763352468013e-09</v>
+        <v>7.395591811146038e-10</v>
       </c>
       <c r="F46" s="9" t="n">
-        <v>0.7553246822404955</v>
+        <v>0.7487919560463553</v>
       </c>
     </row>
     <row r="47">
@@ -3888,19 +3888,19 @@
         </is>
       </c>
       <c r="B47" s="12" t="n">
-        <v>0.2994235045579806</v>
+        <v>0.2822620050016704</v>
       </c>
       <c r="C47" s="25" t="n">
-        <v>0.04971439597402084</v>
+        <v>0.04946939446322386</v>
       </c>
       <c r="D47" s="25" t="n">
-        <v>0.01488565866952448</v>
+        <v>0.0139633304674081</v>
       </c>
       <c r="E47" s="12" t="n">
-        <v>0.3487948030044762</v>
+        <v>0.3168125871267996</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>0.4740803814994422</v>
+        <v>0.4284467817562574</v>
       </c>
     </row>
     <row r="48">
@@ -3910,19 +3910,19 @@
         </is>
       </c>
       <c r="B48" s="9" t="n">
-        <v>0.0005764671747288517</v>
+        <v>0.01773799210959868</v>
       </c>
       <c r="C48" s="24" t="n">
-        <v>0.03064227747705986</v>
+        <v>0.03094508737001762</v>
       </c>
       <c r="D48" s="24" t="n">
-        <v>1.766426712445823e-05</v>
+        <v>0.0005489037156002144</v>
       </c>
       <c r="E48" s="9" t="n">
-        <v>0.0004139020454975051</v>
+        <v>0.01245402066711213</v>
       </c>
       <c r="F48" s="9" t="n">
-        <v>0.1419427420681525</v>
+        <v>0.1297114447333514</v>
       </c>
     </row>
     <row r="50">
@@ -3976,16 +3976,16 @@
         </is>
       </c>
       <c r="B52" s="9" t="n">
-        <v>0.04237184338252779</v>
+        <v>0.04239826333525394</v>
       </c>
       <c r="C52" s="24" t="n">
-        <v>0.06297462881850684</v>
+        <v>0.06287655228620766</v>
       </c>
       <c r="D52" s="24" t="n">
-        <v>0.002668351109370593</v>
+        <v>0.002665856621443495</v>
       </c>
       <c r="E52" s="9" t="n">
-        <v>0.0769223625187077</v>
+        <v>0.07692352810812679</v>
       </c>
       <c r="F52" s="9" t="n">
         <v>0.9718498340506938</v>
@@ -3998,16 +3998,16 @@
         </is>
       </c>
       <c r="B53" s="12" t="n">
-        <v>0.03835312966778117</v>
+        <v>0.03838122897303223</v>
       </c>
       <c r="C53" s="25" t="n">
-        <v>0.06957048072837803</v>
+        <v>0.06945530211249798</v>
       </c>
       <c r="D53" s="25" t="n">
-        <v>0.002668245668425353</v>
+        <v>0.002665779853770914</v>
       </c>
       <c r="E53" s="12" t="n">
-        <v>0.07691932290125048</v>
+        <v>0.07692131297015872</v>
       </c>
       <c r="F53" s="12" t="n">
         <v>0.9005695345361184</v>
@@ -4020,16 +4020,16 @@
         </is>
       </c>
       <c r="B54" s="9" t="n">
-        <v>0.03704034967567654</v>
+        <v>0.0370534553973652</v>
       </c>
       <c r="C54" s="24" t="n">
-        <v>0.07203927821088472</v>
+        <v>0.07194606436802295</v>
       </c>
       <c r="D54" s="24" t="n">
-        <v>0.002668360055314516</v>
+        <v>0.002665850287076504</v>
       </c>
       <c r="E54" s="9" t="n">
-        <v>0.07692262040948493</v>
+        <v>0.07692334532940817</v>
       </c>
       <c r="F54" s="9" t="n">
         <v>0.8647852106386994</v>
@@ -4042,16 +4042,16 @@
         </is>
       </c>
       <c r="B55" s="12" t="n">
-        <v>0.03518145231877982</v>
+        <v>0.03526861812873507</v>
       </c>
       <c r="C55" s="25" t="n">
-        <v>0.07584687705952509</v>
+        <v>0.07558698122430509</v>
       </c>
       <c r="D55" s="25" t="n">
-        <v>0.002668403288798037</v>
+        <v>0.002665848376303883</v>
       </c>
       <c r="E55" s="12" t="n">
-        <v>0.07692386673036102</v>
+        <v>0.07692329019389554</v>
       </c>
       <c r="F55" s="12" t="n">
         <v>0.6547256214279519</v>
@@ -4064,16 +4064,16 @@
         </is>
       </c>
       <c r="B56" s="9" t="n">
-        <v>0.1916974426113651</v>
+        <v>0.1901058368847075</v>
       </c>
       <c r="C56" s="24" t="n">
-        <v>0.01391997775256079</v>
+        <v>0.01402297004707323</v>
       </c>
       <c r="D56" s="24" t="n">
-        <v>0.002668424136373002</v>
+        <v>0.002665848456408042</v>
       </c>
       <c r="E56" s="9" t="n">
-        <v>0.07692446771750751</v>
+        <v>0.07692329250530811</v>
       </c>
       <c r="F56" s="9" t="n">
         <v>0.9800395309996239</v>
@@ -4086,16 +4086,16 @@
         </is>
       </c>
       <c r="B57" s="12" t="n">
-        <v>0.1560290416425018</v>
+        <v>0.1561033628971746</v>
       </c>
       <c r="C57" s="25" t="n">
-        <v>0.01710234285391538</v>
+        <v>0.01707722545808813</v>
       </c>
       <c r="D57" s="25" t="n">
-        <v>0.002668462165337904</v>
+        <v>0.002665812322960801</v>
       </c>
       <c r="E57" s="12" t="n">
-        <v>0.07692556400420462</v>
+        <v>0.07692224987149872</v>
       </c>
       <c r="F57" s="12" t="n">
         <v>0.8261546883028914</v>
@@ -4108,16 +4108,16 @@
         </is>
       </c>
       <c r="B58" s="9" t="n">
-        <v>0.09902372157555807</v>
+        <v>0.09891989158807808</v>
       </c>
       <c r="C58" s="24" t="n">
-        <v>0.0269464453755959</v>
+        <v>0.02695041436455389</v>
       </c>
       <c r="D58" s="24" t="n">
-        <v>0.002668337304323993</v>
+        <v>0.002665932067195453</v>
       </c>
       <c r="E58" s="9" t="n">
-        <v>0.07692196455129049</v>
+        <v>0.07692570510195861</v>
       </c>
       <c r="F58" s="9" t="n">
         <v>0.6542475111182804</v>
@@ -4130,16 +4130,16 @@
         </is>
       </c>
       <c r="B59" s="12" t="n">
-        <v>0.03305541874853363</v>
+        <v>0.03310675547604956</v>
       </c>
       <c r="C59" s="25" t="n">
-        <v>0.08072243923690535</v>
+        <v>0.08052175975620807</v>
       </c>
       <c r="D59" s="25" t="n">
-        <v>0.002668314031378968</v>
+        <v>0.002665814210749988</v>
       </c>
       <c r="E59" s="12" t="n">
-        <v>0.07692129364636055</v>
+        <v>0.07692230434382234</v>
       </c>
       <c r="F59" s="12" t="n">
         <v>0.6432514443485702</v>
@@ -4152,16 +4152,16 @@
         </is>
       </c>
       <c r="B60" s="9" t="n">
-        <v>0.05433105722415058</v>
+        <v>0.05454871770448565</v>
       </c>
       <c r="C60" s="24" t="n">
-        <v>0.04911204681458394</v>
+        <v>0.04887037300574651</v>
       </c>
       <c r="D60" s="24" t="n">
-        <v>0.002668309425878322</v>
+        <v>0.002665816181203382</v>
       </c>
       <c r="E60" s="9" t="n">
-        <v>0.07692116088047792</v>
+        <v>0.07692236120142894</v>
       </c>
       <c r="F60" s="9" t="n">
         <v>0.4797912934834942</v>
@@ -4174,16 +4174,16 @@
         </is>
       </c>
       <c r="B61" s="12" t="n">
-        <v>0.07190731636107728</v>
+        <v>0.07131481415928038</v>
       </c>
       <c r="C61" s="25" t="n">
-        <v>0.03710985177866196</v>
+        <v>0.03738288332119383</v>
       </c>
       <c r="D61" s="25" t="n">
-        <v>0.002668469851960932</v>
+        <v>0.002665953376789001</v>
       </c>
       <c r="E61" s="12" t="n">
-        <v>0.0769257855916865</v>
+        <v>0.07692631999216126</v>
       </c>
       <c r="F61" s="12" t="n">
         <v>0.6813173339403511</v>
@@ -4196,19 +4196,19 @@
         </is>
       </c>
       <c r="B62" s="9" t="n">
-        <v>0.1140716492667996</v>
+        <v>0.1147079339099366</v>
       </c>
       <c r="C62" s="24" t="n">
-        <v>0.02339356683603391</v>
+        <v>0.0232394915358965</v>
       </c>
       <c r="D62" s="24" t="n">
-        <v>0.002668542751219496</v>
+        <v>0.002665754059200145</v>
       </c>
       <c r="E62" s="9" t="n">
-        <v>0.07692788710792808</v>
+        <v>0.07692056866554248</v>
       </c>
       <c r="F62" s="9" t="n">
-        <v>0.7553246822404955</v>
+        <v>0.7487919560463553</v>
       </c>
     </row>
     <row r="63">
@@ -4218,19 +4218,19 @@
         </is>
       </c>
       <c r="B63" s="12" t="n">
-        <v>0.06063975676952887</v>
+        <v>0.06079007889326719</v>
       </c>
       <c r="C63" s="25" t="n">
-        <v>0.04400585315122874</v>
+        <v>0.04385430184744837</v>
       </c>
       <c r="D63" s="25" t="n">
-        <v>0.002668504231526117</v>
+        <v>0.002665906469115539</v>
       </c>
       <c r="E63" s="12" t="n">
-        <v>0.07692677667466921</v>
+        <v>0.07692496646710331</v>
       </c>
       <c r="F63" s="12" t="n">
-        <v>0.4740803814994422</v>
+        <v>0.4284467817562574</v>
       </c>
     </row>
     <row r="64">
@@ -4240,19 +4240,19 @@
         </is>
       </c>
       <c r="B64" s="9" t="n">
-        <v>0.06629782075571977</v>
+        <v>0.06730104265263419</v>
       </c>
       <c r="C64" s="24" t="n">
-        <v>0.04024510211790198</v>
+        <v>0.0396094981648834</v>
       </c>
       <c r="D64" s="24" t="n">
-        <v>0.002668162566508303</v>
+        <v>0.002665760525444253</v>
       </c>
       <c r="E64" s="9" t="n">
-        <v>0.0769169272660708</v>
+        <v>0.07692075524958694</v>
       </c>
       <c r="F64" s="9" t="n">
-        <v>0.1419427420681525</v>
+        <v>0.1297114447333514</v>
       </c>
     </row>
     <row r="66">
@@ -4306,16 +4306,16 @@
         </is>
       </c>
       <c r="B68" s="9" t="n">
-        <v>0.02620344769844228</v>
+        <v>0.06129129745559889</v>
       </c>
       <c r="C68" s="24" t="n">
-        <v>0.06740968278435086</v>
+        <v>0.06571255610075652</v>
       </c>
       <c r="D68" s="24" t="n">
-        <v>0.001766366097208323</v>
+        <v>0.004027607822539197</v>
       </c>
       <c r="E68" s="9" t="n">
-        <v>0.05704715523155528</v>
+        <v>0.1299992912254229</v>
       </c>
       <c r="F68" s="9" t="n">
         <v>0.9718498340506938</v>
@@ -4328,16 +4328,16 @@
         </is>
       </c>
       <c r="B69" s="12" t="n">
-        <v>0.05077551892986816</v>
+        <v>0.01980455968018955</v>
       </c>
       <c r="C69" s="25" t="n">
-        <v>0.07548635024430657</v>
+        <v>0.07247942716059193</v>
       </c>
       <c r="D69" s="25" t="n">
-        <v>0.003832858605776446</v>
+        <v>0.001435423140787894</v>
       </c>
       <c r="E69" s="12" t="n">
-        <v>0.1237872942703699</v>
+        <v>0.04633122169113092</v>
       </c>
       <c r="F69" s="12" t="n">
         <v>0.9005695345361184</v>
@@ -4350,16 +4350,16 @@
         </is>
       </c>
       <c r="B70" s="9" t="n">
-        <v>0.02519040831093613</v>
+        <v>0.02491094989735838</v>
       </c>
       <c r="C70" s="24" t="n">
-        <v>0.07783289142166173</v>
+        <v>0.07480928774820883</v>
       </c>
       <c r="D70" s="24" t="n">
-        <v>0.001960642314932417</v>
+        <v>0.001863570418952696</v>
       </c>
       <c r="E70" s="9" t="n">
-        <v>0.06332156548423279</v>
+        <v>0.06015055196207775</v>
       </c>
       <c r="F70" s="9" t="n">
         <v>0.8647852106386994</v>
@@ -4372,16 +4372,16 @@
         </is>
       </c>
       <c r="B71" s="12" t="n">
-        <v>0.01904658044143235</v>
+        <v>0.0188233496030912</v>
       </c>
       <c r="C71" s="25" t="n">
-        <v>0.08206660721410963</v>
+        <v>0.07976725601333907</v>
       </c>
       <c r="D71" s="25" t="n">
-        <v>0.001563088235858972</v>
+        <v>0.00150148694681836</v>
       </c>
       <c r="E71" s="12" t="n">
-        <v>0.05048202486030171</v>
+        <v>0.0484635663329188</v>
       </c>
       <c r="F71" s="12" t="n">
         <v>0.6547256214279519</v>
@@ -4394,16 +4394,16 @@
         </is>
       </c>
       <c r="B72" s="9" t="n">
-        <v>0.0698853272913602</v>
+        <v>0.06372964737267586</v>
       </c>
       <c r="C72" s="24" t="n">
-        <v>0.006653786894103503</v>
+        <v>0.01095281208977317</v>
       </c>
       <c r="D72" s="24" t="n">
-        <v>0.0004650020748213863</v>
+        <v>0.0006980188522204254</v>
       </c>
       <c r="E72" s="9" t="n">
-        <v>0.01501786384331987</v>
+        <v>0.02252998803479094</v>
       </c>
       <c r="F72" s="9" t="n">
         <v>0.9800395309996239</v>
@@ -4416,16 +4416,16 @@
         </is>
       </c>
       <c r="B73" s="12" t="n">
-        <v>0.3247963366415298</v>
+        <v>0.3209896397522077</v>
       </c>
       <c r="C73" s="25" t="n">
-        <v>0.0170965766851034</v>
+        <v>0.01766059081007425</v>
       </c>
       <c r="D73" s="25" t="n">
-        <v>0.005552905476432574</v>
+        <v>0.005668866681936884</v>
       </c>
       <c r="E73" s="12" t="n">
-        <v>0.1793385081387475</v>
+        <v>0.1829742822970787</v>
       </c>
       <c r="F73" s="12" t="n">
         <v>0.8261546883028914</v>
@@ -4438,16 +4438,16 @@
         </is>
       </c>
       <c r="B74" s="9" t="n">
-        <v>0.09938010970300858</v>
+        <v>0.1515664321754441</v>
       </c>
       <c r="C74" s="24" t="n">
-        <v>0.02657502189855462</v>
+        <v>0.02868467832979765</v>
       </c>
       <c r="D74" s="24" t="n">
-        <v>0.002641028591638213</v>
+        <v>0.004347634352547708</v>
       </c>
       <c r="E74" s="9" t="n">
-        <v>0.08529555015592669</v>
+        <v>0.140328802912638</v>
       </c>
       <c r="F74" s="9" t="n">
         <v>0.6542475111182804</v>
@@ -4460,16 +4460,16 @@
         </is>
       </c>
       <c r="B75" s="12" t="n">
-        <v>0.02251791599980841</v>
+        <v>0.0222215038737016</v>
       </c>
       <c r="C75" s="25" t="n">
-        <v>0.08127192716573621</v>
+        <v>0.0802414429506282</v>
       </c>
       <c r="D75" s="25" t="n">
-        <v>0.001830074429060595</v>
+        <v>0.001783085535358791</v>
       </c>
       <c r="E75" s="12" t="n">
-        <v>0.05910470100446386</v>
+        <v>0.05755273750680341</v>
       </c>
       <c r="F75" s="12" t="n">
         <v>0.6432514443485702</v>
@@ -4482,16 +4482,16 @@
         </is>
       </c>
       <c r="B76" s="9" t="n">
-        <v>0.01799739840041237</v>
+        <v>0.01792687522994341</v>
       </c>
       <c r="C76" s="24" t="n">
-        <v>0.04984858965177769</v>
+        <v>0.04468307590564768</v>
       </c>
       <c r="D76" s="24" t="n">
-        <v>0.0008971449276617164</v>
+        <v>0.0008010279266506368</v>
       </c>
       <c r="E76" s="9" t="n">
-        <v>0.02897449517085264</v>
+        <v>0.02585481688003633</v>
       </c>
       <c r="F76" s="9" t="n">
         <v>0.4797912934834942</v>
@@ -4504,16 +4504,16 @@
         </is>
       </c>
       <c r="B77" s="12" t="n">
-        <v>0.06562781917806712</v>
+        <v>0.06139883262218021</v>
       </c>
       <c r="C77" s="25" t="n">
-        <v>0.03956645689908946</v>
+        <v>0.03926948434702817</v>
       </c>
       <c r="D77" s="25" t="n">
-        <v>0.00259666027889023</v>
+        <v>0.002411100496582508</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>0.08386261616296979</v>
+        <v>0.07782320658801947</v>
       </c>
       <c r="F77" s="12" t="n">
         <v>0.6813173339403511</v>
@@ -4526,19 +4526,19 @@
         </is>
       </c>
       <c r="B78" s="9" t="n">
-        <v>0.2219112355471898</v>
+        <v>0.1822438014945581</v>
       </c>
       <c r="C78" s="24" t="n">
-        <v>0.02564637069020121</v>
+        <v>0.02461766227162885</v>
       </c>
       <c r="D78" s="24" t="n">
-        <v>0.005691217807163784</v>
+        <v>0.004486416356290799</v>
       </c>
       <c r="E78" s="9" t="n">
-        <v>0.1838054898217247</v>
+        <v>0.1448082763163002</v>
       </c>
       <c r="F78" s="9" t="n">
-        <v>0.7553246822404955</v>
+        <v>0.7487919560463553</v>
       </c>
     </row>
     <row r="79">
@@ -4548,19 +4548,19 @@
         </is>
       </c>
       <c r="B79" s="12" t="n">
-        <v>0.03024721272215291</v>
+        <v>0.02896140192186942</v>
       </c>
       <c r="C79" s="25" t="n">
-        <v>0.04411012875787568</v>
+        <v>0.04190259392293433</v>
       </c>
       <c r="D79" s="25" t="n">
-        <v>0.00133420844774102</v>
+        <v>0.001213557864170984</v>
       </c>
       <c r="E79" s="12" t="n">
-        <v>0.04309004602716724</v>
+        <v>0.03917006549654713</v>
       </c>
       <c r="F79" s="12" t="n">
-        <v>0.4740803814994422</v>
+        <v>0.4284467817562574</v>
       </c>
     </row>
     <row r="80">
@@ -4570,19 +4570,19 @@
         </is>
       </c>
       <c r="B80" s="9" t="n">
-        <v>0.02642068913579193</v>
+        <v>0.02613170892118141</v>
       </c>
       <c r="C80" s="24" t="n">
-        <v>0.03149297775010471</v>
+        <v>0.02847005369509953</v>
       </c>
       <c r="D80" s="24" t="n">
-        <v>0.0008320661750959287</v>
+        <v>0.000743971156130746</v>
       </c>
       <c r="E80" s="9" t="n">
-        <v>0.02687268982836784</v>
+        <v>0.02401319275623543</v>
       </c>
       <c r="F80" s="9" t="n">
-        <v>0.1419427420681525</v>
+        <v>0.1297114447333514</v>
       </c>
     </row>
   </sheetData>
@@ -4748,13 +4748,13 @@
         <v>0.732</v>
       </c>
       <c r="L3" s="40" t="n">
-        <v>0.879</v>
+        <v>0.877</v>
       </c>
       <c r="M3" s="43" t="n">
-        <v>0.641</v>
+        <v>0.621</v>
       </c>
       <c r="N3" s="42" t="n">
-        <v>0.189</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="4">
@@ -4794,13 +4794,13 @@
         <v>0.719</v>
       </c>
       <c r="L4" s="40" t="n">
-        <v>0.884</v>
+        <v>0.882</v>
       </c>
       <c r="M4" s="43" t="n">
-        <v>0.629</v>
+        <v>0.613</v>
       </c>
       <c r="N4" s="42" t="n">
-        <v>0.202</v>
+        <v>0.198</v>
       </c>
     </row>
     <row r="5">
@@ -4840,13 +4840,13 @@
         <v>0.673</v>
       </c>
       <c r="L5" s="40" t="n">
-        <v>0.84</v>
+        <v>0.838</v>
       </c>
       <c r="M5" s="43" t="n">
-        <v>0.6</v>
+        <v>0.58</v>
       </c>
       <c r="N5" s="42" t="n">
-        <v>0.162</v>
+        <v>0.163</v>
       </c>
     </row>
     <row r="6">
@@ -4886,13 +4886,13 @@
         <v>0.647</v>
       </c>
       <c r="L6" s="40" t="n">
-        <v>0.851</v>
+        <v>0.844</v>
       </c>
       <c r="M6" s="43" t="n">
-        <v>0.595</v>
+        <v>0.556</v>
       </c>
       <c r="N6" s="42" t="n">
-        <v>0.169</v>
+        <v>0.178</v>
       </c>
     </row>
     <row r="7">
@@ -4932,10 +4932,10 @@
         <v>-0.177</v>
       </c>
       <c r="L7" s="41" t="n">
-        <v>-0.348</v>
+        <v>-0.337</v>
       </c>
       <c r="M7" s="41" t="n">
-        <v>-0.391</v>
+        <v>-0.361</v>
       </c>
       <c r="N7" s="42" t="n">
         <v>-0.139</v>
@@ -4978,13 +4978,13 @@
         <v>0.38</v>
       </c>
       <c r="L8" s="42" t="n">
-        <v>0.22</v>
+        <v>0.225</v>
       </c>
       <c r="M8" s="42" t="n">
-        <v>0.136</v>
+        <v>0.154</v>
       </c>
       <c r="N8" s="42" t="n">
-        <v>0.186</v>
+        <v>0.172</v>
       </c>
     </row>
     <row r="9">
@@ -5024,13 +5024,13 @@
         <v>0.375</v>
       </c>
       <c r="L9" s="42" t="n">
-        <v>0.304</v>
+        <v>0.314</v>
       </c>
       <c r="M9" s="42" t="n">
-        <v>0.054</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="N9" s="42" t="n">
-        <v>-0.07099999999999999</v>
+        <v>-0.075</v>
       </c>
     </row>
     <row r="10">
@@ -5070,13 +5070,13 @@
         <v>0.581</v>
       </c>
       <c r="L10" s="43" t="n">
-        <v>0.616</v>
+        <v>0.611</v>
       </c>
       <c r="M10" s="43" t="n">
-        <v>0.447</v>
+        <v>0.417</v>
       </c>
       <c r="N10" s="42" t="n">
-        <v>0.141</v>
+        <v>0.152</v>
       </c>
     </row>
     <row r="11">
@@ -5116,13 +5116,13 @@
         <v>0.383</v>
       </c>
       <c r="L11" s="43" t="n">
-        <v>0.491</v>
-      </c>
-      <c r="M11" s="43" t="n">
-        <v>0.422</v>
+        <v>0.483</v>
+      </c>
+      <c r="M11" s="42" t="n">
+        <v>0.399</v>
       </c>
       <c r="N11" s="42" t="n">
-        <v>0.209</v>
+        <v>0.205</v>
       </c>
     </row>
     <row r="12">
@@ -5161,14 +5161,14 @@
       <c r="K12" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="L12" s="43" t="n">
-        <v>0.6830000000000001</v>
+      <c r="L12" s="40" t="n">
+        <v>0.704</v>
       </c>
       <c r="M12" s="43" t="n">
-        <v>0.476</v>
+        <v>0.5610000000000001</v>
       </c>
       <c r="N12" s="42" t="n">
-        <v>0.22</v>
+        <v>0.176</v>
       </c>
     </row>
     <row r="13">
@@ -5178,43 +5178,43 @@
         </is>
       </c>
       <c r="B13" s="40" t="n">
-        <v>0.879</v>
+        <v>0.877</v>
       </c>
       <c r="C13" s="40" t="n">
-        <v>0.884</v>
+        <v>0.882</v>
       </c>
       <c r="D13" s="40" t="n">
-        <v>0.84</v>
+        <v>0.838</v>
       </c>
       <c r="E13" s="40" t="n">
-        <v>0.851</v>
+        <v>0.844</v>
       </c>
       <c r="F13" s="41" t="n">
-        <v>-0.348</v>
+        <v>-0.337</v>
       </c>
       <c r="G13" s="42" t="n">
-        <v>0.22</v>
+        <v>0.225</v>
       </c>
       <c r="H13" s="42" t="n">
-        <v>0.304</v>
+        <v>0.314</v>
       </c>
       <c r="I13" s="43" t="n">
-        <v>0.616</v>
+        <v>0.611</v>
       </c>
       <c r="J13" s="43" t="n">
-        <v>0.491</v>
-      </c>
-      <c r="K13" s="43" t="n">
-        <v>0.6830000000000001</v>
+        <v>0.483</v>
+      </c>
+      <c r="K13" s="40" t="n">
+        <v>0.704</v>
       </c>
       <c r="L13" s="39" t="n">
         <v>1</v>
       </c>
       <c r="M13" s="43" t="n">
-        <v>0.658</v>
+        <v>0.64</v>
       </c>
       <c r="N13" s="42" t="n">
-        <v>0.204</v>
+        <v>0.198</v>
       </c>
     </row>
     <row r="14">
@@ -5224,43 +5224,43 @@
         </is>
       </c>
       <c r="B14" s="43" t="n">
-        <v>0.641</v>
+        <v>0.621</v>
       </c>
       <c r="C14" s="43" t="n">
-        <v>0.629</v>
+        <v>0.613</v>
       </c>
       <c r="D14" s="43" t="n">
-        <v>0.6</v>
+        <v>0.58</v>
       </c>
       <c r="E14" s="43" t="n">
-        <v>0.595</v>
+        <v>0.556</v>
       </c>
       <c r="F14" s="41" t="n">
-        <v>-0.391</v>
+        <v>-0.361</v>
       </c>
       <c r="G14" s="42" t="n">
-        <v>0.136</v>
+        <v>0.154</v>
       </c>
       <c r="H14" s="42" t="n">
-        <v>0.054</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="I14" s="43" t="n">
-        <v>0.447</v>
-      </c>
-      <c r="J14" s="43" t="n">
-        <v>0.422</v>
+        <v>0.417</v>
+      </c>
+      <c r="J14" s="42" t="n">
+        <v>0.399</v>
       </c>
       <c r="K14" s="43" t="n">
-        <v>0.476</v>
+        <v>0.5610000000000001</v>
       </c>
       <c r="L14" s="43" t="n">
-        <v>0.658</v>
+        <v>0.64</v>
       </c>
       <c r="M14" s="39" t="n">
         <v>1</v>
       </c>
       <c r="N14" s="43" t="n">
-        <v>0.46</v>
+        <v>0.441</v>
       </c>
     </row>
     <row r="15">
@@ -5270,40 +5270,40 @@
         </is>
       </c>
       <c r="B15" s="42" t="n">
-        <v>0.189</v>
+        <v>0.19</v>
       </c>
       <c r="C15" s="42" t="n">
-        <v>0.202</v>
+        <v>0.198</v>
       </c>
       <c r="D15" s="42" t="n">
-        <v>0.162</v>
+        <v>0.163</v>
       </c>
       <c r="E15" s="42" t="n">
-        <v>0.169</v>
+        <v>0.178</v>
       </c>
       <c r="F15" s="42" t="n">
         <v>-0.139</v>
       </c>
       <c r="G15" s="42" t="n">
-        <v>0.186</v>
+        <v>0.172</v>
       </c>
       <c r="H15" s="42" t="n">
-        <v>-0.07099999999999999</v>
+        <v>-0.075</v>
       </c>
       <c r="I15" s="42" t="n">
-        <v>0.141</v>
+        <v>0.152</v>
       </c>
       <c r="J15" s="42" t="n">
-        <v>0.209</v>
+        <v>0.205</v>
       </c>
       <c r="K15" s="42" t="n">
-        <v>0.22</v>
+        <v>0.176</v>
       </c>
       <c r="L15" s="42" t="n">
-        <v>0.204</v>
+        <v>0.198</v>
       </c>
       <c r="M15" s="43" t="n">
-        <v>0.46</v>
+        <v>0.441</v>
       </c>
       <c r="N15" s="39" t="n">
         <v>1</v>
@@ -5435,7 +5435,7 @@
         </is>
       </c>
       <c r="C22" s="29" t="n">
-        <v>0.8835248952761964</v>
+        <v>0.8818708712318351</v>
       </c>
       <c r="D22" s="45" t="inlineStr">
         <is>
@@ -5460,7 +5460,7 @@
         </is>
       </c>
       <c r="C23" s="28" t="n">
-        <v>0.8791414690292736</v>
+        <v>0.8772590564733882</v>
       </c>
       <c r="D23" s="44" t="inlineStr">
         <is>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C24" s="29" t="n">
-        <v>0.85071265595919</v>
+        <v>0.8442031212496387</v>
       </c>
       <c r="D24" s="45" t="inlineStr">
         <is>
@@ -5510,7 +5510,7 @@
         </is>
       </c>
       <c r="C25" s="28" t="n">
-        <v>0.8396667894157622</v>
+        <v>0.8378878973040726</v>
       </c>
       <c r="D25" s="44" t="inlineStr">
         <is>
@@ -5807,13 +5807,13 @@
         <v>0.12</v>
       </c>
       <c r="D3" s="9" t="n">
-        <v>1.12998593313295e-07</v>
+        <v>1.540461288441797e-08</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>0.04237184338252779</v>
+        <v>0.04239826333525394</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>0.02620344769844228</v>
+        <v>0.06129129745559889</v>
       </c>
     </row>
     <row r="4">
@@ -5829,13 +5829,13 @@
         <v>0.12</v>
       </c>
       <c r="D4" s="12" t="n">
-        <v>9.768383840153099e-08</v>
+        <v>1.286140172707754e-08</v>
       </c>
       <c r="E4" s="12" t="n">
-        <v>0.03835312966778117</v>
+        <v>0.03838122897303223</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>0.05077551892986816</v>
+        <v>0.01980455968018955</v>
       </c>
     </row>
     <row r="5">
@@ -5851,13 +5851,13 @@
         <v>0.12</v>
       </c>
       <c r="D5" s="9" t="n">
-        <v>7.870694893487945e-08</v>
+        <v>1.034391777355504e-08</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>0.03704034967567654</v>
+        <v>0.0370534553973652</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>0.02519040831093613</v>
+        <v>0.02491094989735838</v>
       </c>
     </row>
     <row r="6">
@@ -5873,13 +5873,13 @@
         <v>0.12</v>
       </c>
       <c r="D6" s="12" t="n">
-        <v>0.04190992908765714</v>
+        <v>0.07113737017120696</v>
       </c>
       <c r="E6" s="12" t="n">
-        <v>0.03518145231877982</v>
+        <v>0.03526861812873507</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>0.01904658044143235</v>
+        <v>0.0188233496030912</v>
       </c>
     </row>
     <row r="7">
@@ -5895,13 +5895,13 @@
         <v>0.1333333333333333</v>
       </c>
       <c r="D7" s="46" t="n">
-        <v>0.2886613151522574</v>
+        <v>0.2963200956729828</v>
       </c>
       <c r="E7" s="46" t="n">
-        <v>0.1916974426113651</v>
+        <v>0.1901058368847075</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>0.0698853272913602</v>
+        <v>0.06372964737267586</v>
       </c>
     </row>
     <row r="8">
@@ -5917,13 +5917,13 @@
         <v>0.1333333333333333</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>6.941451318814953e-08</v>
+        <v>9.201562116762712e-09</v>
       </c>
       <c r="E8" s="47" t="n">
-        <v>0.1560290416425018</v>
+        <v>0.1561033628971746</v>
       </c>
       <c r="F8" s="47" t="n">
-        <v>0.3247963366415298</v>
+        <v>0.3209896397522077</v>
       </c>
     </row>
     <row r="9">
@@ -5939,13 +5939,13 @@
         <v>0.1333333333333333</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>6.965110784322271e-08</v>
+        <v>8.935097992254681e-09</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>0.09902372157555807</v>
-      </c>
-      <c r="F9" s="9" t="n">
-        <v>0.09938010970300858</v>
+        <v>0.09891989158807808</v>
+      </c>
+      <c r="F9" s="46" t="n">
+        <v>0.1515664321754441</v>
       </c>
     </row>
     <row r="10">
@@ -5961,13 +5961,13 @@
         <v>0.12</v>
       </c>
       <c r="D10" s="47" t="n">
-        <v>0.123639275433536</v>
+        <v>0.1364634563400894</v>
       </c>
       <c r="E10" s="12" t="n">
-        <v>0.03305541874853363</v>
+        <v>0.03310675547604956</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>0.02251791599980841</v>
+        <v>0.0222215038737016</v>
       </c>
     </row>
     <row r="11">
@@ -5983,13 +5983,13 @@
         <v>0</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>1.08473008170814e-07</v>
+        <v>2.096350137433955e-08</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>0.05433105722415058</v>
+        <v>0.05454871770448565</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>0.01799739840041237</v>
+        <v>0.01792687522994341</v>
       </c>
     </row>
     <row r="12">
@@ -6005,13 +6005,13 @@
         <v>0</v>
       </c>
       <c r="D12" s="47" t="n">
-        <v>0.2457889564637488</v>
+        <v>0.1960790013757596</v>
       </c>
       <c r="E12" s="12" t="n">
-        <v>0.07190731636107728</v>
+        <v>0.07131481415928038</v>
       </c>
       <c r="F12" s="12" t="n">
-        <v>0.06562781917806712</v>
+        <v>0.06139883262218021</v>
       </c>
     </row>
     <row r="13">
@@ -6027,13 +6027,13 @@
         <v>0</v>
       </c>
       <c r="D13" s="9" t="n">
-        <v>1.520208122408094e-08</v>
+        <v>1.618598277387212e-09</v>
       </c>
       <c r="E13" s="46" t="n">
-        <v>0.1140716492667996</v>
+        <v>0.1147079339099366</v>
       </c>
       <c r="F13" s="46" t="n">
-        <v>0.2219112355471898</v>
+        <v>0.1822438014945581</v>
       </c>
     </row>
     <row r="14">
@@ -6049,13 +6049,13 @@
         <v>0</v>
       </c>
       <c r="D14" s="47" t="n">
-        <v>0.2994235045579806</v>
+        <v>0.2822620050016704</v>
       </c>
       <c r="E14" s="12" t="n">
-        <v>0.06063975676952887</v>
+        <v>0.06079007889326719</v>
       </c>
       <c r="F14" s="12" t="n">
-        <v>0.03024721272215291</v>
+        <v>0.02896140192186942</v>
       </c>
     </row>
     <row r="15">
@@ -6071,13 +6071,13 @@
         <v>0</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>0.0005764671747288517</v>
+        <v>0.01773799210959868</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>0.06629782075571977</v>
+        <v>0.06730104265263419</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>0.02642068913579193</v>
+        <v>0.02613170892118141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add analytics report Excel workbook — 8 sheets, all results
</commit_message>
<xml_diff>
--- a/analytics_report.xlsx
+++ b/analytics_report.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Risk Decomposition" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Covariance" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Portfolio Weights" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Cluster Analysis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,11 +23,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="+0.000;-0.000;0.000"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="37">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -122,8 +124,119 @@
       <color rgb="00F0F4F8"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00B03A2E"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="007A90A8"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FF6B6B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00D0D8E4"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="002E6DA4"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="006BCB77"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00B7770D"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001E7B45"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="006B3FA0"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00B03A2E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="006BCB77"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="006BCB77"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00FF6B6B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="002E6DA4"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="002E6DA4"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00B7770D"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FF6B6B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001E7B45"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="006B3FA0"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="006B3FA0"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -178,8 +291,56 @@
         <bgColor rgb="008B2E1A"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B03A2E"/>
+        <bgColor rgb="00B03A2E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00111927"/>
+        <bgColor rgb="00111927"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003A1A1A"/>
+        <bgColor rgb="003A1A1A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E6DA4"/>
+        <bgColor rgb="002E6DA4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E3A1A"/>
+        <bgColor rgb="001E3A1A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B7770D"/>
+        <bgColor rgb="00B7770D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006B3FA0"/>
+        <bgColor rgb="006B3FA0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A2436"/>
+        <bgColor rgb="001A2436"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -245,11 +406,81 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="00B03A2E"/>
+      </left>
+      <right style="thin">
+        <color rgb="001E2D3D"/>
+      </right>
+      <top style="thin">
+        <color rgb="001E2D3D"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="001E2D3D"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="002E6DA4"/>
+      </left>
+      <right style="thin">
+        <color rgb="001E2D3D"/>
+      </right>
+      <top style="thin">
+        <color rgb="001E2D3D"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="001E2D3D"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00B7770D"/>
+      </left>
+      <right style="thin">
+        <color rgb="001E2D3D"/>
+      </right>
+      <top style="thin">
+        <color rgb="001E2D3D"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="001E2D3D"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="001E7B45"/>
+      </left>
+      <right style="thin">
+        <color rgb="001E2D3D"/>
+      </right>
+      <top style="thin">
+        <color rgb="001E2D3D"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="001E2D3D"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="006B3FA0"/>
+      </left>
+      <right style="thin">
+        <color rgb="001E2D3D"/>
+      </right>
+      <top style="thin">
+        <color rgb="001E2D3D"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="001E2D3D"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -386,6 +617,147 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="27" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="28" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="29" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="33" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -744,6 +1116,86 @@
 </wsDr>
 </file>
 
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8667750" cy="3238500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>41</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4667250" cy="4381500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>41</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5334000" cy="3714750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1063,7 +1515,7 @@
     <row r="4" ht="36" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Key Finding: A conventional 60/40 portfolio allocates 80.6% of total risk to Equity Premium. Enhanced HRP reduces this to 53.5% — a 27.1 pp reduction — while maintaining balanced systematic risk exposure across all five factors.</t>
+          <t>Key Finding: A conventional 60/40 portfolio allocates 80.6% of total risk to Equity Premium. Enhanced HRP reduces this to 42.0% — a 38.6 pp reduction — while maintaining balanced systematic risk exposure across all five factors.</t>
         </is>
       </c>
     </row>
@@ -1207,19 +1659,19 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>0.05341435110809257</v>
+        <v>0.0519153225469064</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>0.06196353510197526</v>
+        <v>0.05672701063600807</v>
       </c>
       <c r="D12" s="10" t="n">
-        <v>0.8620287887091489</v>
+        <v>0.9151781834587385</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>-0.1548283411757465</v>
+        <v>-0.1388515020427566</v>
       </c>
       <c r="F12" s="10" t="n">
-        <v>0.3449907859405511</v>
+        <v>0.3738909682872575</v>
       </c>
     </row>
     <row r="13" ht="8" customHeight="1"/>
@@ -1379,22 +1831,22 @@
         </is>
       </c>
       <c r="B20" s="16" t="n">
-        <v>0.535</v>
+        <v>0.42</v>
       </c>
       <c r="C20" s="9" t="n">
-        <v>0.12</v>
+        <v>0.14</v>
       </c>
       <c r="D20" s="9" t="n">
-        <v>0.055</v>
+        <v>0.065</v>
       </c>
       <c r="E20" s="9" t="n">
+        <v>0.191</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>0.031</v>
+      </c>
+      <c r="G20" s="9" t="n">
         <v>0.154</v>
-      </c>
-      <c r="F20" s="9" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="G20" s="9" t="n">
-        <v>0.126</v>
       </c>
     </row>
     <row r="21" ht="8" customHeight="1"/>
@@ -2597,16 +3049,16 @@
         </is>
       </c>
       <c r="B7" s="32" t="n">
-        <v>-0.1257176000642428</v>
+        <v>-0.1050506428004342</v>
       </c>
       <c r="C7" s="34" t="n">
-        <v>0.02542692133678326</v>
+        <v>0.02485925553436985</v>
       </c>
       <c r="D7" s="32" t="n">
-        <v>-0.130784375396225</v>
+        <v>-0.1166178609836621</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>0.322990144323839</v>
+        <v>0.3183738177155639</v>
       </c>
     </row>
     <row r="8" ht="8" customHeight="1"/>
@@ -4306,16 +4758,16 @@
         </is>
       </c>
       <c r="B68" s="9" t="n">
-        <v>0.06129129745559889</v>
+        <v>0.01418954230934598</v>
       </c>
       <c r="C68" s="24" t="n">
-        <v>0.06571255610075652</v>
+        <v>0.0621455954800322</v>
       </c>
       <c r="D68" s="24" t="n">
-        <v>0.004027607822539197</v>
+        <v>0.0008818175564034173</v>
       </c>
       <c r="E68" s="9" t="n">
-        <v>0.1299992912254229</v>
+        <v>0.03108986518121491</v>
       </c>
       <c r="F68" s="9" t="n">
         <v>0.9718498340506938</v>
@@ -4328,16 +4780,16 @@
         </is>
       </c>
       <c r="B69" s="12" t="n">
-        <v>0.01980455968018955</v>
+        <v>0.01071962159834464</v>
       </c>
       <c r="C69" s="25" t="n">
-        <v>0.07247942716059193</v>
+        <v>0.06881032714615799</v>
       </c>
       <c r="D69" s="25" t="n">
-        <v>0.001435423140787894</v>
+        <v>0.0007376206690651158</v>
       </c>
       <c r="E69" s="12" t="n">
-        <v>0.04633122169113092</v>
+        <v>0.0260059770749458</v>
       </c>
       <c r="F69" s="12" t="n">
         <v>0.9005695345361184</v>
@@ -4350,16 +4802,16 @@
         </is>
       </c>
       <c r="B70" s="9" t="n">
-        <v>0.02491094989735838</v>
+        <v>0.01785691413064642</v>
       </c>
       <c r="C70" s="24" t="n">
-        <v>0.07480928774820883</v>
+        <v>0.0699804705840664</v>
       </c>
       <c r="D70" s="24" t="n">
-        <v>0.001863570418952696</v>
+        <v>0.001249635254041901</v>
       </c>
       <c r="E70" s="9" t="n">
-        <v>0.06015055196207775</v>
+        <v>0.04405785674342171</v>
       </c>
       <c r="F70" s="9" t="n">
         <v>0.8647852106386994</v>
@@ -4372,16 +4824,16 @@
         </is>
       </c>
       <c r="B71" s="12" t="n">
-        <v>0.0188233496030912</v>
+        <v>0.01018151128031412</v>
       </c>
       <c r="C71" s="25" t="n">
-        <v>0.07976725601333907</v>
+        <v>0.07713721713992763</v>
       </c>
       <c r="D71" s="25" t="n">
-        <v>0.00150148694681836</v>
+        <v>0.000785373446442213</v>
       </c>
       <c r="E71" s="12" t="n">
-        <v>0.0484635663329188</v>
+        <v>0.02768957636359879</v>
       </c>
       <c r="F71" s="12" t="n">
         <v>0.6547256214279519</v>
@@ -4394,16 +4846,16 @@
         </is>
       </c>
       <c r="B72" s="9" t="n">
-        <v>0.06372964737267586</v>
+        <v>0.0596596557957153</v>
       </c>
       <c r="C72" s="24" t="n">
-        <v>0.01095281208977317</v>
+        <v>0.01185652218885514</v>
       </c>
       <c r="D72" s="24" t="n">
-        <v>0.0006980188522204254</v>
+        <v>0.0007073560327213588</v>
       </c>
       <c r="E72" s="9" t="n">
-        <v>0.02252998803479094</v>
+        <v>0.02493894970987092</v>
       </c>
       <c r="F72" s="9" t="n">
         <v>0.9800395309996239</v>
@@ -4416,16 +4868,16 @@
         </is>
       </c>
       <c r="B73" s="12" t="n">
-        <v>0.3209896397522077</v>
+        <v>0.3316397889964033</v>
       </c>
       <c r="C73" s="25" t="n">
-        <v>0.01766059081007425</v>
+        <v>0.01854942338164662</v>
       </c>
       <c r="D73" s="25" t="n">
-        <v>0.005668866681936884</v>
+        <v>0.006151726856294233</v>
       </c>
       <c r="E73" s="12" t="n">
-        <v>0.1829742822970787</v>
+        <v>0.2168888079002478</v>
       </c>
       <c r="F73" s="12" t="n">
         <v>0.8261546883028914</v>
@@ -4438,16 +4890,16 @@
         </is>
       </c>
       <c r="B74" s="9" t="n">
-        <v>0.1515664321754441</v>
+        <v>0.1092060125556164</v>
       </c>
       <c r="C74" s="24" t="n">
-        <v>0.02868467832979765</v>
+        <v>0.02838237345122105</v>
       </c>
       <c r="D74" s="24" t="n">
-        <v>0.004347634352547708</v>
+        <v>0.003099525831472239</v>
       </c>
       <c r="E74" s="9" t="n">
-        <v>0.140328802912638</v>
+        <v>0.109278659203832</v>
       </c>
       <c r="F74" s="9" t="n">
         <v>0.6542475111182804</v>
@@ -4460,16 +4912,16 @@
         </is>
       </c>
       <c r="B75" s="12" t="n">
-        <v>0.0222215038737016</v>
+        <v>0.009319148736044227</v>
       </c>
       <c r="C75" s="25" t="n">
-        <v>0.0802414429506282</v>
+        <v>0.07416805794013158</v>
       </c>
       <c r="D75" s="25" t="n">
-        <v>0.001783085535358791</v>
+        <v>0.0006911831634076322</v>
       </c>
       <c r="E75" s="12" t="n">
-        <v>0.05755273750680341</v>
+        <v>0.02436874975988587</v>
       </c>
       <c r="F75" s="12" t="n">
         <v>0.6432514443485702</v>
@@ -4482,16 +4934,16 @@
         </is>
       </c>
       <c r="B76" s="9" t="n">
-        <v>0.01792687522994341</v>
+        <v>0.01805983719241161</v>
       </c>
       <c r="C76" s="24" t="n">
-        <v>0.04468307590564768</v>
+        <v>0.04543999203099217</v>
       </c>
       <c r="D76" s="24" t="n">
-        <v>0.0008010279266506368</v>
+        <v>0.0008206388581041995</v>
       </c>
       <c r="E76" s="9" t="n">
-        <v>0.02585481688003633</v>
+        <v>0.02893291392948143</v>
       </c>
       <c r="F76" s="9" t="n">
         <v>0.4797912934834942</v>
@@ -4504,16 +4956,16 @@
         </is>
       </c>
       <c r="B77" s="12" t="n">
-        <v>0.06139883262218021</v>
+        <v>0.1483922296615784</v>
       </c>
       <c r="C77" s="25" t="n">
-        <v>0.03926948434702817</v>
+        <v>0.04167679313253376</v>
       </c>
       <c r="D77" s="25" t="n">
-        <v>0.002411100496582508</v>
+        <v>0.006184512258081045</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>0.07782320658801947</v>
+        <v>0.2180447088165566</v>
       </c>
       <c r="F77" s="12" t="n">
         <v>0.6813173339403511</v>
@@ -4526,16 +4978,16 @@
         </is>
       </c>
       <c r="B78" s="9" t="n">
-        <v>0.1822438014945581</v>
+        <v>0.2280024325953268</v>
       </c>
       <c r="C78" s="24" t="n">
-        <v>0.02461766227162885</v>
+        <v>0.02412051657055184</v>
       </c>
       <c r="D78" s="24" t="n">
-        <v>0.004486416356290799</v>
+        <v>0.005499536453541708</v>
       </c>
       <c r="E78" s="9" t="n">
-        <v>0.1448082763163002</v>
+        <v>0.1938948092586715</v>
       </c>
       <c r="F78" s="9" t="n">
         <v>0.7487919560463553</v>
@@ -4548,16 +5000,16 @@
         </is>
       </c>
       <c r="B79" s="12" t="n">
-        <v>0.02896140192186942</v>
+        <v>0.02821942763967997</v>
       </c>
       <c r="C79" s="25" t="n">
-        <v>0.04190259392293433</v>
+        <v>0.04155512604382863</v>
       </c>
       <c r="D79" s="25" t="n">
-        <v>0.001213557864170984</v>
+        <v>0.001172661872451603</v>
       </c>
       <c r="E79" s="12" t="n">
-        <v>0.03917006549654713</v>
+        <v>0.04134403908487444</v>
       </c>
       <c r="F79" s="12" t="n">
         <v>0.4284467817562574</v>
@@ -4570,16 +5022,16 @@
         </is>
       </c>
       <c r="B80" s="9" t="n">
-        <v>0.02613170892118141</v>
+        <v>0.01455387750857305</v>
       </c>
       <c r="C80" s="24" t="n">
-        <v>0.02847005369509953</v>
+        <v>0.02624160233260154</v>
       </c>
       <c r="D80" s="24" t="n">
-        <v>0.000743971156130746</v>
+        <v>0.0003819170659773676</v>
       </c>
       <c r="E80" s="9" t="n">
-        <v>0.02401319275623543</v>
+        <v>0.01346508697339823</v>
       </c>
       <c r="F80" s="9" t="n">
         <v>0.1297114447333514</v>
@@ -5813,7 +6265,7 @@
         <v>0.04239826333525394</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>0.06129129745559889</v>
+        <v>0.01418954230934598</v>
       </c>
     </row>
     <row r="4">
@@ -5835,7 +6287,7 @@
         <v>0.03838122897303223</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>0.01980455968018955</v>
+        <v>0.01071962159834464</v>
       </c>
     </row>
     <row r="5">
@@ -5857,7 +6309,7 @@
         <v>0.0370534553973652</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>0.02491094989735838</v>
+        <v>0.01785691413064642</v>
       </c>
     </row>
     <row r="6">
@@ -5879,7 +6331,7 @@
         <v>0.03526861812873507</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>0.0188233496030912</v>
+        <v>0.01018151128031412</v>
       </c>
     </row>
     <row r="7">
@@ -5901,7 +6353,7 @@
         <v>0.1901058368847075</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>0.06372964737267586</v>
+        <v>0.0596596557957153</v>
       </c>
     </row>
     <row r="8">
@@ -5923,7 +6375,7 @@
         <v>0.1561033628971746</v>
       </c>
       <c r="F8" s="47" t="n">
-        <v>0.3209896397522077</v>
+        <v>0.3316397889964033</v>
       </c>
     </row>
     <row r="9">
@@ -5945,7 +6397,7 @@
         <v>0.09891989158807808</v>
       </c>
       <c r="F9" s="46" t="n">
-        <v>0.1515664321754441</v>
+        <v>0.1092060125556164</v>
       </c>
     </row>
     <row r="10">
@@ -5967,7 +6419,7 @@
         <v>0.03310675547604956</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>0.0222215038737016</v>
+        <v>0.009319148736044227</v>
       </c>
     </row>
     <row r="11">
@@ -5989,7 +6441,7 @@
         <v>0.05454871770448565</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>0.01792687522994341</v>
+        <v>0.01805983719241161</v>
       </c>
     </row>
     <row r="12">
@@ -6010,8 +6462,8 @@
       <c r="E12" s="12" t="n">
         <v>0.07131481415928038</v>
       </c>
-      <c r="F12" s="12" t="n">
-        <v>0.06139883262218021</v>
+      <c r="F12" s="47" t="n">
+        <v>0.1483922296615784</v>
       </c>
     </row>
     <row r="13">
@@ -6033,7 +6485,7 @@
         <v>0.1147079339099366</v>
       </c>
       <c r="F13" s="46" t="n">
-        <v>0.1822438014945581</v>
+        <v>0.2280024325953268</v>
       </c>
     </row>
     <row r="14">
@@ -6055,7 +6507,7 @@
         <v>0.06079007889326719</v>
       </c>
       <c r="F14" s="12" t="n">
-        <v>0.02896140192186942</v>
+        <v>0.02821942763967997</v>
       </c>
     </row>
     <row r="15">
@@ -6077,7 +6529,7 @@
         <v>0.06730104265263419</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>0.02613170892118141</v>
+        <v>0.01455387750857305</v>
       </c>
     </row>
   </sheetData>
@@ -6087,4 +6539,869 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J86"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>FACTOR-LOADING CLUSTER ANALYSIS — ENHANCED HRP</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Ward linkage on z-scored factor betas  |  5-Factor Model  |  13 Asset Classes  |  Euclidean distance in standardised beta space  |  2004 Q4 to 2024 Q4</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="10" customHeight="1"/>
+    <row r="4" ht="22" customHeight="1">
+      <c r="B4" s="48" t="inlineStr">
+        <is>
+          <t>5-CLUSTER SOLUTION — ECONOMIC INTERPRETATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="B5" s="49" t="inlineStr">
+        <is>
+          <t>CLUSTER 1</t>
+        </is>
+      </c>
+      <c r="D5" s="50" t="inlineStr">
+        <is>
+          <t>CLUSTER 2</t>
+        </is>
+      </c>
+      <c r="F5" s="51" t="inlineStr">
+        <is>
+          <t>CLUSTER 3</t>
+        </is>
+      </c>
+      <c r="H5" s="52" t="inlineStr">
+        <is>
+          <t>CLUSTER 4</t>
+        </is>
+      </c>
+      <c r="J5" s="53" t="inlineStr">
+        <is>
+          <t>CLUSTER 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="B6" s="54" t="inlineStr">
+        <is>
+          <t>Yield-Seeking Diversifiers</t>
+        </is>
+      </c>
+      <c r="D6" s="55" t="inlineStr">
+        <is>
+          <t>Pure Rate Duration</t>
+        </is>
+      </c>
+      <c r="F6" s="56" t="inlineStr">
+        <is>
+          <t>Inflation Hedge</t>
+        </is>
+      </c>
+      <c r="H6" s="57" t="inlineStr">
+        <is>
+          <t>Domestic Equity Beta</t>
+        </is>
+      </c>
+      <c r="J6" s="58" t="inlineStr">
+        <is>
+          <t>Credit-Sensitive Equity</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="B7" s="59" t="inlineStr">
+        <is>
+          <t>Dominant: Equity Premium</t>
+        </is>
+      </c>
+      <c r="D7" s="59" t="inlineStr">
+        <is>
+          <t>Dominant: Term Premium</t>
+        </is>
+      </c>
+      <c r="F7" s="59" t="inlineStr">
+        <is>
+          <t>Dominant: Inflation</t>
+        </is>
+      </c>
+      <c r="H7" s="59" t="inlineStr">
+        <is>
+          <t>Dominant: Equity Premium</t>
+        </is>
+      </c>
+      <c r="J7" s="59" t="inlineStr">
+        <is>
+          <t>Dominant: Credit Spread</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="B8" s="60" t="inlineStr">
+        <is>
+          <t>TIPS
+Investment Grade Credit
+High Yield Credit
+Hedge Funds
+Private Equity
+Private Real Estate</t>
+        </is>
+      </c>
+      <c r="D8" s="60" t="inlineStr">
+        <is>
+          <t>Long Duration Treasury</t>
+        </is>
+      </c>
+      <c r="F8" s="60" t="inlineStr">
+        <is>
+          <t>Commodities</t>
+        </is>
+      </c>
+      <c r="H8" s="60" t="inlineStr">
+        <is>
+          <t>US Large Cap Equity
+US Mid Cap Equity
+US Small Cap Equity</t>
+        </is>
+      </c>
+      <c r="J8" s="60" t="inlineStr">
+        <is>
+          <t>Emerging Market Equity
+REITs</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="36" customHeight="1">
+      <c r="B9" s="61" t="inlineStr">
+        <is>
+          <t>Low equity beta complex. Credit and alternative assets sharing below-average equity exposure.</t>
+        </is>
+      </c>
+      <c r="D9" s="61" t="inlineStr">
+        <is>
+          <t>Positive term premium, negative equity beta. Sole rate hedge in universe.</t>
+        </is>
+      </c>
+      <c r="F9" s="61" t="inlineStr">
+        <is>
+          <t>Dominant inflation beta. Real commodity dynamics orthogonal to equity and credit.</t>
+        </is>
+      </c>
+      <c r="H9" s="61" t="inlineStr">
+        <is>
+          <t>High positive equity loading across all three size segments. Essentially same systematic risk.</t>
+        </is>
+      </c>
+      <c r="J9" s="61" t="inlineStr">
+        <is>
+          <t>High credit spread sensitivity, strongly negative liquidity beta. Seizes during credit stress.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="14" customHeight="1">
+      <c r="B10" s="62" t="inlineStr">
+        <is>
+          <t>ERP:  -0.66</t>
+        </is>
+      </c>
+      <c r="D10" s="62" t="inlineStr">
+        <is>
+          <t>ERP:  -1.01</t>
+        </is>
+      </c>
+      <c r="F10" s="62" t="inlineStr">
+        <is>
+          <t>ERP:  -1.03</t>
+        </is>
+      </c>
+      <c r="H10" s="63" t="inlineStr">
+        <is>
+          <t>ERP:  +1.33</t>
+        </is>
+      </c>
+      <c r="J10" s="63" t="inlineStr">
+        <is>
+          <t>ERP:  +1.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="14" customHeight="1">
+      <c r="B11" s="64" t="inlineStr">
+        <is>
+          <t>TERM:  +0.11</t>
+        </is>
+      </c>
+      <c r="D11" s="63" t="inlineStr">
+        <is>
+          <t>TERM:  +2.58</t>
+        </is>
+      </c>
+      <c r="F11" s="62" t="inlineStr">
+        <is>
+          <t>TERM:  -1.56</t>
+        </is>
+      </c>
+      <c r="H11" s="62" t="inlineStr">
+        <is>
+          <t>TERM:  -0.75</t>
+        </is>
+      </c>
+      <c r="J11" s="64" t="inlineStr">
+        <is>
+          <t>TERM:  +0.29</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="14" customHeight="1">
+      <c r="B12" s="64" t="inlineStr">
+        <is>
+          <t>CREDIT:  -0.45</t>
+        </is>
+      </c>
+      <c r="D12" s="62" t="inlineStr">
+        <is>
+          <t>CREDIT:  -0.83</t>
+        </is>
+      </c>
+      <c r="F12" s="63" t="inlineStr">
+        <is>
+          <t>CREDIT:  +0.98</t>
+        </is>
+      </c>
+      <c r="H12" s="64" t="inlineStr">
+        <is>
+          <t>CREDIT:  -0.43</t>
+        </is>
+      </c>
+      <c r="J12" s="63" t="inlineStr">
+        <is>
+          <t>CREDIT:  +1.93</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="14" customHeight="1">
+      <c r="B13" s="64" t="inlineStr">
+        <is>
+          <t>INFL:  +0.28</t>
+        </is>
+      </c>
+      <c r="D13" s="62" t="inlineStr">
+        <is>
+          <t>INFL:  -0.87</t>
+        </is>
+      </c>
+      <c r="F13" s="63" t="inlineStr">
+        <is>
+          <t>INFL:  +2.06</t>
+        </is>
+      </c>
+      <c r="H13" s="62" t="inlineStr">
+        <is>
+          <t>INFL:  -0.50</t>
+        </is>
+      </c>
+      <c r="J13" s="62" t="inlineStr">
+        <is>
+          <t>INFL:  -0.68</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="14" customHeight="1">
+      <c r="B14" s="64" t="inlineStr">
+        <is>
+          <t>LIQ:  +0.49</t>
+        </is>
+      </c>
+      <c r="D14" s="64" t="inlineStr">
+        <is>
+          <t>LIQ:  -0.22</t>
+        </is>
+      </c>
+      <c r="F14" s="63" t="inlineStr">
+        <is>
+          <t>LIQ:  +0.86</t>
+        </is>
+      </c>
+      <c r="H14" s="64" t="inlineStr">
+        <is>
+          <t>LIQ:  -0.03</t>
+        </is>
+      </c>
+      <c r="J14" s="62" t="inlineStr">
+        <is>
+          <t>LIQ:  -1.74</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="12" customHeight="1"/>
+    <row r="70" ht="20" customHeight="1">
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>FULL ASSET DETAIL — CLUSTER ASSIGNMENT AND STANDARDISED BETAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="7" t="inlineStr">
+        <is>
+          <t>Asset Class</t>
+        </is>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>Cl.</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>Cluster Name</t>
+        </is>
+      </c>
+      <c r="D71" s="7" t="inlineStr">
+        <is>
+          <t>ERP (z)</t>
+        </is>
+      </c>
+      <c r="E71" s="7" t="inlineStr">
+        <is>
+          <t>Term (z)</t>
+        </is>
+      </c>
+      <c r="F71" s="7" t="inlineStr">
+        <is>
+          <t>Credit (z)</t>
+        </is>
+      </c>
+      <c r="G71" s="7" t="inlineStr">
+        <is>
+          <t>Inflation (z)</t>
+        </is>
+      </c>
+      <c r="H71" s="7" t="inlineStr">
+        <is>
+          <t>Liquidity (z)</t>
+        </is>
+      </c>
+      <c r="I71" s="7" t="inlineStr">
+        <is>
+          <t>R-Sq</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="16" customHeight="1">
+      <c r="B72" s="65" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="C72" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="D72" s="67" t="inlineStr">
+        <is>
+          <t>Yield-Seeking Diversifiers</t>
+        </is>
+      </c>
+      <c r="E72" s="68" t="n">
+        <v>-0.269</v>
+      </c>
+      <c r="F72" s="68" t="n">
+        <v>-0.644</v>
+      </c>
+      <c r="G72" s="68" t="n">
+        <v>-0.231</v>
+      </c>
+      <c r="H72" s="68" t="n">
+        <v>0.198</v>
+      </c>
+      <c r="I72" s="69" t="n">
+        <v>0.906</v>
+      </c>
+      <c r="J72" s="70" t="n">
+        <v>0.4472956521780461</v>
+      </c>
+    </row>
+    <row r="73" ht="16" customHeight="1">
+      <c r="B73" s="71" t="inlineStr">
+        <is>
+          <t>Investment Grade Credit</t>
+        </is>
+      </c>
+      <c r="C73" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="D73" s="72" t="inlineStr">
+        <is>
+          <t>Yield-Seeking Diversifiers</t>
+        </is>
+      </c>
+      <c r="E73" s="73" t="n">
+        <v>-0.436</v>
+      </c>
+      <c r="F73" s="69" t="n">
+        <v>0.839</v>
+      </c>
+      <c r="G73" s="73" t="n">
+        <v>-0.6870000000000001</v>
+      </c>
+      <c r="H73" s="73" t="n">
+        <v>-0.546</v>
+      </c>
+      <c r="I73" s="73" t="n">
+        <v>0.054</v>
+      </c>
+      <c r="J73" s="33" t="n">
+        <v>0.6374629953920316</v>
+      </c>
+    </row>
+    <row r="74" ht="16" customHeight="1">
+      <c r="B74" s="65" t="inlineStr">
+        <is>
+          <t>Hedge Funds</t>
+        </is>
+      </c>
+      <c r="C74" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="D74" s="67" t="inlineStr">
+        <is>
+          <t>Yield-Seeking Diversifiers</t>
+        </is>
+      </c>
+      <c r="E74" s="68" t="n">
+        <v>-0.456</v>
+      </c>
+      <c r="F74" s="68" t="n">
+        <v>-0.499</v>
+      </c>
+      <c r="G74" s="68" t="n">
+        <v>-0.677</v>
+      </c>
+      <c r="H74" s="68" t="n">
+        <v>-0.192</v>
+      </c>
+      <c r="I74" s="68" t="n">
+        <v>0.07199999999999999</v>
+      </c>
+      <c r="J74" s="74" t="n">
+        <v>0.7443129475785015</v>
+      </c>
+    </row>
+    <row r="75" ht="16" customHeight="1">
+      <c r="B75" s="71" t="inlineStr">
+        <is>
+          <t>High Yield Credit</t>
+        </is>
+      </c>
+      <c r="C75" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="D75" s="72" t="inlineStr">
+        <is>
+          <t>Yield-Seeking Diversifiers</t>
+        </is>
+      </c>
+      <c r="E75" s="73" t="n">
+        <v>-0.578</v>
+      </c>
+      <c r="F75" s="73" t="n">
+        <v>0.183</v>
+      </c>
+      <c r="G75" s="73" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="H75" s="73" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="I75" s="75" t="n">
+        <v>2.197</v>
+      </c>
+      <c r="J75" s="16" t="n">
+        <v>0.8431315161474411</v>
+      </c>
+    </row>
+    <row r="76" ht="16" customHeight="1">
+      <c r="B76" s="65" t="inlineStr">
+        <is>
+          <t>TIPS</t>
+        </is>
+      </c>
+      <c r="C76" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="D76" s="67" t="inlineStr">
+        <is>
+          <t>Yield-Seeking Diversifiers</t>
+        </is>
+      </c>
+      <c r="E76" s="76" t="n">
+        <v>-1.027</v>
+      </c>
+      <c r="F76" s="68" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G76" s="76" t="n">
+        <v>-0.819</v>
+      </c>
+      <c r="H76" s="68" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="I76" s="68" t="n">
+        <v>-0.193</v>
+      </c>
+      <c r="J76" s="74" t="n">
+        <v>0.8015086616077469</v>
+      </c>
+    </row>
+    <row r="77" ht="16" customHeight="1">
+      <c r="B77" s="71" t="inlineStr">
+        <is>
+          <t>Private Real Estate</t>
+        </is>
+      </c>
+      <c r="C77" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="D77" s="72" t="inlineStr">
+        <is>
+          <t>Yield-Seeking Diversifiers</t>
+        </is>
+      </c>
+      <c r="E77" s="76" t="n">
+        <v>-1.17</v>
+      </c>
+      <c r="F77" s="73" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="G77" s="73" t="n">
+        <v>-0.771</v>
+      </c>
+      <c r="H77" s="75" t="n">
+        <v>1.641</v>
+      </c>
+      <c r="I77" s="73" t="n">
+        <v>-0.104</v>
+      </c>
+      <c r="J77" s="27" t="n">
+        <v>0.08716459731266091</v>
+      </c>
+    </row>
+    <row r="78" ht="16" customHeight="1">
+      <c r="B78" s="77" t="inlineStr">
+        <is>
+          <t>Long Duration Treasury</t>
+        </is>
+      </c>
+      <c r="C78" s="78" t="n">
+        <v>2</v>
+      </c>
+      <c r="D78" s="79" t="inlineStr">
+        <is>
+          <t>Pure Rate Duration</t>
+        </is>
+      </c>
+      <c r="E78" s="76" t="n">
+        <v>-1.014</v>
+      </c>
+      <c r="F78" s="75" t="n">
+        <v>2.582</v>
+      </c>
+      <c r="G78" s="76" t="n">
+        <v>-0.834</v>
+      </c>
+      <c r="H78" s="76" t="n">
+        <v>-0.867</v>
+      </c>
+      <c r="I78" s="68" t="n">
+        <v>-0.221</v>
+      </c>
+      <c r="J78" s="74" t="n">
+        <v>0.9812439847251684</v>
+      </c>
+    </row>
+    <row r="79" ht="16" customHeight="1">
+      <c r="B79" s="80" t="inlineStr">
+        <is>
+          <t>Commodities</t>
+        </is>
+      </c>
+      <c r="C79" s="81" t="n">
+        <v>3</v>
+      </c>
+      <c r="D79" s="82" t="inlineStr">
+        <is>
+          <t>Inflation Hedge</t>
+        </is>
+      </c>
+      <c r="E79" s="76" t="n">
+        <v>-1.034</v>
+      </c>
+      <c r="F79" s="83" t="n">
+        <v>-1.56</v>
+      </c>
+      <c r="G79" s="69" t="n">
+        <v>0.981</v>
+      </c>
+      <c r="H79" s="75" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="I79" s="69" t="n">
+        <v>0.865</v>
+      </c>
+      <c r="J79" s="33" t="n">
+        <v>0.4370483747153048</v>
+      </c>
+    </row>
+    <row r="80" ht="16" customHeight="1">
+      <c r="B80" s="84" t="inlineStr">
+        <is>
+          <t>US Small Cap Equity</t>
+        </is>
+      </c>
+      <c r="C80" s="85" t="n">
+        <v>4</v>
+      </c>
+      <c r="D80" s="86" t="inlineStr">
+        <is>
+          <t>Domestic Equity Beta</t>
+        </is>
+      </c>
+      <c r="E80" s="75" t="n">
+        <v>1.666</v>
+      </c>
+      <c r="F80" s="76" t="n">
+        <v>-1.037</v>
+      </c>
+      <c r="G80" s="68" t="n">
+        <v>-0.531</v>
+      </c>
+      <c r="H80" s="76" t="n">
+        <v>-0.853</v>
+      </c>
+      <c r="I80" s="68" t="n">
+        <v>-0.317</v>
+      </c>
+      <c r="J80" s="74" t="n">
+        <v>0.8712833012703342</v>
+      </c>
+    </row>
+    <row r="81" ht="16" customHeight="1">
+      <c r="B81" s="87" t="inlineStr">
+        <is>
+          <t>US Mid Cap Equity</t>
+        </is>
+      </c>
+      <c r="C81" s="85" t="n">
+        <v>4</v>
+      </c>
+      <c r="D81" s="88" t="inlineStr">
+        <is>
+          <t>Domestic Equity Beta</t>
+        </is>
+      </c>
+      <c r="E81" s="69" t="n">
+        <v>1.174</v>
+      </c>
+      <c r="F81" s="73" t="n">
+        <v>-0.672</v>
+      </c>
+      <c r="G81" s="73" t="n">
+        <v>-0.304</v>
+      </c>
+      <c r="H81" s="73" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="I81" s="73" t="n">
+        <v>0.407</v>
+      </c>
+      <c r="J81" s="16" t="n">
+        <v>0.9123635173053706</v>
+      </c>
+    </row>
+    <row r="82" ht="16" customHeight="1">
+      <c r="B82" s="84" t="inlineStr">
+        <is>
+          <t>US Large Cap Equity</t>
+        </is>
+      </c>
+      <c r="C82" s="85" t="n">
+        <v>4</v>
+      </c>
+      <c r="D82" s="86" t="inlineStr">
+        <is>
+          <t>Domestic Equity Beta</t>
+        </is>
+      </c>
+      <c r="E82" s="69" t="n">
+        <v>1.153</v>
+      </c>
+      <c r="F82" s="68" t="n">
+        <v>-0.529</v>
+      </c>
+      <c r="G82" s="68" t="n">
+        <v>-0.443</v>
+      </c>
+      <c r="H82" s="68" t="n">
+        <v>-0.458</v>
+      </c>
+      <c r="I82" s="68" t="n">
+        <v>-0.192</v>
+      </c>
+      <c r="J82" s="74" t="n">
+        <v>0.9906918940400172</v>
+      </c>
+    </row>
+    <row r="83" ht="16" customHeight="1">
+      <c r="B83" s="89" t="inlineStr">
+        <is>
+          <t>REITs</t>
+        </is>
+      </c>
+      <c r="C83" s="90" t="n">
+        <v>5</v>
+      </c>
+      <c r="D83" s="91" t="inlineStr">
+        <is>
+          <t>Credit-Sensitive Equity</t>
+        </is>
+      </c>
+      <c r="E83" s="75" t="n">
+        <v>1.321</v>
+      </c>
+      <c r="F83" s="73" t="n">
+        <v>0.503</v>
+      </c>
+      <c r="G83" s="75" t="n">
+        <v>2.588</v>
+      </c>
+      <c r="H83" s="83" t="n">
+        <v>-1.859</v>
+      </c>
+      <c r="I83" s="83" t="n">
+        <v>-2.023</v>
+      </c>
+      <c r="J83" s="33" t="n">
+        <v>0.6337080092805776</v>
+      </c>
+    </row>
+    <row r="84" ht="16" customHeight="1">
+      <c r="B84" s="92" t="inlineStr">
+        <is>
+          <t>Emerging Market Equity</t>
+        </is>
+      </c>
+      <c r="C84" s="90" t="n">
+        <v>5</v>
+      </c>
+      <c r="D84" s="93" t="inlineStr">
+        <is>
+          <t>Credit-Sensitive Equity</t>
+        </is>
+      </c>
+      <c r="E84" s="68" t="n">
+        <v>0.669</v>
+      </c>
+      <c r="F84" s="68" t="n">
+        <v>0.073</v>
+      </c>
+      <c r="G84" s="75" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="H84" s="68" t="n">
+        <v>0.491</v>
+      </c>
+      <c r="I84" s="83" t="n">
+        <v>-1.452</v>
+      </c>
+      <c r="J84" s="70" t="n">
+        <v>0.6355398384728477</v>
+      </c>
+    </row>
+    <row r="86" ht="14" customHeight="1">
+      <c r="B86" s="94" t="inlineStr">
+        <is>
+          <t>Green = positive factor tilt  |  Red = negative factor tilt  |  Bold = strong tilt (|z| &gt; 1.2)  |  R-sq: green &gt;= 0.70, amber &gt;= 0.40, red &lt; 0.40</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="45">
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="B1:J1"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="B86:J86"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B4:J4"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="B70:J70"/>
+    <mergeCell ref="B2:J2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: tracking error ddof=1, sortino semi-deviation, net beta normalisation
</commit_message>
<xml_diff>
--- a/analytics_report.xlsx
+++ b/analytics_report.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backtest Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio Analytics" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Factor Model" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stress Testing" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Decomposition" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Covariance" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Net Factor Exposure" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Backtest Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Portfolio Analytics" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Factor Model" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Stress Testing" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Risk Decomposition" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Covariance" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Net Factor Exposure" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -454,7 +454,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -469,13 +469,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -484,7 +484,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>2</col>
@@ -499,13 +499,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -524,13 +524,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -549,13 +549,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -574,13 +574,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -589,7 +589,7 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -604,13 +604,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -619,7 +619,7 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -634,13 +634,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1064,13 +1064,13 @@
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>0.06245310112278192</v>
+        <v>0.06245310112278191</v>
       </c>
       <c r="C9" s="12" t="n">
         <v>0.1128462018830994</v>
       </c>
       <c r="D9" s="13" t="n">
-        <v>0.5534355616813658</v>
+        <v>0.5534355616813655</v>
       </c>
       <c r="E9" s="13" t="n">
         <v>1.04098829241875</v>
@@ -1092,25 +1092,25 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>0.07315951727129649</v>
+        <v>0.07315951727129666</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>0.08814883647169879</v>
+        <v>0.08814883647169917</v>
       </c>
       <c r="D10" s="10" t="n">
-        <v>0.8299544293450227</v>
+        <v>0.8299544293450209</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>1.707951735971823</v>
+        <v>1.707951735971837</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>-0.1999559307284841</v>
+        <v>-0.1999559307284849</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>0.3658782062865555</v>
+        <v>0.3658782062865549</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>0.05566283756079447</v>
+        <v>0.05566283756079451</v>
       </c>
     </row>
     <row r="11">
@@ -1120,25 +1120,25 @@
         </is>
       </c>
       <c r="B11" s="12" t="n">
-        <v>0.05891136643510455</v>
+        <v>0.05891136643505968</v>
       </c>
       <c r="C11" s="12" t="n">
-        <v>0.0693118656153645</v>
+        <v>0.06931186561532279</v>
       </c>
       <c r="D11" s="13" t="n">
-        <v>0.8499463390875105</v>
+        <v>0.8499463390873745</v>
       </c>
       <c r="E11" s="13" t="n">
-        <v>1.563746143547528</v>
+        <v>1.563746143545916</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>-0.1665091655056802</v>
+        <v>-0.1665091655061419</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.3538025444797205</v>
+        <v>0.35380254447847</v>
       </c>
       <c r="H11" s="12" t="n">
-        <v>0.05681108284766658</v>
+        <v>0.0568110828478045</v>
       </c>
     </row>
     <row r="12">
@@ -1151,10 +1151,10 @@
         <v>0.05191532254690638</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>0.05672701063600803</v>
+        <v>0.05672701063600805</v>
       </c>
       <c r="D12" s="10" t="n">
-        <v>0.9151781834587387</v>
+        <v>0.9151781834587384</v>
       </c>
       <c r="E12" s="10" t="n">
         <v>1.720196379330979</v>
@@ -1574,13 +1574,13 @@
         </is>
       </c>
       <c r="B4" s="12" t="n">
-        <v>0.06245310112278192</v>
+        <v>0.06245310112278191</v>
       </c>
       <c r="C4" s="12" t="n">
         <v>0.1128462018830994</v>
       </c>
       <c r="D4" s="26" t="n">
-        <v>0.5534355616813658</v>
+        <v>0.5534355616813655</v>
       </c>
       <c r="E4" s="13" t="n">
         <v>1.04098829241875</v>
@@ -1602,25 +1602,25 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.07315951727129649</v>
+        <v>0.07315951727129666</v>
       </c>
       <c r="C5" s="9" t="n">
-        <v>0.08814883647169879</v>
+        <v>0.08814883647169917</v>
       </c>
       <c r="D5" s="27" t="n">
-        <v>0.8299544293450227</v>
+        <v>0.8299544293450209</v>
       </c>
       <c r="E5" s="10" t="n">
-        <v>1.707951735971823</v>
+        <v>1.707951735971837</v>
       </c>
       <c r="F5" s="28" t="n">
-        <v>-0.1999559307284841</v>
+        <v>-0.1999559307284849</v>
       </c>
       <c r="G5" s="10" t="n">
-        <v>0.3658782062865555</v>
+        <v>0.3658782062865549</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>0.05566283756079447</v>
+        <v>0.05566283756079451</v>
       </c>
     </row>
     <row r="6">
@@ -1630,25 +1630,25 @@
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v>0.05891136643510455</v>
+        <v>0.05891136643505968</v>
       </c>
       <c r="C6" s="12" t="n">
-        <v>0.0693118656153645</v>
+        <v>0.06931186561532279</v>
       </c>
       <c r="D6" s="29" t="n">
-        <v>0.8499463390875105</v>
+        <v>0.8499463390873745</v>
       </c>
       <c r="E6" s="13" t="n">
-        <v>1.563746143547528</v>
+        <v>1.563746143545916</v>
       </c>
       <c r="F6" s="30" t="n">
-        <v>-0.1665091655056802</v>
+        <v>-0.1665091655061419</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.3538025444797205</v>
+        <v>0.35380254447847</v>
       </c>
       <c r="H6" s="12" t="n">
-        <v>0.05681108284766658</v>
+        <v>0.0568110828478045</v>
       </c>
     </row>
     <row r="7">
@@ -1661,10 +1661,10 @@
         <v>0.05191532254690638</v>
       </c>
       <c r="C7" s="9" t="n">
-        <v>0.05672701063600803</v>
+        <v>0.05672701063600805</v>
       </c>
       <c r="D7" s="27" t="n">
-        <v>0.9151781834587387</v>
+        <v>0.9151781834587384</v>
       </c>
       <c r="E7" s="10" t="n">
         <v>1.720196379330979</v>
@@ -1721,7 +1721,7 @@
         <v>0.03956381298337185</v>
       </c>
       <c r="C31" s="28" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.3846153846153845</v>
       </c>
       <c r="D31" s="32" t="inlineStr">
         <is>
@@ -1754,10 +1754,10 @@
         </is>
       </c>
       <c r="B33" s="9" t="n">
-        <v>0.05566283756079447</v>
+        <v>0.05566283756079451</v>
       </c>
       <c r="C33" s="16" t="n">
-        <v>0.6755292397488624</v>
+        <v>0.6755292397488672</v>
       </c>
       <c r="D33" s="32" t="inlineStr">
         <is>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="B34" s="12" t="n">
-        <v>0.05681108284766658</v>
+        <v>0.0568110828478045</v>
       </c>
       <c r="C34" s="30" t="n">
-        <v>0.448205120433019</v>
+        <v>0.4482051204348193</v>
       </c>
       <c r="D34" s="34" t="inlineStr">
         <is>
@@ -1793,7 +1793,7 @@
         <v>0.06544241006043219</v>
       </c>
       <c r="C35" s="16" t="n">
-        <v>0.6355342602606396</v>
+        <v>0.6355342602606397</v>
       </c>
       <c r="D35" s="32" t="inlineStr">
         <is>
@@ -1927,19 +1927,19 @@
         </is>
       </c>
       <c r="B3" s="35" t="n">
-        <v>0.9625042408608266</v>
+        <v>0.9625042408608269</v>
       </c>
       <c r="C3" s="35" t="n">
-        <v>0.0234555669595009</v>
+        <v>0.02345556695950097</v>
       </c>
       <c r="D3" s="35" t="n">
-        <v>0.9221660405720561</v>
+        <v>0.9221660405720516</v>
       </c>
       <c r="E3" s="35" t="n">
-        <v>0.3996132467526641</v>
+        <v>0.3996132467526616</v>
       </c>
       <c r="F3" s="35" t="n">
-        <v>-0.005854488358147542</v>
+        <v>-0.005854488358147634</v>
       </c>
       <c r="G3" s="9" t="n">
         <v>0</v>
@@ -1963,16 +1963,16 @@
         <v>0.9713542877937703</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>-0.02791969853016988</v>
+        <v>-0.02791969853016975</v>
       </c>
       <c r="D4" s="36" t="n">
-        <v>1.307588071319309</v>
+        <v>1.307588071319306</v>
       </c>
       <c r="E4" s="36" t="n">
-        <v>2.069722843884615</v>
+        <v>2.069722843884614</v>
       </c>
       <c r="F4" s="36" t="n">
-        <v>0.03673514360340343</v>
+        <v>0.03673514360340332</v>
       </c>
       <c r="G4" s="12" t="n">
         <v>0</v>
@@ -1996,16 +1996,16 @@
         <v>1.184029795675607</v>
       </c>
       <c r="C5" s="35" t="n">
-        <v>-0.1590176041375174</v>
+        <v>-0.1590176041375175</v>
       </c>
       <c r="D5" s="35" t="n">
-        <v>0.6769370592425008</v>
+        <v>0.676937059242492</v>
       </c>
       <c r="E5" s="35" t="n">
-        <v>-2.052830116472312</v>
+        <v>-2.052830116472316</v>
       </c>
       <c r="F5" s="35" t="n">
-        <v>-0.01476517062835918</v>
+        <v>-0.01476517062835937</v>
       </c>
       <c r="G5" s="9" t="n">
         <v>0</v>
@@ -2026,19 +2026,19 @@
         </is>
       </c>
       <c r="B6" s="36" t="n">
-        <v>0.7532197633494773</v>
+        <v>0.7532197633494774</v>
       </c>
       <c r="C6" s="36" t="n">
         <v>0.2392008134777396</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>5.685573550590403</v>
+        <v>5.685573550590397</v>
       </c>
       <c r="E6" s="36" t="n">
         <v>6.29629067295865</v>
       </c>
       <c r="F6" s="36" t="n">
-        <v>-0.09556594450963732</v>
+        <v>-0.09556594450963743</v>
       </c>
       <c r="G6" s="12" t="n">
         <v>0</v>
@@ -2059,19 +2059,19 @@
         </is>
       </c>
       <c r="B7" s="35" t="n">
-        <v>0.0252225065068102</v>
+        <v>0.02522250650681003</v>
       </c>
       <c r="C7" s="35" t="n">
         <v>1.139230258689664</v>
       </c>
       <c r="D7" s="35" t="n">
-        <v>-0.1658015292723474</v>
+        <v>-0.1658015292723478</v>
       </c>
       <c r="E7" s="35" t="n">
-        <v>-2.135877837199863</v>
+        <v>-2.135877837199861</v>
       </c>
       <c r="F7" s="35" t="n">
-        <v>-0.007930514856370094</v>
+        <v>-0.007930514856369857</v>
       </c>
       <c r="G7" s="9" t="n">
         <v>0</v>
@@ -2092,25 +2092,25 @@
         </is>
       </c>
       <c r="B8" s="36" t="n">
-        <v>0.01944828438149542</v>
+        <v>0.0194482843814953</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>0.4459887403586636</v>
+        <v>0.4459887403586637</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>-0.1250616872544205</v>
+        <v>-0.1250616872544132</v>
       </c>
       <c r="E8" s="36" t="n">
-        <v>6.421673019699718</v>
+        <v>6.421673019699722</v>
       </c>
       <c r="F8" s="36" t="n">
-        <v>-0.005981872260687733</v>
+        <v>-0.005981872260688031</v>
       </c>
       <c r="G8" s="12" t="n">
         <v>0</v>
       </c>
       <c r="H8" s="12" t="n">
-        <v>0.8015086616077466</v>
+        <v>0.8015086616077469</v>
       </c>
       <c r="I8" s="22" t="inlineStr">
         <is>
@@ -2125,19 +2125,19 @@
         </is>
       </c>
       <c r="B9" s="35" t="n">
-        <v>0.2750954294387476</v>
+        <v>0.2750954294387477</v>
       </c>
       <c r="C9" s="35" t="n">
         <v>0.5137951400731287</v>
       </c>
       <c r="D9" s="35" t="n">
-        <v>0.242991449215862</v>
+        <v>0.2429914492158691</v>
       </c>
       <c r="E9" s="35" t="n">
-        <v>-0.1457078507988908</v>
+        <v>-0.1457078507988893</v>
       </c>
       <c r="F9" s="35" t="n">
-        <v>0.01162261473965012</v>
+        <v>0.01162261473964993</v>
       </c>
       <c r="G9" s="9" t="n">
         <v>0</v>
@@ -2161,22 +2161,22 @@
         <v>1.035110339377469</v>
       </c>
       <c r="C10" s="36" t="n">
-        <v>0.3934971993740882</v>
+        <v>0.3934971993740877</v>
       </c>
       <c r="D10" s="36" t="n">
-        <v>9.35242161574546</v>
+        <v>9.352421615745463</v>
       </c>
       <c r="E10" s="36" t="n">
-        <v>-8.299634434854095</v>
+        <v>-8.299634434854106</v>
       </c>
       <c r="F10" s="36" t="n">
-        <v>-0.13621110133405</v>
+        <v>-0.136211101334049</v>
       </c>
       <c r="G10" s="12" t="n">
         <v>0</v>
       </c>
       <c r="H10" s="12" t="n">
-        <v>0.6337080092805774</v>
+        <v>0.6337080092805776</v>
       </c>
       <c r="I10" s="22" t="inlineStr">
         <is>
@@ -2191,19 +2191,19 @@
         </is>
       </c>
       <c r="B11" s="35" t="n">
-        <v>0.01657438583919307</v>
+        <v>0.01657438583919279</v>
       </c>
       <c r="C11" s="35" t="n">
-        <v>-0.3464828245407029</v>
+        <v>-0.3464828245407032</v>
       </c>
       <c r="D11" s="35" t="n">
-        <v>4.883589691416407</v>
+        <v>4.883589691416405</v>
       </c>
       <c r="E11" s="35" t="n">
-        <v>16.03885891630619</v>
+        <v>16.0388589163062</v>
       </c>
       <c r="F11" s="35" t="n">
-        <v>0.06933460659340056</v>
+        <v>0.06933460659340032</v>
       </c>
       <c r="G11" s="9" t="n">
         <v>0</v>
@@ -2227,16 +2227,16 @@
         <v>0.2139108894699562</v>
       </c>
       <c r="C12" s="36" t="n">
-        <v>0.2787451901424916</v>
+        <v>0.2787451901424915</v>
       </c>
       <c r="D12" s="36" t="n">
         <v>3.43229865495527</v>
       </c>
       <c r="E12" s="36" t="n">
-        <v>3.647889816547429</v>
+        <v>3.647889816547432</v>
       </c>
       <c r="F12" s="36" t="n">
-        <v>0.1641715585741691</v>
+        <v>0.1641715585741692</v>
       </c>
       <c r="G12" s="12" t="n">
         <v>0</v>
@@ -2260,16 +2260,16 @@
         <v>0.2662615280266115</v>
       </c>
       <c r="C13" s="35" t="n">
-        <v>0.03413008712923789</v>
+        <v>0.03413008712923776</v>
       </c>
       <c r="D13" s="35" t="n">
-        <v>0.2697224940806265</v>
+        <v>0.2697224940806349</v>
       </c>
       <c r="E13" s="35" t="n">
         <v>2.055745923262592</v>
       </c>
       <c r="F13" s="35" t="n">
-        <v>0.01290119732786074</v>
+        <v>0.01290119732786036</v>
       </c>
       <c r="G13" s="9" t="n">
         <v>0</v>
@@ -2290,25 +2290,25 @@
         </is>
       </c>
       <c r="B14" s="36" t="n">
-        <v>0.3475645787692834</v>
+        <v>0.3475645787692835</v>
       </c>
       <c r="C14" s="36" t="n">
-        <v>-0.01789473558713036</v>
+        <v>-0.01789473558713058</v>
       </c>
       <c r="D14" s="36" t="n">
-        <v>1.510698166693949</v>
+        <v>1.510698166693959</v>
       </c>
       <c r="E14" s="36" t="n">
-        <v>4.47479691252725</v>
+        <v>4.474796912527248</v>
       </c>
       <c r="F14" s="36" t="n">
-        <v>0.07225876810085399</v>
+        <v>0.07225876810085358</v>
       </c>
       <c r="G14" s="12" t="n">
         <v>0</v>
       </c>
       <c r="H14" s="12" t="n">
-        <v>0.447295652178046</v>
+        <v>0.4472956521780461</v>
       </c>
       <c r="I14" s="22" t="inlineStr">
         <is>
@@ -2323,25 +2323,25 @@
         </is>
       </c>
       <c r="B15" s="35" t="n">
-        <v>-0.04225721639330339</v>
+        <v>-0.0422572163933037</v>
       </c>
       <c r="C15" s="35" t="n">
-        <v>0.2525396594451279</v>
+        <v>0.2525396594451277</v>
       </c>
       <c r="D15" s="35" t="n">
-        <v>0.008416326420856109</v>
+        <v>0.008416326420867809</v>
       </c>
       <c r="E15" s="35" t="n">
-        <v>13.43606605605532</v>
+        <v>13.43606605605533</v>
       </c>
       <c r="F15" s="35" t="n">
-        <v>0.0004025644516648638</v>
+        <v>0.0004025644516642721</v>
       </c>
       <c r="G15" s="9" t="n">
         <v>0</v>
       </c>
       <c r="H15" s="9" t="n">
-        <v>0.08716459731266069</v>
+        <v>0.08716459731266091</v>
       </c>
       <c r="I15" s="19" t="inlineStr">
         <is>
@@ -2394,13 +2394,13 @@
         </is>
       </c>
       <c r="B19" s="35" t="n">
-        <v>0.01657438583919307</v>
+        <v>0.01657438583919279</v>
       </c>
       <c r="C19" s="35" t="n">
-        <v>0.6128143614867044</v>
+        <v>0.612814361486727</v>
       </c>
       <c r="D19" s="35" t="n">
-        <v>0.5962399756475114</v>
+        <v>0.5962399756475342</v>
       </c>
       <c r="E19" s="19" t="inlineStr">
         <is>
@@ -2415,13 +2415,13 @@
         </is>
       </c>
       <c r="B20" s="36" t="n">
-        <v>-0.04225721639330339</v>
+        <v>-0.0422572163933037</v>
       </c>
       <c r="C20" s="36" t="n">
-        <v>0.1943926134830142</v>
+        <v>0.1943926134830137</v>
       </c>
       <c r="D20" s="36" t="n">
-        <v>0.2366498298763176</v>
+        <v>0.2366498298763174</v>
       </c>
       <c r="E20" s="22" t="inlineStr">
         <is>
@@ -2439,10 +2439,10 @@
         <v>0.2139108894699562</v>
       </c>
       <c r="C21" s="35" t="n">
-        <v>0.2968736681280802</v>
+        <v>0.2968736681282671</v>
       </c>
       <c r="D21" s="35" t="n">
-        <v>0.08296277865812401</v>
+        <v>0.08296277865831087</v>
       </c>
       <c r="E21" s="19" t="inlineStr">
         <is>
@@ -2457,13 +2457,13 @@
         </is>
       </c>
       <c r="B22" s="36" t="n">
-        <v>0.01944828438149542</v>
+        <v>0.0194482843814953</v>
       </c>
       <c r="C22" s="36" t="n">
-        <v>0.1007620091545411</v>
+        <v>0.1007620091545305</v>
       </c>
       <c r="D22" s="36" t="n">
-        <v>0.08131372477304566</v>
+        <v>0.08131372477303518</v>
       </c>
       <c r="E22" s="22" t="inlineStr">
         <is>
@@ -2478,13 +2478,13 @@
         </is>
       </c>
       <c r="B23" s="35" t="n">
-        <v>0.0252225065068102</v>
+        <v>0.02522250650681003</v>
       </c>
       <c r="C23" s="35" t="n">
-        <v>0.07165021511634978</v>
+        <v>0.07165021511635317</v>
       </c>
       <c r="D23" s="35" t="n">
-        <v>0.04642770860953958</v>
+        <v>0.04642770860954314</v>
       </c>
       <c r="E23" s="19" t="inlineStr">
         <is>
@@ -2499,13 +2499,13 @@
         </is>
       </c>
       <c r="B24" s="36" t="n">
-        <v>0.9625042408608266</v>
+        <v>0.9625042408608269</v>
       </c>
       <c r="C24" s="36" t="n">
-        <v>0.9793425414193194</v>
+        <v>0.9793425414193206</v>
       </c>
       <c r="D24" s="36" t="n">
-        <v>0.01683830055849278</v>
+        <v>0.01683830055849378</v>
       </c>
       <c r="E24" s="22" t="inlineStr">
         <is>
@@ -2523,10 +2523,10 @@
         <v>1.035110339377469</v>
       </c>
       <c r="C25" s="35" t="n">
-        <v>1.031110052707944</v>
+        <v>1.031110052707938</v>
       </c>
       <c r="D25" s="35" t="n">
-        <v>-0.004000286669525455</v>
+        <v>-0.004000286669531006</v>
       </c>
       <c r="E25" s="19" t="inlineStr">
         <is>
@@ -2541,13 +2541,13 @@
         </is>
       </c>
       <c r="B26" s="36" t="n">
-        <v>0.7532197633494773</v>
+        <v>0.7532197633494774</v>
       </c>
       <c r="C26" s="36" t="n">
-        <v>0.744929893975867</v>
+        <v>0.7449298939758666</v>
       </c>
       <c r="D26" s="36" t="n">
-        <v>-0.008289869373610315</v>
+        <v>-0.008289869373610759</v>
       </c>
       <c r="E26" s="22" t="inlineStr">
         <is>
@@ -2562,13 +2562,13 @@
         </is>
       </c>
       <c r="B27" s="35" t="n">
-        <v>0.2750954294387476</v>
+        <v>0.2750954294387477</v>
       </c>
       <c r="C27" s="35" t="n">
-        <v>0.2323437215866304</v>
+        <v>0.2323437215866302</v>
       </c>
       <c r="D27" s="35" t="n">
-        <v>-0.04275170785211721</v>
+        <v>-0.04275170785211746</v>
       </c>
       <c r="E27" s="19" t="inlineStr">
         <is>
@@ -2583,13 +2583,13 @@
         </is>
       </c>
       <c r="B28" s="36" t="n">
-        <v>0.3475645787692834</v>
+        <v>0.3475645787692835</v>
       </c>
       <c r="C28" s="36" t="n">
-        <v>0.2923064843573309</v>
+        <v>0.2923064843573329</v>
       </c>
       <c r="D28" s="36" t="n">
-        <v>-0.05525809441195256</v>
+        <v>-0.05525809441195068</v>
       </c>
       <c r="E28" s="22" t="inlineStr">
         <is>
@@ -2607,10 +2607,10 @@
         <v>0.2662615280266115</v>
       </c>
       <c r="C29" s="35" t="n">
-        <v>0.1884016479536867</v>
+        <v>0.1884016479536835</v>
       </c>
       <c r="D29" s="35" t="n">
-        <v>-0.07785988007292477</v>
+        <v>-0.07785988007292804</v>
       </c>
       <c r="E29" s="19" t="inlineStr">
         <is>
@@ -2628,10 +2628,10 @@
         <v>0.9713542877937703</v>
       </c>
       <c r="C30" s="36" t="n">
-        <v>0.81507742405682</v>
+        <v>0.8150774240568861</v>
       </c>
       <c r="D30" s="36" t="n">
-        <v>-0.1562768637369503</v>
+        <v>-0.1562768637368842</v>
       </c>
       <c r="E30" s="22" t="inlineStr">
         <is>
@@ -2649,10 +2649,10 @@
         <v>1.184029795675607</v>
       </c>
       <c r="C31" s="35" t="n">
-        <v>0.9628322446122726</v>
+        <v>0.9628322446122715</v>
       </c>
       <c r="D31" s="35" t="n">
-        <v>-0.2211975510633342</v>
+        <v>-0.2211975510633357</v>
       </c>
       <c r="E31" s="19" t="inlineStr">
         <is>
@@ -2771,16 +2771,16 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>-0.1830486748285108</v>
+        <v>-0.1830486748285078</v>
       </c>
       <c r="C5" s="9" t="n">
-        <v>0.03683695337861526</v>
+        <v>0.03683695337861703</v>
       </c>
       <c r="D5" s="9" t="n">
-        <v>-0.1786484994678722</v>
+        <v>-0.1786484994678725</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>0.5145573060842663</v>
+        <v>0.5145573060842727</v>
       </c>
     </row>
     <row r="6">
@@ -2790,16 +2790,16 @@
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v>-0.1665091655056802</v>
+        <v>-0.1665091655061418</v>
       </c>
       <c r="C6" s="12" t="n">
-        <v>0.01971956610044479</v>
+        <v>0.01971956610018144</v>
       </c>
       <c r="D6" s="12" t="n">
-        <v>-0.1449286097239181</v>
+        <v>-0.1449286097236309</v>
       </c>
       <c r="E6" s="12" t="n">
-        <v>0.3378735970067459</v>
+        <v>0.3378735970052109</v>
       </c>
     </row>
     <row r="7">
@@ -2818,7 +2818,7 @@
         <v>-0.1166178609836621</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>0.3183738177155637</v>
+        <v>0.3183738177155639</v>
       </c>
     </row>
   </sheetData>
@@ -2922,7 +2922,7 @@
         <v>0.1129636311829188</v>
       </c>
       <c r="F4" s="9" t="n">
-        <v>0.9718498340506941</v>
+        <v>0.9718498340506938</v>
       </c>
     </row>
     <row r="5">
@@ -2935,16 +2935,16 @@
         <v>0.07692307692307693</v>
       </c>
       <c r="C5" s="36" t="n">
-        <v>0.0867109415098225</v>
+        <v>0.08671094150982253</v>
       </c>
       <c r="D5" s="36" t="n">
-        <v>0.006670072423832502</v>
+        <v>0.006670072423832504</v>
       </c>
       <c r="E5" s="12" t="n">
         <v>0.1288018186574803</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>0.9005695345361189</v>
+        <v>0.9005695345361184</v>
       </c>
     </row>
     <row r="6">
@@ -2957,16 +2957,16 @@
         <v>0.07692307692307693</v>
       </c>
       <c r="C6" s="35" t="n">
-        <v>0.09160479264684694</v>
+        <v>0.09160479264684693</v>
       </c>
       <c r="D6" s="35" t="n">
-        <v>0.00704652251129592</v>
+        <v>0.007046522511295919</v>
       </c>
       <c r="E6" s="9" t="n">
         <v>0.1360712233682609</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>0.8647852106386996</v>
+        <v>0.8647852106386994</v>
       </c>
     </row>
     <row r="7">
@@ -2988,7 +2988,7 @@
         <v>0.1333256415144526</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>0.6547256214279523</v>
+        <v>0.6547256214279519</v>
       </c>
     </row>
     <row r="8">
@@ -3001,16 +3001,16 @@
         <v>0.07692307692307693</v>
       </c>
       <c r="C8" s="35" t="n">
-        <v>-0.01890725699586818</v>
+        <v>-0.01890725699586819</v>
       </c>
       <c r="D8" s="35" t="n">
         <v>-0.001454404384297553</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>-0.02808514178820585</v>
+        <v>-0.02808514178820586</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>0.9800395309996238</v>
+        <v>0.9800395309996239</v>
       </c>
     </row>
     <row r="9">
@@ -3023,13 +3023,13 @@
         <v>0.07692307692307693</v>
       </c>
       <c r="C9" s="36" t="n">
-        <v>0.0099511054760176</v>
+        <v>0.009951105476017614</v>
       </c>
       <c r="D9" s="36" t="n">
-        <v>0.000765469652001354</v>
+        <v>0.0007654696520013551</v>
       </c>
       <c r="E9" s="12" t="n">
-        <v>0.01478153114988708</v>
+        <v>0.0147815311498871</v>
       </c>
       <c r="F9" s="12" t="n">
         <v>0.8261546883028913</v>
@@ -3045,16 +3045,16 @@
         <v>0.07692307692307693</v>
       </c>
       <c r="C10" s="35" t="n">
-        <v>0.01592770997060339</v>
+        <v>0.01592770997060341</v>
       </c>
       <c r="D10" s="35" t="n">
-        <v>0.001225208459277184</v>
+        <v>0.001225208459277186</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>0.02365927500660577</v>
+        <v>0.0236592750066058</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>0.6542475111182807</v>
+        <v>0.6542475111182804</v>
       </c>
     </row>
     <row r="11">
@@ -3067,16 +3067,16 @@
         <v>0.07692307692307693</v>
       </c>
       <c r="C11" s="36" t="n">
-        <v>0.08804865704708363</v>
+        <v>0.08804865704708366</v>
       </c>
       <c r="D11" s="36" t="n">
-        <v>0.006772973619006434</v>
+        <v>0.006772973619006437</v>
       </c>
       <c r="E11" s="12" t="n">
         <v>0.1307888827009042</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>0.643251444348571</v>
+        <v>0.6432514443485702</v>
       </c>
     </row>
     <row r="12">
@@ -3089,16 +3089,16 @@
         <v>0.07692307692307693</v>
       </c>
       <c r="C12" s="35" t="n">
-        <v>0.07513341722441097</v>
+        <v>0.075133417224411</v>
       </c>
       <c r="D12" s="35" t="n">
-        <v>0.005779493632646999</v>
+        <v>0.005779493632647001</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>0.111604379008607</v>
+        <v>0.1116043790086071</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>0.4797912934834941</v>
+        <v>0.4797912934834942</v>
       </c>
     </row>
     <row r="13">
@@ -3111,13 +3111,13 @@
         <v>0.07692307692307693</v>
       </c>
       <c r="C13" s="36" t="n">
-        <v>0.03992411329824732</v>
+        <v>0.03992411329824733</v>
       </c>
       <c r="D13" s="36" t="n">
-        <v>0.003071085638326718</v>
+        <v>0.003071085638326719</v>
       </c>
       <c r="E13" s="12" t="n">
-        <v>0.05930391610981454</v>
+        <v>0.05930391610981455</v>
       </c>
       <c r="F13" s="12" t="n">
         <v>0.6813173339403511</v>
@@ -3133,13 +3133,13 @@
         <v>0.07692307692307693</v>
       </c>
       <c r="C14" s="35" t="n">
-        <v>0.02736526641155148</v>
+        <v>0.0273652664115515</v>
       </c>
       <c r="D14" s="35" t="n">
-        <v>0.002105020493196268</v>
+        <v>0.002105020493196269</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>0.04064880418182309</v>
+        <v>0.04064880418182311</v>
       </c>
       <c r="F14" s="9" t="n">
         <v>0.7487919560463553</v>
@@ -3155,16 +3155,16 @@
         <v>0.07692307692307693</v>
       </c>
       <c r="C15" s="36" t="n">
-        <v>0.05235587803403792</v>
+        <v>0.05235587803403795</v>
       </c>
       <c r="D15" s="36" t="n">
-        <v>0.004027375233387533</v>
+        <v>0.004027375233387536</v>
       </c>
       <c r="E15" s="12" t="n">
-        <v>0.07777025817934878</v>
+        <v>0.07777025817934882</v>
       </c>
       <c r="F15" s="12" t="n">
-        <v>0.4284467817562572</v>
+        <v>0.4284467817562575</v>
       </c>
     </row>
     <row r="16">
@@ -3177,16 +3177,16 @@
         <v>0.07692307692307693</v>
       </c>
       <c r="C16" s="35" t="n">
-        <v>0.03929254921739967</v>
+        <v>0.03929254921739969</v>
       </c>
       <c r="D16" s="35" t="n">
-        <v>0.003022503785953822</v>
+        <v>0.003022503785953823</v>
       </c>
       <c r="E16" s="9" t="n">
-        <v>0.05836578072810263</v>
+        <v>0.05836578072810264</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>0.1297114447333512</v>
+        <v>0.1297114447333514</v>
       </c>
     </row>
     <row r="18">
@@ -3252,7 +3252,7 @@
         <v>0.1592867957876898</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>0.9718498340506941</v>
+        <v>0.9718498340506938</v>
       </c>
     </row>
     <row r="21">
@@ -3274,7 +3274,7 @@
         <v>0.1785964511717921</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>0.9005695345361189</v>
+        <v>0.9005695345361184</v>
       </c>
     </row>
     <row r="22">
@@ -3287,16 +3287,16 @@
         <v>0.12</v>
       </c>
       <c r="C22" s="35" t="n">
-        <v>0.09111479827874774</v>
+        <v>0.09111479827874773</v>
       </c>
       <c r="D22" s="35" t="n">
         <v>0.01093377579344973</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>0.1937819015792191</v>
+        <v>0.193781901579219</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>0.8647852106386996</v>
+        <v>0.8647852106386994</v>
       </c>
     </row>
     <row r="23">
@@ -3309,7 +3309,7 @@
         <v>0.12</v>
       </c>
       <c r="C23" s="36" t="n">
-        <v>0.08745089141391918</v>
+        <v>0.08745089141391921</v>
       </c>
       <c r="D23" s="36" t="n">
         <v>0.0104941069696703</v>
@@ -3318,7 +3318,7 @@
         <v>0.1859895467379832</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.6547256214279523</v>
+        <v>0.6547256214279519</v>
       </c>
     </row>
     <row r="24">
@@ -3331,16 +3331,16 @@
         <v>0.1333333333333333</v>
       </c>
       <c r="C24" s="35" t="n">
-        <v>-0.002026303910268674</v>
+        <v>-0.002026303910268667</v>
       </c>
       <c r="D24" s="35" t="n">
-        <v>-0.0002701738547024898</v>
+        <v>-0.000270173854702489</v>
       </c>
       <c r="E24" s="9" t="n">
-        <v>-0.004788355304724753</v>
+        <v>-0.004788355304724739</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>0.9800395309996238</v>
+        <v>0.9800395309996239</v>
       </c>
     </row>
     <row r="25">
@@ -3353,13 +3353,13 @@
         <v>0.1333333333333333</v>
       </c>
       <c r="C25" s="36" t="n">
-        <v>0.01128184223015829</v>
+        <v>0.01128184223015831</v>
       </c>
       <c r="D25" s="36" t="n">
-        <v>0.001504245630687772</v>
+        <v>0.001504245630687774</v>
       </c>
       <c r="E25" s="12" t="n">
-        <v>0.02666010207850971</v>
+        <v>0.02666010207850974</v>
       </c>
       <c r="F25" s="12" t="n">
         <v>0.8261546883028913</v>
@@ -3375,16 +3375,16 @@
         <v>0.1333333333333333</v>
       </c>
       <c r="C26" s="35" t="n">
-        <v>0.02366079429953972</v>
+        <v>0.02366079429953975</v>
       </c>
       <c r="D26" s="35" t="n">
-        <v>0.003154772573271963</v>
+        <v>0.003154772573271966</v>
       </c>
       <c r="E26" s="9" t="n">
-        <v>0.05591278254167706</v>
+        <v>0.05591278254167711</v>
       </c>
       <c r="F26" s="9" t="n">
-        <v>0.6542475111182807</v>
+        <v>0.6542475111182804</v>
       </c>
     </row>
     <row r="27">
@@ -3397,16 +3397,16 @@
         <v>0.12</v>
       </c>
       <c r="C27" s="36" t="n">
-        <v>0.09618294399599181</v>
+        <v>0.0961829439959918</v>
       </c>
       <c r="D27" s="36" t="n">
-        <v>0.01154195327951902</v>
+        <v>0.01154195327951901</v>
       </c>
       <c r="E27" s="12" t="n">
         <v>0.2045607754078538</v>
       </c>
       <c r="F27" s="12" t="n">
-        <v>0.643251444348571</v>
+        <v>0.6432514443485702</v>
       </c>
     </row>
     <row r="28">
@@ -3419,7 +3419,7 @@
         <v>0</v>
       </c>
       <c r="C28" s="35" t="n">
-        <v>0.04363145447238433</v>
+        <v>0.04363145447238432</v>
       </c>
       <c r="D28" s="35" t="n">
         <v>0</v>
@@ -3428,7 +3428,7 @@
         <v>0</v>
       </c>
       <c r="F28" s="9" t="n">
-        <v>0.4797912934834941</v>
+        <v>0.4797912934834942</v>
       </c>
     </row>
     <row r="29">
@@ -3441,7 +3441,7 @@
         <v>0</v>
       </c>
       <c r="C29" s="36" t="n">
-        <v>0.03736801761619854</v>
+        <v>0.03736801761619855</v>
       </c>
       <c r="D29" s="36" t="n">
         <v>0</v>
@@ -3463,7 +3463,7 @@
         <v>0</v>
       </c>
       <c r="C30" s="35" t="n">
-        <v>0.02593079077558951</v>
+        <v>0.02593079077558953</v>
       </c>
       <c r="D30" s="35" t="n">
         <v>0</v>
@@ -3485,7 +3485,7 @@
         <v>0</v>
       </c>
       <c r="C31" s="36" t="n">
-        <v>0.03961123437025103</v>
+        <v>0.03961123437025107</v>
       </c>
       <c r="D31" s="36" t="n">
         <v>0</v>
@@ -3494,7 +3494,7 @@
         <v>0</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.4284467817562572</v>
+        <v>0.4284467817562575</v>
       </c>
     </row>
     <row r="32">
@@ -3507,7 +3507,7 @@
         <v>0</v>
       </c>
       <c r="C32" s="35" t="n">
-        <v>0.01678542567237087</v>
+        <v>0.01678542567237088</v>
       </c>
       <c r="D32" s="35" t="n">
         <v>0</v>
@@ -3516,7 +3516,7 @@
         <v>0</v>
       </c>
       <c r="F32" s="9" t="n">
-        <v>0.1297114447333512</v>
+        <v>0.1297114447333514</v>
       </c>
     </row>
     <row r="34">
@@ -3570,19 +3570,19 @@
         </is>
       </c>
       <c r="B36" s="9" t="n">
-        <v>1.540461442864476e-08</v>
+        <v>1.540461288441797e-08</v>
       </c>
       <c r="C36" s="35" t="n">
-        <v>0.05604810820385811</v>
+        <v>0.05604810820385785</v>
       </c>
       <c r="D36" s="35" t="n">
-        <v>8.633994963353952e-10</v>
+        <v>8.633994097844016e-10</v>
       </c>
       <c r="E36" s="9" t="n">
-        <v>1.958958350204883e-08</v>
+        <v>1.958958153830204e-08</v>
       </c>
       <c r="F36" s="9" t="n">
-        <v>0.9718498340506941</v>
+        <v>0.9718498340506938</v>
       </c>
     </row>
     <row r="37">
@@ -3592,19 +3592,19 @@
         </is>
       </c>
       <c r="B37" s="12" t="n">
-        <v>1.28614030174759e-08</v>
+        <v>1.286140172707754e-08</v>
       </c>
       <c r="C37" s="36" t="n">
-        <v>0.05994390698587164</v>
+        <v>0.05994390698587128</v>
       </c>
       <c r="D37" s="36" t="n">
-        <v>7.709627461873842e-10</v>
+        <v>7.709626688358602e-10</v>
       </c>
       <c r="E37" s="12" t="n">
-        <v>1.749229546404531e-08</v>
+        <v>1.749229370902436e-08</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>0.9005695345361189</v>
+        <v>0.9005695345361184</v>
       </c>
     </row>
     <row r="38">
@@ -3614,19 +3614,19 @@
         </is>
       </c>
       <c r="B38" s="9" t="n">
-        <v>1.034391881227816e-08</v>
+        <v>1.034391777355504e-08</v>
       </c>
       <c r="C38" s="35" t="n">
-        <v>0.06375923942128763</v>
+        <v>0.06375923942128729</v>
       </c>
       <c r="D38" s="35" t="n">
-        <v>6.595203961064042e-10</v>
+        <v>6.595203298782051e-10</v>
       </c>
       <c r="E38" s="9" t="n">
-        <v>1.496379129900713e-08</v>
+        <v>1.496378979636218e-08</v>
       </c>
       <c r="F38" s="9" t="n">
-        <v>0.8647852106386996</v>
+        <v>0.8647852106386994</v>
       </c>
     </row>
     <row r="39">
@@ -3636,19 +3636,19 @@
         </is>
       </c>
       <c r="B39" s="12" t="n">
-        <v>0.07113737017120601</v>
+        <v>0.07113737017120696</v>
       </c>
       <c r="C39" s="36" t="n">
-        <v>0.06717134055346052</v>
+        <v>0.0671713405534603</v>
       </c>
       <c r="D39" s="36" t="n">
-        <v>0.004778392517847663</v>
+        <v>0.004778392517847712</v>
       </c>
       <c r="E39" s="12" t="n">
-        <v>0.1084164626354841</v>
+        <v>0.1084164626354847</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>0.6547256214279523</v>
+        <v>0.6547256214279519</v>
       </c>
     </row>
     <row r="40">
@@ -3658,19 +3658,19 @@
         </is>
       </c>
       <c r="B40" s="9" t="n">
-        <v>0.2963200956729806</v>
+        <v>0.2963200956729828</v>
       </c>
       <c r="C40" s="35" t="n">
-        <v>0.02027839680564883</v>
+        <v>0.02027839680564917</v>
       </c>
       <c r="D40" s="35" t="n">
-        <v>0.006008896481544524</v>
+        <v>0.00600889648154467</v>
       </c>
       <c r="E40" s="9" t="n">
-        <v>0.1363352421214034</v>
+        <v>0.1363352421214061</v>
       </c>
       <c r="F40" s="9" t="n">
-        <v>0.9800395309996238</v>
+        <v>0.9800395309996239</v>
       </c>
     </row>
     <row r="41">
@@ -3680,16 +3680,16 @@
         </is>
       </c>
       <c r="B41" s="12" t="n">
-        <v>9.201563042783877e-09</v>
+        <v>9.201562116762712e-09</v>
       </c>
       <c r="C41" s="36" t="n">
-        <v>0.01515708195138129</v>
+        <v>0.01515708195138125</v>
       </c>
       <c r="D41" s="36" t="n">
-        <v>1.394688451202766e-10</v>
+        <v>1.394688310844975e-10</v>
       </c>
       <c r="E41" s="12" t="n">
-        <v>3.164394465151101e-09</v>
+        <v>3.164394146694722e-09</v>
       </c>
       <c r="F41" s="12" t="n">
         <v>0.8261546883028913</v>
@@ -3702,19 +3702,19 @@
         </is>
       </c>
       <c r="B42" s="9" t="n">
-        <v>8.935098891791349e-09</v>
+        <v>8.935097992254681e-09</v>
       </c>
       <c r="C42" s="35" t="n">
-        <v>0.02639673412319072</v>
+        <v>0.02639673412319088</v>
       </c>
       <c r="D42" s="35" t="n">
-        <v>2.358574298110323e-10</v>
+        <v>2.358574060662035e-10</v>
       </c>
       <c r="E42" s="9" t="n">
-        <v>5.351345275822377e-09</v>
+        <v>5.351344737078344e-09</v>
       </c>
       <c r="F42" s="9" t="n">
-        <v>0.6542475111182807</v>
+        <v>0.6542475111182804</v>
       </c>
     </row>
     <row r="43">
@@ -3724,19 +3724,19 @@
         </is>
       </c>
       <c r="B43" s="12" t="n">
-        <v>0.1364634563400886</v>
+        <v>0.1364634563400894</v>
       </c>
       <c r="C43" s="36" t="n">
-        <v>0.08498129605168174</v>
+        <v>0.08498129605168149</v>
       </c>
       <c r="D43" s="36" t="n">
-        <v>0.01159684138347282</v>
+        <v>0.01159684138347285</v>
       </c>
       <c r="E43" s="12" t="n">
-        <v>0.2631195565966686</v>
+        <v>0.2631195565966681</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>0.643251444348571</v>
+        <v>0.6432514443485702</v>
       </c>
     </row>
     <row r="44">
@@ -3746,19 +3746,19 @@
         </is>
       </c>
       <c r="B44" s="9" t="n">
-        <v>2.096350346927755e-08</v>
+        <v>2.096350137433955e-08</v>
       </c>
       <c r="C44" s="35" t="n">
-        <v>0.02052878880749777</v>
+        <v>0.02052878880749672</v>
       </c>
       <c r="D44" s="35" t="n">
-        <v>4.303553353860456e-10</v>
+        <v>4.303552923794839e-10</v>
       </c>
       <c r="E44" s="9" t="n">
-        <v>9.764288505934306e-09</v>
+        <v>9.764287530162752e-09</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>0.4797912934834941</v>
+        <v>0.4797912934834942</v>
       </c>
     </row>
     <row r="45">
@@ -3768,16 +3768,16 @@
         </is>
       </c>
       <c r="B45" s="12" t="n">
-        <v>0.1960790013757557</v>
+        <v>0.1960790013757596</v>
       </c>
       <c r="C45" s="36" t="n">
-        <v>0.03660795132295</v>
+        <v>0.03660795132295001</v>
       </c>
       <c r="D45" s="36" t="n">
-        <v>0.007178050537816312</v>
+        <v>0.007178050537816456</v>
       </c>
       <c r="E45" s="12" t="n">
-        <v>0.162862059787276</v>
+        <v>0.1628620597872786</v>
       </c>
       <c r="F45" s="12" t="n">
         <v>0.6813173339403511</v>
@@ -3790,16 +3790,16 @@
         </is>
       </c>
       <c r="B46" s="9" t="n">
-        <v>1.618598447722783e-09</v>
+        <v>1.618598277387212e-09</v>
       </c>
       <c r="C46" s="35" t="n">
-        <v>0.02013819062703096</v>
+        <v>0.02013819062703088</v>
       </c>
       <c r="D46" s="35" t="n">
-        <v>3.259564408885779e-11</v>
+        <v>3.259564065860747e-11</v>
       </c>
       <c r="E46" s="9" t="n">
-        <v>7.39559258943208e-10</v>
+        <v>7.395591811146036e-10</v>
       </c>
       <c r="F46" s="9" t="n">
         <v>0.7487919560463553</v>
@@ -3812,19 +3812,19 @@
         </is>
       </c>
       <c r="B47" s="12" t="n">
-        <v>0.2822620050016614</v>
+        <v>0.2822620050016704</v>
       </c>
       <c r="C47" s="36" t="n">
-        <v>0.04946939446322393</v>
+        <v>0.04946939446322386</v>
       </c>
       <c r="D47" s="36" t="n">
-        <v>0.01396333046740768</v>
+        <v>0.0139633304674081</v>
       </c>
       <c r="E47" s="12" t="n">
-        <v>0.3168125871267913</v>
+        <v>0.3168125871267995</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>0.4284467817562572</v>
+        <v>0.4284467817562575</v>
       </c>
     </row>
     <row r="48">
@@ -3834,19 +3834,19 @@
         </is>
       </c>
       <c r="B48" s="9" t="n">
-        <v>0.01773799210960737</v>
+        <v>0.01773799210959868</v>
       </c>
       <c r="C48" s="35" t="n">
-        <v>0.03094508737001937</v>
+        <v>0.03094508737001761</v>
       </c>
       <c r="D48" s="35" t="n">
-        <v>0.0005489037156005142</v>
+        <v>0.0005489037156002144</v>
       </c>
       <c r="E48" s="9" t="n">
-        <v>0.01245402066711899</v>
+        <v>0.01245402066711213</v>
       </c>
       <c r="F48" s="9" t="n">
-        <v>0.1297114447333512</v>
+        <v>0.1297114447333514</v>
       </c>
     </row>
     <row r="50">
@@ -3900,19 +3900,19 @@
         </is>
       </c>
       <c r="B52" s="9" t="n">
-        <v>0.04239826333589958</v>
+        <v>0.04239826333525394</v>
       </c>
       <c r="C52" s="35" t="n">
-        <v>0.06287655228621657</v>
+        <v>0.06287655228620767</v>
       </c>
       <c r="D52" s="35" t="n">
-        <v>0.00266585662148447</v>
+        <v>0.002665856621443495</v>
       </c>
       <c r="E52" s="9" t="n">
-        <v>0.07692352810926284</v>
+        <v>0.0769235281081268</v>
       </c>
       <c r="F52" s="9" t="n">
-        <v>0.9718498340506941</v>
+        <v>0.9718498340506938</v>
       </c>
     </row>
     <row r="53">
@@ -3922,19 +3922,19 @@
         </is>
       </c>
       <c r="B53" s="12" t="n">
-        <v>0.03838122897153512</v>
+        <v>0.03838122897303223</v>
       </c>
       <c r="C53" s="36" t="n">
-        <v>0.06945530211246037</v>
+        <v>0.06945530211249798</v>
       </c>
       <c r="D53" s="36" t="n">
-        <v>0.002665779853665489</v>
+        <v>0.002665779853770914</v>
       </c>
       <c r="E53" s="12" t="n">
-        <v>0.0769213129670704</v>
+        <v>0.07692131297015872</v>
       </c>
       <c r="F53" s="12" t="n">
-        <v>0.9005695345361189</v>
+        <v>0.9005695345361184</v>
       </c>
     </row>
     <row r="54">
@@ -3944,19 +3944,19 @@
         </is>
       </c>
       <c r="B54" s="9" t="n">
-        <v>0.03705345539751015</v>
+        <v>0.0370534553973652</v>
       </c>
       <c r="C54" s="35" t="n">
-        <v>0.0719460643679987</v>
+        <v>0.07194606436802295</v>
       </c>
       <c r="D54" s="35" t="n">
-        <v>0.002665850287086035</v>
+        <v>0.002665850287076504</v>
       </c>
       <c r="E54" s="9" t="n">
-        <v>0.07692334532963691</v>
+        <v>0.07692334532940817</v>
       </c>
       <c r="F54" s="9" t="n">
-        <v>0.8647852106386996</v>
+        <v>0.8647852106386994</v>
       </c>
     </row>
     <row r="55">
@@ -3966,19 +3966,19 @@
         </is>
       </c>
       <c r="B55" s="12" t="n">
-        <v>0.03526861812925119</v>
+        <v>0.03526861812873507</v>
       </c>
       <c r="C55" s="36" t="n">
-        <v>0.07558698122436444</v>
+        <v>0.07558698122430507</v>
       </c>
       <c r="D55" s="36" t="n">
-        <v>0.002665848376344989</v>
+        <v>0.002665848376303882</v>
       </c>
       <c r="E55" s="12" t="n">
-        <v>0.0769232901950354</v>
+        <v>0.07692329019389553</v>
       </c>
       <c r="F55" s="12" t="n">
-        <v>0.6547256214279523</v>
+        <v>0.6547256214279519</v>
       </c>
     </row>
     <row r="56">
@@ -3988,19 +3988,19 @@
         </is>
       </c>
       <c r="B56" s="9" t="n">
-        <v>0.1901058368842273</v>
+        <v>0.1901058368847075</v>
       </c>
       <c r="C56" s="35" t="n">
-        <v>0.01402297004717164</v>
+        <v>0.01402297004707323</v>
       </c>
       <c r="D56" s="35" t="n">
-        <v>0.002665848456420016</v>
+        <v>0.002665848456408041</v>
       </c>
       <c r="E56" s="9" t="n">
-        <v>0.07692329250560737</v>
+        <v>0.07692329250530809</v>
       </c>
       <c r="F56" s="9" t="n">
-        <v>0.9800395309996238</v>
+        <v>0.9800395309996239</v>
       </c>
     </row>
     <row r="57">
@@ -4010,16 +4010,16 @@
         </is>
       </c>
       <c r="B57" s="12" t="n">
-        <v>0.1561033628963286</v>
+        <v>0.1561033628971746</v>
       </c>
       <c r="C57" s="36" t="n">
-        <v>0.01707722545810178</v>
+        <v>0.01707722545808812</v>
       </c>
       <c r="D57" s="36" t="n">
-        <v>0.002665812322948484</v>
+        <v>0.002665812322960799</v>
       </c>
       <c r="E57" s="12" t="n">
-        <v>0.07692224987109705</v>
+        <v>0.07692224987149869</v>
       </c>
       <c r="F57" s="12" t="n">
         <v>0.8261546883028913</v>
@@ -4032,19 +4032,19 @@
         </is>
       </c>
       <c r="B58" s="9" t="n">
-        <v>0.0989198915904857</v>
+        <v>0.09891989158807808</v>
       </c>
       <c r="C58" s="35" t="n">
-        <v>0.02695041436466309</v>
+        <v>0.02695041436455389</v>
       </c>
       <c r="D58" s="35" t="n">
-        <v>0.002665932067271142</v>
+        <v>0.002665932067195453</v>
       </c>
       <c r="E58" s="9" t="n">
-        <v>0.07692570510409633</v>
+        <v>0.07692570510195859</v>
       </c>
       <c r="F58" s="9" t="n">
-        <v>0.6542475111182807</v>
+        <v>0.6542475111182804</v>
       </c>
     </row>
     <row r="59">
@@ -4054,19 +4054,19 @@
         </is>
       </c>
       <c r="B59" s="12" t="n">
-        <v>0.03310675547563253</v>
+        <v>0.03310675547604956</v>
       </c>
       <c r="C59" s="36" t="n">
-        <v>0.08052175975617794</v>
+        <v>0.08052175975620805</v>
       </c>
       <c r="D59" s="36" t="n">
-        <v>0.002665814210715412</v>
+        <v>0.002665814210749987</v>
       </c>
       <c r="E59" s="12" t="n">
-        <v>0.07692230434277839</v>
+        <v>0.07692230434382233</v>
       </c>
       <c r="F59" s="12" t="n">
-        <v>0.643251444348571</v>
+        <v>0.6432514443485702</v>
       </c>
     </row>
     <row r="60">
@@ -4076,19 +4076,19 @@
         </is>
       </c>
       <c r="B60" s="9" t="n">
-        <v>0.05454871770404718</v>
+        <v>0.05454871770448565</v>
       </c>
       <c r="C60" s="35" t="n">
-        <v>0.04887037300549023</v>
+        <v>0.04887037300574652</v>
       </c>
       <c r="D60" s="35" t="n">
-        <v>0.002665816181167974</v>
+        <v>0.002665816181203382</v>
       </c>
       <c r="E60" s="9" t="n">
-        <v>0.07692236120036099</v>
+        <v>0.07692236120142895</v>
       </c>
       <c r="F60" s="9" t="n">
-        <v>0.4797912934834941</v>
+        <v>0.4797912934834942</v>
       </c>
     </row>
     <row r="61">
@@ -4098,16 +4098,16 @@
         </is>
       </c>
       <c r="B61" s="12" t="n">
-        <v>0.07131481416206895</v>
+        <v>0.07131481415928038</v>
       </c>
       <c r="C61" s="36" t="n">
-        <v>0.03738288332129727</v>
+        <v>0.03738288332119384</v>
       </c>
       <c r="D61" s="36" t="n">
-        <v>0.002665953376900622</v>
+        <v>0.002665953376789001</v>
       </c>
       <c r="E61" s="12" t="n">
-        <v>0.07692631999533582</v>
+        <v>0.07692631999216128</v>
       </c>
       <c r="F61" s="12" t="n">
         <v>0.6813173339403511</v>
@@ -4120,16 +4120,16 @@
         </is>
       </c>
       <c r="B62" s="9" t="n">
-        <v>0.1147079339070491</v>
+        <v>0.1147079339099366</v>
       </c>
       <c r="C62" s="35" t="n">
-        <v>0.02323949153589772</v>
+        <v>0.0232394915358965</v>
       </c>
       <c r="D62" s="35" t="n">
-        <v>0.002665754059133183</v>
+        <v>0.002665754059200145</v>
       </c>
       <c r="E62" s="9" t="n">
-        <v>0.07692056866356399</v>
+        <v>0.07692056866554249</v>
       </c>
       <c r="F62" s="9" t="n">
         <v>0.7487919560463553</v>
@@ -4142,19 +4142,19 @@
         </is>
       </c>
       <c r="B63" s="12" t="n">
-        <v>0.06079007889478735</v>
+        <v>0.06079007889326719</v>
       </c>
       <c r="C63" s="36" t="n">
-        <v>0.04385430184748499</v>
+        <v>0.04385430184744837</v>
       </c>
       <c r="D63" s="36" t="n">
-        <v>0.002665906469184431</v>
+        <v>0.002665906469115539</v>
       </c>
       <c r="E63" s="12" t="n">
-        <v>0.07692496646904494</v>
+        <v>0.07692496646710331</v>
       </c>
       <c r="F63" s="12" t="n">
-        <v>0.4284467817562572</v>
+        <v>0.4284467817562575</v>
       </c>
     </row>
     <row r="64">
@@ -4164,19 +4164,19 @@
         </is>
       </c>
       <c r="B64" s="9" t="n">
-        <v>0.06730104265117719</v>
+        <v>0.06730104265263419</v>
       </c>
       <c r="C64" s="35" t="n">
-        <v>0.03960949816448898</v>
+        <v>0.0396094981648834</v>
       </c>
       <c r="D64" s="35" t="n">
-        <v>0.002665760525359998</v>
+        <v>0.002665760525444253</v>
       </c>
       <c r="E64" s="9" t="n">
-        <v>0.07692075524710948</v>
+        <v>0.07692075524958694</v>
       </c>
       <c r="F64" s="9" t="n">
-        <v>0.1297114447333512</v>
+        <v>0.1297114447333514</v>
       </c>
     </row>
     <row r="66">
@@ -4230,10 +4230,10 @@
         </is>
       </c>
       <c r="B68" s="9" t="n">
-        <v>0.01418954230934599</v>
+        <v>0.01418954230934598</v>
       </c>
       <c r="C68" s="35" t="n">
-        <v>0.06214559548003216</v>
+        <v>0.0621455954800322</v>
       </c>
       <c r="D68" s="35" t="n">
         <v>0.0008818175564034171</v>
@@ -4242,7 +4242,7 @@
         <v>0.03108986518121491</v>
       </c>
       <c r="F68" s="9" t="n">
-        <v>0.9718498340506941</v>
+        <v>0.9718498340506938</v>
       </c>
     </row>
     <row r="69">
@@ -4252,19 +4252,19 @@
         </is>
       </c>
       <c r="B69" s="12" t="n">
-        <v>0.01071962159834465</v>
+        <v>0.01071962159834464</v>
       </c>
       <c r="C69" s="36" t="n">
-        <v>0.06881032714615794</v>
+        <v>0.06881032714615799</v>
       </c>
       <c r="D69" s="36" t="n">
-        <v>0.0007376206690651155</v>
+        <v>0.0007376206690651157</v>
       </c>
       <c r="E69" s="12" t="n">
         <v>0.0260059770749458</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>0.9005695345361189</v>
+        <v>0.9005695345361184</v>
       </c>
     </row>
     <row r="70">
@@ -4274,19 +4274,19 @@
         </is>
       </c>
       <c r="B70" s="9" t="n">
-        <v>0.01785691413064644</v>
+        <v>0.01785691413064642</v>
       </c>
       <c r="C70" s="35" t="n">
-        <v>0.06998047058406635</v>
+        <v>0.0699804705840664</v>
       </c>
       <c r="D70" s="35" t="n">
         <v>0.001249635254041901</v>
       </c>
       <c r="E70" s="9" t="n">
-        <v>0.04405785674342173</v>
+        <v>0.04405785674342171</v>
       </c>
       <c r="F70" s="9" t="n">
-        <v>0.8647852106386996</v>
+        <v>0.8647852106386994</v>
       </c>
     </row>
     <row r="71">
@@ -4296,19 +4296,19 @@
         </is>
       </c>
       <c r="B71" s="12" t="n">
-        <v>0.01018151128031413</v>
+        <v>0.01018151128031412</v>
       </c>
       <c r="C71" s="36" t="n">
-        <v>0.07713721713992756</v>
+        <v>0.07713721713992762</v>
       </c>
       <c r="D71" s="36" t="n">
-        <v>0.0007853734464422126</v>
+        <v>0.0007853734464422128</v>
       </c>
       <c r="E71" s="12" t="n">
         <v>0.02768957636359879</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>0.6547256214279523</v>
+        <v>0.6547256214279519</v>
       </c>
     </row>
     <row r="72">
@@ -4318,19 +4318,19 @@
         </is>
       </c>
       <c r="B72" s="9" t="n">
-        <v>0.05965965579571525</v>
+        <v>0.0596596557957153</v>
       </c>
       <c r="C72" s="35" t="n">
-        <v>0.01185652218885519</v>
+        <v>0.01185652218885514</v>
       </c>
       <c r="D72" s="35" t="n">
-        <v>0.0007073560327213609</v>
+        <v>0.0007073560327213587</v>
       </c>
       <c r="E72" s="9" t="n">
-        <v>0.024938949709871</v>
+        <v>0.02493894970987092</v>
       </c>
       <c r="F72" s="9" t="n">
-        <v>0.9800395309996238</v>
+        <v>0.9800395309996239</v>
       </c>
     </row>
     <row r="73">
@@ -4340,16 +4340,16 @@
         </is>
       </c>
       <c r="B73" s="12" t="n">
-        <v>0.3316397889964035</v>
+        <v>0.3316397889964033</v>
       </c>
       <c r="C73" s="36" t="n">
         <v>0.01854942338164661</v>
       </c>
       <c r="D73" s="36" t="n">
-        <v>0.006151726856294234</v>
+        <v>0.00615172685629423</v>
       </c>
       <c r="E73" s="12" t="n">
-        <v>0.2168888079002479</v>
+        <v>0.2168888079002477</v>
       </c>
       <c r="F73" s="12" t="n">
         <v>0.8261546883028913</v>
@@ -4362,19 +4362,19 @@
         </is>
       </c>
       <c r="B74" s="9" t="n">
-        <v>0.1092060125556165</v>
+        <v>0.1092060125556164</v>
       </c>
       <c r="C74" s="35" t="n">
-        <v>0.02838237345122104</v>
+        <v>0.02838237345122105</v>
       </c>
       <c r="D74" s="35" t="n">
-        <v>0.00309952583147224</v>
+        <v>0.003099525831472238</v>
       </c>
       <c r="E74" s="9" t="n">
-        <v>0.1092786592038321</v>
+        <v>0.109278659203832</v>
       </c>
       <c r="F74" s="9" t="n">
-        <v>0.6542475111182807</v>
+        <v>0.6542475111182804</v>
       </c>
     </row>
     <row r="75">
@@ -4384,19 +4384,19 @@
         </is>
       </c>
       <c r="B75" s="12" t="n">
-        <v>0.009319148736044234</v>
+        <v>0.009319148736044227</v>
       </c>
       <c r="C75" s="36" t="n">
-        <v>0.07416805794013152</v>
+        <v>0.07416805794013157</v>
       </c>
       <c r="D75" s="36" t="n">
-        <v>0.000691183163407632</v>
+        <v>0.0006911831634076319</v>
       </c>
       <c r="E75" s="12" t="n">
-        <v>0.02436874975988587</v>
+        <v>0.02436874975988586</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>0.643251444348571</v>
+        <v>0.6432514443485702</v>
       </c>
     </row>
     <row r="76">
@@ -4406,19 +4406,19 @@
         </is>
       </c>
       <c r="B76" s="9" t="n">
-        <v>0.01805983719241162</v>
+        <v>0.01805983719241161</v>
       </c>
       <c r="C76" s="35" t="n">
-        <v>0.04543999203099211</v>
+        <v>0.04543999203099216</v>
       </c>
       <c r="D76" s="35" t="n">
-        <v>0.0008206388581041986</v>
+        <v>0.0008206388581041992</v>
       </c>
       <c r="E76" s="9" t="n">
-        <v>0.02893291392948142</v>
+        <v>0.02893291392948143</v>
       </c>
       <c r="F76" s="9" t="n">
-        <v>0.4797912934834941</v>
+        <v>0.4797912934834942</v>
       </c>
     </row>
     <row r="77">
@@ -4428,16 +4428,16 @@
         </is>
       </c>
       <c r="B77" s="12" t="n">
-        <v>0.1483922296615783</v>
+        <v>0.1483922296615784</v>
       </c>
       <c r="C77" s="36" t="n">
-        <v>0.04167679313253375</v>
+        <v>0.04167679313253376</v>
       </c>
       <c r="D77" s="36" t="n">
-        <v>0.006184512258081034</v>
+        <v>0.006184512258081044</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>0.2180447088165564</v>
+        <v>0.2180447088165566</v>
       </c>
       <c r="F77" s="12" t="n">
         <v>0.6813173339403511</v>
@@ -4450,16 +4450,16 @@
         </is>
       </c>
       <c r="B78" s="9" t="n">
-        <v>0.2280024325953267</v>
+        <v>0.2280024325953268</v>
       </c>
       <c r="C78" s="35" t="n">
-        <v>0.02412051657055183</v>
+        <v>0.02412051657055184</v>
       </c>
       <c r="D78" s="35" t="n">
-        <v>0.005499536453541702</v>
+        <v>0.005499536453541706</v>
       </c>
       <c r="E78" s="9" t="n">
-        <v>0.1938948092586714</v>
+        <v>0.1938948092586715</v>
       </c>
       <c r="F78" s="9" t="n">
         <v>0.7487919560463553</v>
@@ -4472,19 +4472,19 @@
         </is>
       </c>
       <c r="B79" s="12" t="n">
-        <v>0.02821942763967994</v>
+        <v>0.02821942763967997</v>
       </c>
       <c r="C79" s="36" t="n">
-        <v>0.0415551260438286</v>
+        <v>0.04155512604382863</v>
       </c>
       <c r="D79" s="36" t="n">
-        <v>0.0011726618724516</v>
+        <v>0.001172661872451602</v>
       </c>
       <c r="E79" s="12" t="n">
-        <v>0.04134403908487437</v>
+        <v>0.04134403908487444</v>
       </c>
       <c r="F79" s="12" t="n">
-        <v>0.4284467817562572</v>
+        <v>0.4284467817562575</v>
       </c>
     </row>
     <row r="80">
@@ -4494,19 +4494,19 @@
         </is>
       </c>
       <c r="B80" s="9" t="n">
-        <v>0.01455387750857303</v>
+        <v>0.01455387750857305</v>
       </c>
       <c r="C80" s="35" t="n">
-        <v>0.0262416023326015</v>
+        <v>0.02624160233260154</v>
       </c>
       <c r="D80" s="35" t="n">
-        <v>0.0003819170659773665</v>
+        <v>0.0003819170659773675</v>
       </c>
       <c r="E80" s="9" t="n">
-        <v>0.0134650869733982</v>
+        <v>0.01346508697339823</v>
       </c>
       <c r="F80" s="9" t="n">
-        <v>0.1297114447333512</v>
+        <v>0.1297114447333514</v>
       </c>
     </row>
   </sheetData>
@@ -5309,7 +5309,7 @@
         </is>
       </c>
       <c r="C20" s="36" t="n">
-        <v>0.9564794466324268</v>
+        <v>0.9564794466324271</v>
       </c>
       <c r="D20" s="22" t="inlineStr">
         <is>
@@ -5334,7 +5334,7 @@
         </is>
       </c>
       <c r="C21" s="35" t="n">
-        <v>0.9327840363384615</v>
+        <v>0.9327840363384619</v>
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
@@ -5359,7 +5359,7 @@
         </is>
       </c>
       <c r="C22" s="36" t="n">
-        <v>0.8818708712318348</v>
+        <v>0.8818708712318351</v>
       </c>
       <c r="D22" s="22" t="inlineStr">
         <is>
@@ -5384,7 +5384,7 @@
         </is>
       </c>
       <c r="C23" s="35" t="n">
-        <v>0.877259056473388</v>
+        <v>0.8772590564733882</v>
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
@@ -5409,7 +5409,7 @@
         </is>
       </c>
       <c r="C24" s="36" t="n">
-        <v>0.8442031212496384</v>
+        <v>0.8442031212496387</v>
       </c>
       <c r="D24" s="22" t="inlineStr">
         <is>
@@ -5434,7 +5434,7 @@
         </is>
       </c>
       <c r="C25" s="35" t="n">
-        <v>0.8378878973040724</v>
+        <v>0.8378878973040726</v>
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
@@ -5459,7 +5459,7 @@
         </is>
       </c>
       <c r="C26" s="36" t="n">
-        <v>0.8114105175622475</v>
+        <v>0.8114105175622477</v>
       </c>
       <c r="D26" s="22" t="inlineStr">
         <is>
@@ -5484,7 +5484,7 @@
         </is>
       </c>
       <c r="C27" s="35" t="n">
-        <v>0.7802907386399156</v>
+        <v>0.7802907386399155</v>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
@@ -5509,7 +5509,7 @@
         </is>
       </c>
       <c r="C28" s="36" t="n">
-        <v>0.752725532749333</v>
+        <v>0.7527255327493332</v>
       </c>
       <c r="D28" s="22" t="inlineStr">
         <is>
@@ -5534,7 +5534,7 @@
         </is>
       </c>
       <c r="C29" s="35" t="n">
-        <v>0.7403645624314057</v>
+        <v>0.7403645624314058</v>
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
@@ -5559,7 +5559,7 @@
         </is>
       </c>
       <c r="C30" s="36" t="n">
-        <v>0.7359354048313768</v>
+        <v>0.7359354048313766</v>
       </c>
       <c r="D30" s="22" t="inlineStr">
         <is>
@@ -5609,7 +5609,7 @@
         </is>
       </c>
       <c r="C32" s="36" t="n">
-        <v>0.7315398350882374</v>
+        <v>0.7315398350882377</v>
       </c>
       <c r="D32" s="22" t="inlineStr">
         <is>
@@ -5634,7 +5634,7 @@
         </is>
       </c>
       <c r="C33" s="35" t="n">
-        <v>0.7186127346808739</v>
+        <v>0.7186127346808743</v>
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
@@ -5730,13 +5730,13 @@
         <v>0.213020599450317</v>
       </c>
       <c r="D3" s="35" t="n">
-        <v>2.153964607978918</v>
+        <v>2.15396460797892</v>
       </c>
       <c r="E3" s="35" t="n">
-        <v>3.246662089897636</v>
+        <v>3.246662089897637</v>
       </c>
       <c r="F3" s="35" t="n">
-        <v>0.007778258572596224</v>
+        <v>0.007778258572596125</v>
       </c>
     </row>
     <row r="4">
@@ -5749,16 +5749,16 @@
         <v>0.6313817072904651</v>
       </c>
       <c r="C4" s="36" t="n">
-        <v>0.3361745051400978</v>
+        <v>0.3361745051400977</v>
       </c>
       <c r="D4" s="36" t="n">
         <v>2.146979458188246</v>
       </c>
       <c r="E4" s="36" t="n">
-        <v>0.3615911096991376</v>
+        <v>0.3615911096991364</v>
       </c>
       <c r="F4" s="36" t="n">
-        <v>-0.02618469033086923</v>
+        <v>-0.02618469033086921</v>
       </c>
     </row>
     <row r="5">
@@ -5768,19 +5768,19 @@
         </is>
       </c>
       <c r="B5" s="35" t="n">
-        <v>0.341608936545249</v>
+        <v>0.3416089365452504</v>
       </c>
       <c r="C5" s="35" t="n">
-        <v>0.4623755448547909</v>
+        <v>0.4623755448547925</v>
       </c>
       <c r="D5" s="35" t="n">
-        <v>2.731154020882956</v>
+        <v>2.731154020882983</v>
       </c>
       <c r="E5" s="35" t="n">
-        <v>0.8990702173393044</v>
+        <v>0.8990702173391955</v>
       </c>
       <c r="F5" s="35" t="n">
-        <v>0.02485752388917012</v>
+        <v>0.02485752388917111</v>
       </c>
     </row>
     <row r="6">
@@ -5790,19 +5790,19 @@
         </is>
       </c>
       <c r="B6" s="36" t="n">
-        <v>0.2828260983026297</v>
+        <v>0.2828260983022897</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>0.3733154718690183</v>
+        <v>0.3733154718682769</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>1.232021384742424</v>
+        <v>1.232021384734952</v>
       </c>
       <c r="E6" s="36" t="n">
-        <v>3.096735624978685</v>
+        <v>3.096735624995443</v>
       </c>
       <c r="F6" s="36" t="n">
-        <v>0.01283247003358824</v>
+        <v>0.0128324700331053</v>
       </c>
     </row>
     <row r="7">
@@ -5815,16 +5815,16 @@
         <v>0.2024684798488106</v>
       </c>
       <c r="C7" s="35" t="n">
-        <v>0.3213380633688087</v>
+        <v>0.3213380633688086</v>
       </c>
       <c r="D7" s="35" t="n">
-        <v>0.8611775407280976</v>
+        <v>0.8611775407281035</v>
       </c>
       <c r="E7" s="35" t="n">
-        <v>3.585820188471191</v>
+        <v>3.585820188471193</v>
       </c>
       <c r="F7" s="35" t="n">
-        <v>0.02721739711619323</v>
+        <v>0.02721739711619306</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: restore Tier 2 private assets and GFC stress test metrics
</commit_message>
<xml_diff>
--- a/analytics_report.xlsx
+++ b/analytics_report.xlsx
@@ -27,7 +27,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -88,6 +88,11 @@
     <font>
       <name val="Arial"/>
       <color rgb="00B7770D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001E7B45"/>
       <sz val="10"/>
     </font>
     <font>
@@ -318,16 +323,16 @@
     <xf numFmtId="164" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -339,25 +344,25 @@
     <xf numFmtId="165" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="15" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="15" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="15" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="15" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1019,25 +1024,25 @@
         </is>
       </c>
       <c r="B8" s="9" t="n">
-        <v>0.07378527590086548</v>
+        <v>0.07378527980854011</v>
       </c>
       <c r="C8" s="9" t="n">
-        <v>0.1102367794102579</v>
+        <v>0.1102367739317823</v>
       </c>
       <c r="D8" s="10" t="n">
-        <v>0.4865415659165658</v>
+        <v>0.4865416255444058</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>0.6069203385934979</v>
+        <v>0.6069202987975629</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>-0.1958991860781159</v>
+        <v>-0.1958990938318969</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>0.376649221357373</v>
+        <v>0.3766494186637537</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>0.02666080197108656</v>
+        <v>0.02666080497247821</v>
       </c>
     </row>
     <row r="9">
@@ -1047,22 +1052,22 @@
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>0.07998380339703903</v>
+        <v>0.07998380778198988</v>
       </c>
       <c r="C9" s="12" t="n">
-        <v>0.1069805129364676</v>
+        <v>0.1069805109235594</v>
       </c>
       <c r="D9" s="13" t="n">
-        <v>0.5592916048885708</v>
+        <v>0.5592916564003224</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>0.7881504656053266</v>
+        <v>0.7881504192348465</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>-0.241238590731507</v>
+        <v>-0.2412384953320925</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.3315547614272841</v>
+        <v>0.3315549107197132</v>
       </c>
       <c r="H9" s="12" t="n">
         <v>0</v>
@@ -1075,25 +1080,25 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>0.06222171082584271</v>
+        <v>0.07663819523679472</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>0.0973601500872822</v>
+        <v>0.08321356109257802</v>
       </c>
       <c r="D10" s="10" t="n">
-        <v>0.432119405764338</v>
+        <v>0.6788279923382992</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>0.5783968614119489</v>
+        <v>0.9323885697872637</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>-0.27765624040269</v>
+        <v>-0.2151224545325302</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>0.2240962088069816</v>
+        <v>0.3562538155458137</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>0.05645299427673103</v>
+        <v>0.06996092679099582</v>
       </c>
     </row>
     <row r="11">
@@ -1103,25 +1108,25 @@
         </is>
       </c>
       <c r="B11" s="12" t="n">
-        <v>0.05336149921976885</v>
+        <v>0.05975307784699102</v>
       </c>
       <c r="C11" s="12" t="n">
-        <v>0.07659729222579761</v>
+        <v>0.0638817408097252</v>
       </c>
       <c r="D11" s="13" t="n">
-        <v>0.4335792771481806</v>
+        <v>0.6199357863454225</v>
       </c>
       <c r="E11" s="13" t="n">
-        <v>0.5934387331649268</v>
+        <v>0.8940035467859482</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>-0.2057596347263281</v>
+        <v>-0.1476443968503109</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.2593390063641134</v>
+        <v>0.4047094175038122</v>
       </c>
       <c r="H11" s="12" t="n">
-        <v>0.05369797654498694</v>
+        <v>0.04860572903543283</v>
       </c>
     </row>
     <row r="12">
@@ -1131,25 +1136,25 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>0.03786650154700966</v>
+        <v>0.04841833252063688</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>0.06181265212606881</v>
+        <v>0.05539011011202866</v>
       </c>
       <c r="D12" s="10" t="n">
-        <v>0.2866080052005819</v>
+        <v>0.5103407781364672</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>0.3782437630813464</v>
+        <v>0.6499482531048663</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>-0.1798794517404291</v>
+        <v>-0.1602422571166676</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>0.2105104345195139</v>
+        <v>0.3021570801101792</v>
       </c>
       <c r="H12" s="9" t="n">
-        <v>0.07404845446758664</v>
+        <v>0.067186603360334</v>
       </c>
     </row>
     <row r="13" ht="8" customHeight="1"/>
@@ -1529,25 +1534,25 @@
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>0.07378527590086548</v>
+        <v>0.07378527980854011</v>
       </c>
       <c r="C3" s="9" t="n">
-        <v>0.1102367794102579</v>
+        <v>0.1102367739317823</v>
       </c>
       <c r="D3" s="24" t="n">
-        <v>0.4865415659165658</v>
+        <v>0.4865416255444058</v>
       </c>
       <c r="E3" s="10" t="n">
-        <v>0.6069203385934979</v>
+        <v>0.6069202987975629</v>
       </c>
       <c r="F3" s="25" t="n">
-        <v>-0.1958991860781159</v>
+        <v>-0.1958990938318969</v>
       </c>
       <c r="G3" s="10" t="n">
-        <v>0.376649221357373</v>
+        <v>0.3766494186637537</v>
       </c>
       <c r="H3" s="9" t="n">
-        <v>0.02666080197108656</v>
+        <v>0.02666080497247821</v>
       </c>
     </row>
     <row r="4">
@@ -1557,22 +1562,22 @@
         </is>
       </c>
       <c r="B4" s="12" t="n">
-        <v>0.07998380339703903</v>
+        <v>0.07998380778198988</v>
       </c>
       <c r="C4" s="12" t="n">
-        <v>0.1069805129364676</v>
+        <v>0.1069805109235594</v>
       </c>
       <c r="D4" s="26" t="n">
-        <v>0.5592916048885708</v>
+        <v>0.5592916564003224</v>
       </c>
       <c r="E4" s="13" t="n">
-        <v>0.7881504656053266</v>
+        <v>0.7881504192348465</v>
       </c>
       <c r="F4" s="27" t="n">
-        <v>-0.241238590731507</v>
+        <v>-0.2412384953320925</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.3315547614272841</v>
+        <v>0.3315549107197132</v>
       </c>
       <c r="H4" s="12" t="n">
         <v>0</v>
@@ -1585,25 +1590,25 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.06222171082584271</v>
+        <v>0.07663819523679472</v>
       </c>
       <c r="C5" s="9" t="n">
-        <v>0.0973601500872822</v>
+        <v>0.08321356109257802</v>
       </c>
       <c r="D5" s="24" t="n">
-        <v>0.432119405764338</v>
+        <v>0.6788279923382992</v>
       </c>
       <c r="E5" s="10" t="n">
-        <v>0.5783968614119489</v>
-      </c>
-      <c r="F5" s="14" t="n">
-        <v>-0.27765624040269</v>
+        <v>0.9323885697872637</v>
+      </c>
+      <c r="F5" s="25" t="n">
+        <v>-0.2151224545325302</v>
       </c>
       <c r="G5" s="10" t="n">
-        <v>0.2240962088069816</v>
+        <v>0.3562538155458137</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>0.05645299427673103</v>
+        <v>0.06996092679099582</v>
       </c>
     </row>
     <row r="6">
@@ -1613,25 +1618,25 @@
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v>0.05336149921976885</v>
+        <v>0.05975307784699102</v>
       </c>
       <c r="C6" s="12" t="n">
-        <v>0.07659729222579761</v>
+        <v>0.0638817408097252</v>
       </c>
       <c r="D6" s="26" t="n">
-        <v>0.4335792771481806</v>
+        <v>0.6199357863454225</v>
       </c>
       <c r="E6" s="13" t="n">
-        <v>0.5934387331649268</v>
-      </c>
-      <c r="F6" s="27" t="n">
-        <v>-0.2057596347263281</v>
+        <v>0.8940035467859482</v>
+      </c>
+      <c r="F6" s="28" t="n">
+        <v>-0.1476443968503109</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.2593390063641134</v>
+        <v>0.4047094175038122</v>
       </c>
       <c r="H6" s="12" t="n">
-        <v>0.05369797654498694</v>
+        <v>0.04860572903543283</v>
       </c>
     </row>
     <row r="7">
@@ -1641,25 +1646,25 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>0.03786650154700966</v>
+        <v>0.04841833252063688</v>
       </c>
       <c r="C7" s="9" t="n">
-        <v>0.06181265212606881</v>
-      </c>
-      <c r="D7" s="28" t="n">
-        <v>0.2866080052005819</v>
+        <v>0.05539011011202866</v>
+      </c>
+      <c r="D7" s="24" t="n">
+        <v>0.5103407781364672</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>0.3782437630813464</v>
+        <v>0.6499482531048663</v>
       </c>
       <c r="F7" s="25" t="n">
-        <v>-0.1798794517404291</v>
+        <v>-0.1602422571166676</v>
       </c>
       <c r="G7" s="10" t="n">
-        <v>0.2105104345195139</v>
+        <v>0.3021570801101792</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>0.07404845446758664</v>
+        <v>0.067186603360334</v>
       </c>
     </row>
     <row r="29">
@@ -1701,7 +1706,7 @@
         </is>
       </c>
       <c r="B31" s="9" t="n">
-        <v>0.02666080197108656</v>
+        <v>0.02666080497247821</v>
       </c>
       <c r="C31" s="29" t="n">
         <v>0.1111111111111111</v>
@@ -1737,10 +1742,10 @@
         </is>
       </c>
       <c r="B33" s="9" t="n">
-        <v>0.05645299427673103</v>
+        <v>0.06996092679099582</v>
       </c>
       <c r="C33" s="25" t="n">
-        <v>0.364425723493131</v>
+        <v>0.3644257856776272</v>
       </c>
       <c r="D33" s="30" t="inlineStr">
         <is>
@@ -1755,10 +1760,10 @@
         </is>
       </c>
       <c r="B34" s="12" t="n">
-        <v>0.05369797654498694</v>
+        <v>0.04860572903543283</v>
       </c>
       <c r="C34" s="27" t="n">
-        <v>0.2945578217774981</v>
+        <v>0.2945580612696407</v>
       </c>
       <c r="D34" s="32" t="inlineStr">
         <is>
@@ -1773,10 +1778,10 @@
         </is>
       </c>
       <c r="B35" s="9" t="n">
-        <v>0.07404845446758664</v>
+        <v>0.067186603360334</v>
       </c>
       <c r="C35" s="16" t="n">
-        <v>0.5717326055122662</v>
+        <v>0.571732280411839</v>
       </c>
       <c r="D35" s="30" t="inlineStr">
         <is>
@@ -1943,25 +1948,25 @@
         </is>
       </c>
       <c r="B4" s="34" t="n">
-        <v>0.971354889535758</v>
+        <v>0.9713543546890465</v>
       </c>
       <c r="C4" s="34" t="n">
-        <v>-0.0279185738583745</v>
+        <v>-0.02791868690570089</v>
       </c>
       <c r="D4" s="34" t="n">
-        <v>1.307574570963585</v>
+        <v>1.307584296732336</v>
       </c>
       <c r="E4" s="34" t="n">
-        <v>2.069750684644512</v>
+        <v>2.069745671519761</v>
       </c>
       <c r="F4" s="34" t="n">
-        <v>0.03673471269025674</v>
+        <v>0.03673461445983179</v>
       </c>
       <c r="G4" s="12" t="n">
-        <v>0.02838076840528056</v>
+        <v>0.02838075985627555</v>
       </c>
       <c r="H4" s="12" t="n">
-        <v>0.9123631766041419</v>
+        <v>0.9123633301070473</v>
       </c>
       <c r="I4" s="22" t="inlineStr">
         <is>
@@ -1976,25 +1981,25 @@
         </is>
       </c>
       <c r="B5" s="33" t="n">
-        <v>1.184029620083211</v>
+        <v>1.184030233295581</v>
       </c>
       <c r="C5" s="33" t="n">
-        <v>-0.1590181004859705</v>
+        <v>-0.1590173667035335</v>
       </c>
       <c r="D5" s="33" t="n">
-        <v>0.6769277744832372</v>
+        <v>0.6769344744648144</v>
       </c>
       <c r="E5" s="33" t="n">
-        <v>-2.052810693745579</v>
+        <v>-2.052829348795206</v>
       </c>
       <c r="F5" s="33" t="n">
-        <v>-0.01476509282000907</v>
+        <v>-0.01476554280325399</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>0.02543144571233723</v>
+        <v>0.02543145418845582</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>0.8712835998068817</v>
+        <v>0.8712834190739561</v>
       </c>
       <c r="I5" s="19" t="inlineStr">
         <is>
@@ -2009,25 +2014,25 @@
         </is>
       </c>
       <c r="B6" s="34" t="n">
-        <v>0.7532195145960868</v>
+        <v>0.7532192116329343</v>
       </c>
       <c r="C6" s="34" t="n">
-        <v>0.239200635449679</v>
+        <v>0.2392006264404306</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>5.685577809098848</v>
+        <v>5.685559710072019</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>6.296292096835225</v>
+        <v>6.296323430647663</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>-0.0955658312106086</v>
+        <v>-0.09556557578946366</v>
       </c>
       <c r="G6" s="12" t="n">
-        <v>0.0206718781744882</v>
+        <v>0.02067188264244709</v>
       </c>
       <c r="H6" s="12" t="n">
-        <v>0.6355403296685542</v>
+        <v>0.6355401248164949</v>
       </c>
       <c r="I6" s="22" t="inlineStr">
         <is>
@@ -2042,25 +2047,25 @@
         </is>
       </c>
       <c r="B7" s="33" t="n">
-        <v>0.02522245718052332</v>
+        <v>0.02522360442670393</v>
       </c>
       <c r="C7" s="33" t="n">
-        <v>1.139232287873908</v>
+        <v>1.13922957972593</v>
       </c>
       <c r="D7" s="33" t="n">
-        <v>-0.1657940661604688</v>
+        <v>-0.1658095440767343</v>
       </c>
       <c r="E7" s="33" t="n">
-        <v>-2.13589950876659</v>
+        <v>-2.135898143828797</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>-0.007930157885479423</v>
+        <v>-0.007930898215471631</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>0.01148282418385831</v>
+        <v>0.01148281541820169</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>0.9812438336595104</v>
+        <v>0.981243967023252</v>
       </c>
       <c r="I7" s="19" t="inlineStr">
         <is>
@@ -2075,25 +2080,25 @@
         </is>
       </c>
       <c r="B8" s="34" t="n">
-        <v>0.01944981703587667</v>
+        <v>0.01944867126558009</v>
       </c>
       <c r="C8" s="34" t="n">
-        <v>0.4459870996647048</v>
+        <v>0.4459868868234478</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>-0.1250823047768445</v>
+        <v>-0.1250762247422195</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>6.421690474074236</v>
+        <v>6.421664708875722</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>-0.005982858425101597</v>
+        <v>-0.005982567608695194</v>
       </c>
       <c r="G8" s="12" t="n">
-        <v>0.008734871552751659</v>
+        <v>0.008734870137983752</v>
       </c>
       <c r="H8" s="12" t="n">
-        <v>0.8015107862181039</v>
+        <v>0.8015088821539471</v>
       </c>
       <c r="I8" s="22" t="inlineStr">
         <is>
@@ -2108,25 +2113,25 @@
         </is>
       </c>
       <c r="B9" s="33" t="n">
-        <v>0.2750935238828958</v>
+        <v>0.2750960153447685</v>
       </c>
       <c r="C9" s="33" t="n">
-        <v>0.5137949658837728</v>
+        <v>0.5137940982593163</v>
       </c>
       <c r="D9" s="33" t="n">
-        <v>0.2430069382283973</v>
+        <v>0.2429920809566087</v>
       </c>
       <c r="E9" s="33" t="n">
-        <v>-0.1456786200674224</v>
+        <v>-0.145757769728357</v>
       </c>
       <c r="F9" s="33" t="n">
-        <v>0.011623355600392</v>
+        <v>0.01162264495667739</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>0.01057001448042171</v>
+        <v>0.01057001868840936</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>0.6374633033903678</v>
+        <v>0.6374618458308732</v>
       </c>
       <c r="I9" s="19" t="inlineStr">
         <is>
@@ -2141,25 +2146,25 @@
         </is>
       </c>
       <c r="B10" s="34" t="n">
-        <v>1.035110447452133</v>
+        <v>1.035110678337744</v>
       </c>
       <c r="C10" s="34" t="n">
-        <v>0.3934959490536423</v>
+        <v>0.3934964445308032</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>9.352440086495633</v>
+        <v>9.352425086801601</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>-8.299662990213015</v>
+        <v>-8.299633141497763</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>-0.1362108916081567</v>
+        <v>-0.1362115190006306</v>
       </c>
       <c r="G10" s="12" t="n">
-        <v>0.0240698586185005</v>
+        <v>0.02406984915621184</v>
       </c>
       <c r="H10" s="12" t="n">
-        <v>0.6337084793755835</v>
+        <v>0.6337083217606877</v>
       </c>
       <c r="I10" s="22" t="inlineStr">
         <is>
@@ -2174,25 +2179,25 @@
         </is>
       </c>
       <c r="B11" s="33" t="n">
-        <v>0.1086076548864854</v>
+        <v>0.1086074255047768</v>
       </c>
       <c r="C11" s="33" t="n">
-        <v>-0.322256513988238</v>
+        <v>-0.3222563603329497</v>
       </c>
       <c r="D11" s="33" t="n">
-        <v>4.246990685914242</v>
+        <v>4.246994947560707</v>
       </c>
       <c r="E11" s="33" t="n">
-        <v>15.42135885368741</v>
+        <v>15.42136218884538</v>
       </c>
       <c r="F11" s="33" t="n">
-        <v>0.0372673088981893</v>
+        <v>0.03726719926776158</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>0.004127872859151399</v>
+        <v>0.004127876963690224</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>0.4445765852026022</v>
+        <v>0.4445765743655131</v>
       </c>
       <c r="I11" s="19" t="inlineStr">
         <is>
@@ -2245,13 +2250,13 @@
         </is>
       </c>
       <c r="B15" s="33" t="n">
-        <v>0.1086076548864854</v>
+        <v>0.1086074255047768</v>
       </c>
       <c r="C15" s="33" t="n">
-        <v>0.815131539955253</v>
+        <v>0.8151360605982694</v>
       </c>
       <c r="D15" s="33" t="n">
-        <v>0.7065238850687676</v>
+        <v>0.7065286350934925</v>
       </c>
       <c r="E15" s="19" t="inlineStr">
         <is>
@@ -2266,13 +2271,13 @@
         </is>
       </c>
       <c r="B16" s="34" t="n">
-        <v>0.01944981703587667</v>
+        <v>0.01944867126558009</v>
       </c>
       <c r="C16" s="34" t="n">
-        <v>0.1007609043221211</v>
+        <v>0.1007618020644612</v>
       </c>
       <c r="D16" s="34" t="n">
-        <v>0.08131108728624448</v>
+        <v>0.08131313079888108</v>
       </c>
       <c r="E16" s="22" t="inlineStr">
         <is>
@@ -2287,13 +2292,13 @@
         </is>
       </c>
       <c r="B17" s="33" t="n">
-        <v>0.02522245718052332</v>
+        <v>0.02522360442670393</v>
       </c>
       <c r="C17" s="33" t="n">
-        <v>0.07165142618821491</v>
+        <v>0.07165818859001716</v>
       </c>
       <c r="D17" s="33" t="n">
-        <v>0.04642896900769159</v>
+        <v>0.04643458416331323</v>
       </c>
       <c r="E17" s="19" t="inlineStr">
         <is>
@@ -2329,13 +2334,13 @@
         </is>
       </c>
       <c r="B19" s="33" t="n">
-        <v>1.035110447452133</v>
+        <v>1.035110678337744</v>
       </c>
       <c r="C19" s="33" t="n">
-        <v>1.031109852175071</v>
+        <v>1.031110217491761</v>
       </c>
       <c r="D19" s="33" t="n">
-        <v>-0.004000595277062535</v>
+        <v>-0.004000460845982268</v>
       </c>
       <c r="E19" s="19" t="inlineStr">
         <is>
@@ -2350,13 +2355,13 @@
         </is>
       </c>
       <c r="B20" s="34" t="n">
-        <v>0.7532195145960868</v>
+        <v>0.7532192116329343</v>
       </c>
       <c r="C20" s="34" t="n">
-        <v>0.7449314332372436</v>
+        <v>0.7449323836182584</v>
       </c>
       <c r="D20" s="34" t="n">
-        <v>-0.00828808135884318</v>
+        <v>-0.00828682801467584</v>
       </c>
       <c r="E20" s="22" t="inlineStr">
         <is>
@@ -2371,13 +2376,13 @@
         </is>
       </c>
       <c r="B21" s="33" t="n">
-        <v>0.2750935238828958</v>
+        <v>0.2750960153447685</v>
       </c>
       <c r="C21" s="33" t="n">
-        <v>0.2323422009434037</v>
+        <v>0.2323438705888303</v>
       </c>
       <c r="D21" s="33" t="n">
-        <v>-0.04275132293949202</v>
+        <v>-0.04275214475593819</v>
       </c>
       <c r="E21" s="19" t="inlineStr">
         <is>
@@ -2392,13 +2397,13 @@
         </is>
       </c>
       <c r="B22" s="34" t="n">
-        <v>0.971354889535758</v>
+        <v>0.9713543546890465</v>
       </c>
       <c r="C22" s="34" t="n">
-        <v>0.8150671969591841</v>
+        <v>0.8150714885287655</v>
       </c>
       <c r="D22" s="34" t="n">
-        <v>-0.1562876925765739</v>
+        <v>-0.156282866160281</v>
       </c>
       <c r="E22" s="22" t="inlineStr">
         <is>
@@ -2413,13 +2418,13 @@
         </is>
       </c>
       <c r="B23" s="33" t="n">
-        <v>1.184029620083211</v>
+        <v>1.184030233295581</v>
       </c>
       <c r="C23" s="33" t="n">
-        <v>0.9628307198768065</v>
+        <v>0.9628342395707845</v>
       </c>
       <c r="D23" s="33" t="n">
-        <v>-0.2211989002064045</v>
+        <v>-0.2211959937247967</v>
       </c>
       <c r="E23" s="19" t="inlineStr">
         <is>
@@ -2500,16 +2505,16 @@
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v/>
+        <v>-0.3134746014276183</v>
       </c>
       <c r="C3" s="9" t="n">
-        <v>-0.04948767209921656</v>
+        <v>-0.04948761433926584</v>
       </c>
       <c r="D3" s="9" t="n">
-        <v>-0.1548212961496473</v>
+        <v>-0.1548212823410495</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>0.2143160465292979</v>
+        <v>0.5954501587549845</v>
       </c>
     </row>
     <row r="4">
@@ -2519,16 +2524,16 @@
         </is>
       </c>
       <c r="B4" s="12" t="n">
-        <v/>
+        <v>-0.2495977639371679</v>
       </c>
       <c r="C4" s="12" t="n">
-        <v>-0.003713680052704005</v>
+        <v>-0.003713611804167738</v>
       </c>
       <c r="D4" s="12" t="n">
-        <v>-0.2018217653802958</v>
+        <v>-0.2018217565810658</v>
       </c>
       <c r="E4" s="12" t="n">
-        <v>0.2151526914615902</v>
+        <v>0.6016793798524094</v>
       </c>
     </row>
     <row r="5">
@@ -2538,16 +2543,16 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v/>
+        <v>-0.1954153004416594</v>
       </c>
       <c r="C5" s="9" t="n">
-        <v>0.0581581967231346</v>
+        <v>0.0468524310147842</v>
       </c>
       <c r="D5" s="9" t="n">
-        <v>-0.250885602361373</v>
+        <v>-0.2346489343424729</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>0.1374424892823327</v>
+        <v>0.4831002441572396</v>
       </c>
     </row>
     <row r="6">
@@ -2557,16 +2562,16 @@
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v/>
+        <v>-0.1730524664274122</v>
       </c>
       <c r="C6" s="12" t="n">
-        <v>0.0378862523994854</v>
+        <v>0.02429344316360349</v>
       </c>
       <c r="D6" s="12" t="n">
-        <v>-0.1806387327290133</v>
+        <v>-0.1674660311134522</v>
       </c>
       <c r="E6" s="12" t="n">
-        <v>0.1274251187978204</v>
+        <v>0.3559225224980567</v>
       </c>
     </row>
     <row r="7">
@@ -2576,16 +2581,16 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v/>
+        <v>-0.06759692357441749</v>
       </c>
       <c r="C7" s="9" t="n">
-        <v>0.05676145018542478</v>
+        <v>0.05076908147634351</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>-0.1583714697754696</v>
+        <v>-0.1475039470866329</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>0.09376517010863307</v>
+        <v>0.2180544335778652</v>
       </c>
     </row>
   </sheetData>
@@ -2680,13 +2685,13 @@
         <v>0.1111111111111111</v>
       </c>
       <c r="C4" s="33" t="n">
-        <v>0.07664168083031668</v>
+        <v>0.07664168351224593</v>
       </c>
       <c r="D4" s="33" t="n">
-        <v>0.008515742314479631</v>
+        <v>0.008515742612471769</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>0.1437031813131897</v>
+        <v>0.1437032210168355</v>
       </c>
       <c r="F4" s="9" t="n">
         <v>0.9718498340506939</v>
@@ -2702,16 +2707,16 @@
         <v>0.1111111111111111</v>
       </c>
       <c r="C5" s="34" t="n">
-        <v>0.08782259806744334</v>
+        <v>0.08782255892101108</v>
       </c>
       <c r="D5" s="34" t="n">
-        <v>0.009758066451938149</v>
+        <v>0.009758062102334564</v>
       </c>
       <c r="E5" s="12" t="n">
-        <v>0.1646674054738244</v>
+        <v>0.1646673718078441</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>0.9005691996051071</v>
+        <v>0.9005692931844215</v>
       </c>
     </row>
     <row r="6">
@@ -2724,16 +2729,16 @@
         <v>0.1111111111111111</v>
       </c>
       <c r="C6" s="33" t="n">
-        <v>0.09343994377207028</v>
+        <v>0.09343996140347188</v>
       </c>
       <c r="D6" s="33" t="n">
-        <v>0.01038221597467448</v>
+        <v>0.0103822179337191</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>0.17519993085095</v>
+        <v>0.1752000061849139</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>0.8647854557196933</v>
+        <v>0.8647853697421607</v>
       </c>
     </row>
     <row r="7">
@@ -2746,16 +2751,16 @@
         <v>0.1111111111111111</v>
       </c>
       <c r="C7" s="34" t="n">
-        <v>0.09133108763780659</v>
+        <v>0.09133107047002956</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>0.01014789862642295</v>
+        <v>0.01014789671889217</v>
       </c>
       <c r="E7" s="12" t="n">
-        <v>0.1712458247804364</v>
+        <v>0.1712458339118004</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>0.6547261440685357</v>
+        <v>0.654725765269208</v>
       </c>
     </row>
     <row r="8">
@@ -2768,16 +2773,16 @@
         <v>0.1111111111111111</v>
       </c>
       <c r="C8" s="33" t="n">
-        <v>-0.01422440861340878</v>
+        <v>-0.01422437146584231</v>
       </c>
       <c r="D8" s="33" t="n">
-        <v>-0.001580489845934309</v>
+        <v>-0.001580485718426923</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>-0.0266707716728077</v>
+        <v>-0.0266707084566442</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>0.9800393733856876</v>
+        <v>0.9800394596124378</v>
       </c>
     </row>
     <row r="9">
@@ -2790,16 +2795,16 @@
         <v>0.1111111111111111</v>
       </c>
       <c r="C9" s="34" t="n">
-        <v>0.01048969378157021</v>
+        <v>0.01048960388641192</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>0.001165521531285578</v>
+        <v>0.001165511542934658</v>
       </c>
       <c r="E9" s="12" t="n">
-        <v>0.01966817991309695</v>
+        <v>0.01966801610545594</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>0.8261569337194916</v>
+        <v>0.8261549596926778</v>
       </c>
     </row>
     <row r="10">
@@ -2812,16 +2817,16 @@
         <v>0.1111111111111111</v>
       </c>
       <c r="C10" s="33" t="n">
-        <v>0.01878514918907328</v>
+        <v>0.01878512858404903</v>
       </c>
       <c r="D10" s="33" t="n">
-        <v>0.00208723879878592</v>
+        <v>0.002087236509338781</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>0.03522216202289886</v>
+        <v>0.03522213188743362</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>0.6542475904087065</v>
+        <v>0.654246587683997</v>
       </c>
     </row>
     <row r="11">
@@ -2834,16 +2839,16 @@
         <v>0.1111111111111111</v>
       </c>
       <c r="C11" s="34" t="n">
-        <v>0.09287907293206586</v>
+        <v>0.09287908065450565</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>0.01031989699245176</v>
+        <v>0.01031989785050063</v>
       </c>
       <c r="E11" s="12" t="n">
-        <v>0.1741482978081821</v>
+        <v>0.1741483543090792</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>0.6432518675233434</v>
+        <v>0.6432517319898794</v>
       </c>
     </row>
     <row r="12">
@@ -2856,16 +2861,16 @@
         <v>0.1111111111111111</v>
       </c>
       <c r="C12" s="33" t="n">
-        <v>0.07616840530007137</v>
+        <v>0.07616837823989694</v>
       </c>
       <c r="D12" s="33" t="n">
-        <v>0.008463156144452373</v>
+        <v>0.008463153137766327</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>0.1428157895102292</v>
+        <v>0.1428157732332814</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>0.4913807456936256</v>
+        <v>0.4913808005382763</v>
       </c>
     </row>
     <row r="14">
@@ -2922,13 +2927,13 @@
         <v>0.12</v>
       </c>
       <c r="C16" s="33" t="n">
-        <v>0.07480404287209469</v>
+        <v>0.07480404058153603</v>
       </c>
       <c r="D16" s="33" t="n">
-        <v>0.008976485144651363</v>
+        <v>0.008976484869784323</v>
       </c>
       <c r="E16" s="9" t="n">
-        <v>0.1582967093658338</v>
+        <v>0.158296737888037</v>
       </c>
       <c r="F16" s="9" t="n">
         <v>0.9718498340506939</v>
@@ -2944,16 +2949,16 @@
         <v>0.12</v>
       </c>
       <c r="C17" s="34" t="n">
-        <v>0.08443784634742667</v>
+        <v>0.08443779803315991</v>
       </c>
       <c r="D17" s="34" t="n">
-        <v>0.0101325415616912</v>
+        <v>0.01013253576397919</v>
       </c>
       <c r="E17" s="12" t="n">
-        <v>0.1786832998530584</v>
+        <v>0.178683235279637</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>0.9005691996051071</v>
+        <v>0.9005692931844215</v>
       </c>
     </row>
     <row r="18">
@@ -2966,16 +2971,16 @@
         <v>0.12</v>
       </c>
       <c r="C18" s="33" t="n">
-        <v>0.091633228354804</v>
+        <v>0.09163325284247642</v>
       </c>
       <c r="D18" s="33" t="n">
-        <v>0.01099598740257648</v>
+        <v>0.01099599034109717</v>
       </c>
       <c r="E18" s="9" t="n">
-        <v>0.1939098203814409</v>
+        <v>0.1939099130777978</v>
       </c>
       <c r="F18" s="9" t="n">
-        <v>0.8647854557196933</v>
+        <v>0.8647853697421607</v>
       </c>
     </row>
     <row r="19">
@@ -2988,16 +2993,16 @@
         <v>0.12</v>
       </c>
       <c r="C19" s="34" t="n">
-        <v>0.08827070665032773</v>
+        <v>0.08827067970023333</v>
       </c>
       <c r="D19" s="34" t="n">
-        <v>0.01059248479803933</v>
+        <v>0.010592481564028</v>
       </c>
       <c r="E19" s="12" t="n">
-        <v>0.18679421405118</v>
+        <v>0.1867941963974024</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>0.6547261440685357</v>
+        <v>0.654725765269208</v>
       </c>
     </row>
     <row r="20">
@@ -3010,16 +3015,16 @@
         <v>0.1333333333333333</v>
       </c>
       <c r="C20" s="33" t="n">
-        <v>-0.001968814218307936</v>
+        <v>-0.001968768015688312</v>
       </c>
       <c r="D20" s="33" t="n">
-        <v>-0.0002625085624410581</v>
+        <v>-0.0002625024020917749</v>
       </c>
       <c r="E20" s="9" t="n">
-        <v>-0.004629233040009552</v>
+        <v>-0.004629125380556697</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>0.9800393733856876</v>
+        <v>0.9800394596124378</v>
       </c>
     </row>
     <row r="21">
@@ -3032,16 +3037,16 @@
         <v>0.1333333333333333</v>
       </c>
       <c r="C21" s="34" t="n">
-        <v>0.01159941221845756</v>
+        <v>0.01159932567640918</v>
       </c>
       <c r="D21" s="34" t="n">
-        <v>0.001546588295794342</v>
+        <v>0.001546576756854557</v>
       </c>
       <c r="E21" s="12" t="n">
-        <v>0.02727346327909126</v>
+        <v>0.02727326554380059</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>0.8261569337194916</v>
+        <v>0.8261549596926778</v>
       </c>
     </row>
     <row r="22">
@@ -3054,16 +3059,16 @@
         <v>0.1333333333333333</v>
       </c>
       <c r="C22" s="33" t="n">
-        <v>0.02377789275031428</v>
+        <v>0.02377789461211848</v>
       </c>
       <c r="D22" s="33" t="n">
-        <v>0.003170385700041904</v>
+        <v>0.003170385948282464</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>0.05590847816822411</v>
+        <v>0.05590849433150584</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>0.6542475904087065</v>
+        <v>0.654246587683997</v>
       </c>
     </row>
     <row r="23">
@@ -3076,16 +3081,16 @@
         <v>0.12</v>
       </c>
       <c r="C23" s="34" t="n">
-        <v>0.09628952361557561</v>
+        <v>0.09628951981970114</v>
       </c>
       <c r="D23" s="34" t="n">
-        <v>0.01155474283386907</v>
+        <v>0.01155474237836414</v>
       </c>
       <c r="E23" s="12" t="n">
-        <v>0.203763247941181</v>
+        <v>0.2037632828623759</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.6432518675233434</v>
+        <v>0.6432517319898794</v>
       </c>
     </row>
     <row r="24">
@@ -3098,7 +3103,7 @@
         <v>0</v>
       </c>
       <c r="C24" s="33" t="n">
-        <v>0.04900614811888308</v>
+        <v>0.04900610376782925</v>
       </c>
       <c r="D24" s="33" t="n">
         <v>0</v>
@@ -3107,7 +3112,7 @@
         <v>0</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>0.4913807456936256</v>
+        <v>0.4913808005382763</v>
       </c>
     </row>
     <row r="26">
@@ -3161,16 +3166,16 @@
         </is>
       </c>
       <c r="B28" s="9" t="n">
-        <v>0.1113000326304729</v>
+        <v>0.1112995622680132</v>
       </c>
       <c r="C28" s="33" t="n">
-        <v>0.05525967850759534</v>
+        <v>0.05525968237192978</v>
       </c>
       <c r="D28" s="33" t="n">
-        <v>0.006150404021044805</v>
+        <v>0.006150378459065228</v>
       </c>
       <c r="E28" s="9" t="n">
-        <v>0.1232608271314797</v>
+        <v>0.123260483719362</v>
       </c>
       <c r="F28" s="9" t="n">
         <v>0.9718498340506939</v>
@@ -3183,19 +3188,19 @@
         </is>
       </c>
       <c r="B29" s="12" t="n">
-        <v>1.182884879237745e-07</v>
+        <v>1.182944781530638e-07</v>
       </c>
       <c r="C29" s="34" t="n">
-        <v>0.05849008269077163</v>
+        <v>0.05849004051353848</v>
       </c>
       <c r="D29" s="34" t="n">
-        <v>6.918703440027913e-09</v>
+        <v>6.919048819700591e-09</v>
       </c>
       <c r="E29" s="12" t="n">
-        <v>1.386583882582699e-07</v>
+        <v>1.386655000290496e-07</v>
       </c>
       <c r="F29" s="12" t="n">
-        <v>0.9005691996051071</v>
+        <v>0.9005692931844215</v>
       </c>
     </row>
     <row r="30">
@@ -3205,19 +3210,19 @@
         </is>
       </c>
       <c r="B30" s="9" t="n">
-        <v>3.383969452262664e-08</v>
+        <v>3.383947803280196e-08</v>
       </c>
       <c r="C30" s="33" t="n">
-        <v>0.0626857816860128</v>
+        <v>0.06268585950187984</v>
       </c>
       <c r="D30" s="33" t="n">
-        <v>2.121267703166737e-09</v>
+        <v>2.121256765581173e-09</v>
       </c>
       <c r="E30" s="9" t="n">
-        <v>4.251252613079699e-08</v>
+        <v>4.251236517536906e-08</v>
       </c>
       <c r="F30" s="9" t="n">
-        <v>0.8647854557196933</v>
+        <v>0.8647853697421607</v>
       </c>
     </row>
     <row r="31">
@@ -3227,19 +3232,19 @@
         </is>
       </c>
       <c r="B31" s="12" t="n">
-        <v>0.1941851828535534</v>
+        <v>0.1941851401027252</v>
       </c>
       <c r="C31" s="34" t="n">
-        <v>0.07269128437007231</v>
+        <v>0.07269131211729911</v>
       </c>
       <c r="D31" s="34" t="n">
-        <v>0.01411557034726214</v>
+        <v>0.01411557262774865</v>
       </c>
       <c r="E31" s="12" t="n">
-        <v>0.2828914768009913</v>
+        <v>0.2828919100917447</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.6547261440685357</v>
+        <v>0.654725765269208</v>
       </c>
     </row>
     <row r="32">
@@ -3249,19 +3254,19 @@
         </is>
       </c>
       <c r="B32" s="9" t="n">
-        <v>0.3499996938711326</v>
+        <v>0.3499996939032552</v>
       </c>
       <c r="C32" s="33" t="n">
-        <v>0.03028038966751817</v>
+        <v>0.03028031615699537</v>
       </c>
       <c r="D32" s="33" t="n">
-        <v>0.01059812711392997</v>
+        <v>0.01059810138624217</v>
       </c>
       <c r="E32" s="9" t="n">
-        <v>0.2123980651738803</v>
+        <v>0.2123978405669681</v>
       </c>
       <c r="F32" s="9" t="n">
-        <v>0.9800393733856876</v>
+        <v>0.9800394596124378</v>
       </c>
     </row>
     <row r="33">
@@ -3271,19 +3276,19 @@
         </is>
       </c>
       <c r="B33" s="12" t="n">
-        <v>0.1013184647973846</v>
+        <v>0.101322928358229</v>
       </c>
       <c r="C33" s="34" t="n">
-        <v>0.01675403652588427</v>
+        <v>0.01675398763389107</v>
       </c>
       <c r="D33" s="34" t="n">
-        <v>0.001697493259961901</v>
+        <v>0.001697563088743399</v>
       </c>
       <c r="E33" s="12" t="n">
-        <v>0.03401962254139395</v>
+        <v>0.03402106859850826</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.8261569337194916</v>
+        <v>0.8261549596926778</v>
       </c>
     </row>
     <row r="34">
@@ -3293,19 +3298,19 @@
         </is>
       </c>
       <c r="B34" s="9" t="n">
-        <v>0.04962229361749572</v>
+        <v>0.04961823822884117</v>
       </c>
       <c r="C34" s="33" t="n">
-        <v>0.0312707736028073</v>
+        <v>0.03127074460076728</v>
       </c>
       <c r="D34" s="33" t="n">
-        <v>0.001551727509364738</v>
+        <v>0.001551599255194119</v>
       </c>
       <c r="E34" s="9" t="n">
-        <v>0.03109831738411177</v>
+        <v>0.03109578963420348</v>
       </c>
       <c r="F34" s="9" t="n">
-        <v>0.6542475904087065</v>
+        <v>0.654246587683997</v>
       </c>
     </row>
     <row r="35">
@@ -3315,19 +3320,19 @@
         </is>
       </c>
       <c r="B35" s="12" t="n">
-        <v>0.17363643054771</v>
+        <v>0.1736368658373325</v>
       </c>
       <c r="C35" s="34" t="n">
-        <v>0.08842281076561428</v>
+        <v>0.08842286006646781</v>
       </c>
       <c r="D35" s="34" t="n">
-        <v>0.01535342124033689</v>
+        <v>0.0153534682903145</v>
       </c>
       <c r="E35" s="12" t="n">
-        <v>0.3076993633111713</v>
+        <v>0.3077007278218259</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>0.6432518675233434</v>
+        <v>0.6432517319898794</v>
       </c>
     </row>
     <row r="36">
@@ -3337,19 +3342,19 @@
         </is>
       </c>
       <c r="B36" s="9" t="n">
-        <v>0.01993774955406831</v>
+        <v>0.01993741916764761</v>
       </c>
       <c r="C36" s="33" t="n">
-        <v>0.02160335653579116</v>
+        <v>0.02160331428831735</v>
       </c>
       <c r="D36" s="33" t="n">
-        <v>0.0004307223121378489</v>
+        <v>0.0004307143323766138</v>
       </c>
       <c r="E36" s="9" t="n">
-        <v>0.008632146486057308</v>
+        <v>0.008631998389522265</v>
       </c>
       <c r="F36" s="9" t="n">
-        <v>0.4913807456936256</v>
+        <v>0.4913808005382763</v>
       </c>
     </row>
     <row r="38">
@@ -3403,16 +3408,16 @@
         </is>
       </c>
       <c r="B40" s="9" t="n">
-        <v>0.07066834344722557</v>
+        <v>0.07066828745635954</v>
       </c>
       <c r="C40" s="33" t="n">
-        <v>0.06189973281410109</v>
+        <v>0.06189971578576542</v>
       </c>
       <c r="D40" s="33" t="n">
-        <v>0.004374351577798394</v>
+        <v>0.004374346908615427</v>
       </c>
       <c r="E40" s="9" t="n">
-        <v>0.1111060815861452</v>
+        <v>0.1111060767534358</v>
       </c>
       <c r="F40" s="9" t="n">
         <v>0.9718498340506939</v>
@@ -3425,19 +3430,19 @@
         </is>
       </c>
       <c r="B41" s="12" t="n">
-        <v>0.06358658755192337</v>
+        <v>0.06358657635061872</v>
       </c>
       <c r="C41" s="34" t="n">
-        <v>0.06879635141332556</v>
+        <v>0.06879628490735507</v>
       </c>
       <c r="D41" s="34" t="n">
-        <v>0.004374525222396313</v>
+        <v>0.004374520222900451</v>
       </c>
       <c r="E41" s="12" t="n">
-        <v>0.1111104920617369</v>
+        <v>0.1111104788437722</v>
       </c>
       <c r="F41" s="12" t="n">
-        <v>0.9005691996051071</v>
+        <v>0.9005692931844215</v>
       </c>
     </row>
     <row r="42">
@@ -3447,19 +3452,19 @@
         </is>
       </c>
       <c r="B42" s="9" t="n">
-        <v>0.06106325534172019</v>
+        <v>0.06106318561939598</v>
       </c>
       <c r="C42" s="33" t="n">
-        <v>0.0716716355372151</v>
+        <v>0.07167165933255069</v>
       </c>
       <c r="D42" s="33" t="n">
-        <v>0.004376503381567673</v>
+        <v>0.004376499837473657</v>
       </c>
       <c r="E42" s="9" t="n">
-        <v>0.1111607361974389</v>
+        <v>0.1111607599973496</v>
       </c>
       <c r="F42" s="9" t="n">
-        <v>0.8647854557196933</v>
+        <v>0.8647853697421607</v>
       </c>
     </row>
     <row r="43">
@@ -3469,19 +3474,19 @@
         </is>
       </c>
       <c r="B43" s="12" t="n">
-        <v>0.05775356931503555</v>
+        <v>0.0577535240921918</v>
       </c>
       <c r="C43" s="34" t="n">
-        <v>0.07569763672300714</v>
+        <v>0.07569760669607641</v>
       </c>
       <c r="D43" s="34" t="n">
-        <v>0.004371808709466574</v>
+        <v>0.004371803552043108</v>
       </c>
       <c r="E43" s="12" t="n">
-        <v>0.1110414941538565</v>
+        <v>0.1110414768539677</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>0.6547261440685357</v>
+        <v>0.654725765269208</v>
       </c>
     </row>
     <row r="44">
@@ -3491,19 +3496,19 @@
         </is>
       </c>
       <c r="B44" s="9" t="n">
-        <v>0.219456840240033</v>
+        <v>0.2194568708623782</v>
       </c>
       <c r="C44" s="33" t="n">
-        <v>0.01993219484577339</v>
+        <v>0.01993217108192795</v>
       </c>
       <c r="D44" s="33" t="n">
-        <v>0.0043742564999021</v>
+        <v>0.004374251895133492</v>
       </c>
       <c r="E44" s="9" t="n">
-        <v>0.111103666660798</v>
+        <v>0.1111036634617063</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>0.9800393733856876</v>
+        <v>0.9800394596124378</v>
       </c>
     </row>
     <row r="45">
@@ -3513,19 +3518,19 @@
         </is>
       </c>
       <c r="B45" s="12" t="n">
-        <v>0.2451136482795938</v>
+        <v>0.2451141804419785</v>
       </c>
       <c r="C45" s="34" t="n">
-        <v>0.01784709350445088</v>
+        <v>0.01784703629190622</v>
       </c>
       <c r="D45" s="34" t="n">
-        <v>0.004374566200062996</v>
+        <v>0.00437456167400884</v>
       </c>
       <c r="E45" s="12" t="n">
-        <v>0.1111115328715339</v>
+        <v>0.1111115316798015</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>0.8261569337194916</v>
+        <v>0.8261549596926778</v>
       </c>
     </row>
     <row r="46">
@@ -3535,19 +3540,19 @@
         </is>
       </c>
       <c r="B46" s="9" t="n">
-        <v>0.1447863145280247</v>
+        <v>0.1447859601512068</v>
       </c>
       <c r="C46" s="33" t="n">
-        <v>0.03021220785439191</v>
+        <v>0.03021225020406927</v>
       </c>
       <c r="D46" s="33" t="n">
-        <v>0.004374314228992046</v>
+        <v>0.004374309654124662</v>
       </c>
       <c r="E46" s="9" t="n">
-        <v>0.1111051329473695</v>
+        <v>0.1111051305092543</v>
       </c>
       <c r="F46" s="9" t="n">
-        <v>0.6542475904087065</v>
+        <v>0.654246587683997</v>
       </c>
     </row>
     <row r="47">
@@ -3557,19 +3562,19 @@
         </is>
       </c>
       <c r="B47" s="12" t="n">
-        <v>0.05237042256659726</v>
+        <v>0.05237036521179319</v>
       </c>
       <c r="C47" s="34" t="n">
-        <v>0.0835333836812642</v>
+        <v>0.08353339284924265</v>
       </c>
       <c r="D47" s="34" t="n">
-        <v>0.004374678601805506</v>
+        <v>0.004374674290895031</v>
       </c>
       <c r="E47" s="12" t="n">
-        <v>0.1111143878128781</v>
+        <v>0.1111143920886036</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>0.6432518675233434</v>
+        <v>0.6432517319898794</v>
       </c>
     </row>
     <row r="48">
@@ -3579,19 +3584,19 @@
         </is>
       </c>
       <c r="B48" s="9" t="n">
-        <v>0.0852010187298466</v>
+        <v>0.08520104981407732</v>
       </c>
       <c r="C48" s="33" t="n">
-        <v>0.05136020669527075</v>
+        <v>0.05136014188675325</v>
       </c>
       <c r="D48" s="33" t="n">
-        <v>0.004375941932612556</v>
+        <v>0.004375938007351343</v>
       </c>
       <c r="E48" s="9" t="n">
-        <v>0.1111464757082432</v>
+        <v>0.111146489812109</v>
       </c>
       <c r="F48" s="9" t="n">
-        <v>0.4913807456936256</v>
+        <v>0.4913808005382763</v>
       </c>
     </row>
     <row r="50">
@@ -3645,16 +3650,16 @@
         </is>
       </c>
       <c r="B52" s="9" t="n">
-        <v>0.0131031441029488</v>
+        <v>0.01310313745444653</v>
       </c>
       <c r="C52" s="33" t="n">
-        <v>0.03894766068625865</v>
+        <v>0.03894746836907385</v>
       </c>
       <c r="D52" s="33" t="n">
-        <v>0.0005103368104448009</v>
+        <v>0.0005103340315426829</v>
       </c>
       <c r="E52" s="9" t="n">
-        <v>0.01734019266614253</v>
+        <v>0.01734011091038029</v>
       </c>
       <c r="F52" s="9" t="n">
         <v>0.9718498340506939</v>
@@ -3667,19 +3672,19 @@
         </is>
       </c>
       <c r="B53" s="12" t="n">
-        <v>0.01889748360197973</v>
+        <v>0.01889748527636672</v>
       </c>
       <c r="C53" s="34" t="n">
-        <v>0.04139329986147902</v>
+        <v>0.04139305967161434</v>
       </c>
       <c r="D53" s="34" t="n">
-        <v>0.0007822292053641297</v>
+        <v>0.0007822247356881008</v>
       </c>
       <c r="E53" s="12" t="n">
-        <v>0.02657853568954868</v>
+        <v>0.02657840323262889</v>
       </c>
       <c r="F53" s="12" t="n">
-        <v>0.9005691996051071</v>
+        <v>0.9005692931844215</v>
       </c>
     </row>
     <row r="54">
@@ -3689,19 +3694,19 @@
         </is>
       </c>
       <c r="B54" s="9" t="n">
-        <v>0.008125992735504559</v>
+        <v>0.008125988522225262</v>
       </c>
       <c r="C54" s="33" t="n">
-        <v>0.03948168045054935</v>
+        <v>0.03948149543843042</v>
       </c>
       <c r="D54" s="33" t="n">
-        <v>0.0003208278485266763</v>
+        <v>0.0003208261787729745</v>
       </c>
       <c r="E54" s="9" t="n">
-        <v>0.01090106884758666</v>
+        <v>0.01090102007514579</v>
       </c>
       <c r="F54" s="9" t="n">
-        <v>0.8647854557196933</v>
+        <v>0.8647853697421607</v>
       </c>
     </row>
     <row r="55">
@@ -3711,19 +3716,19 @@
         </is>
       </c>
       <c r="B55" s="12" t="n">
-        <v>0.02978057137314431</v>
+        <v>0.02978060544931362</v>
       </c>
       <c r="C55" s="34" t="n">
-        <v>0.05471704480868797</v>
+        <v>0.05471677519182176</v>
       </c>
       <c r="D55" s="34" t="n">
-        <v>0.001629504858252668</v>
+        <v>0.001629498693446435</v>
       </c>
       <c r="E55" s="12" t="n">
-        <v>0.0553672155608159</v>
+        <v>0.05536704653473169</v>
       </c>
       <c r="F55" s="12" t="n">
-        <v>0.6547261440685357</v>
+        <v>0.654725765269208</v>
       </c>
     </row>
     <row r="56">
@@ -3733,19 +3738,19 @@
         </is>
       </c>
       <c r="B56" s="9" t="n">
-        <v>0.06443536846822434</v>
+        <v>0.06443562047933843</v>
       </c>
       <c r="C56" s="33" t="n">
-        <v>0.04035307816359169</v>
+        <v>0.04035314262922677</v>
       </c>
       <c r="D56" s="33" t="n">
-        <v>0.002600165460298088</v>
+        <v>0.002600179783605468</v>
       </c>
       <c r="E56" s="9" t="n">
-        <v>0.08834826162377085</v>
+        <v>0.0883488128321626</v>
       </c>
       <c r="F56" s="9" t="n">
-        <v>0.9800393733856876</v>
+        <v>0.9800394596124378</v>
       </c>
     </row>
     <row r="57">
@@ -3755,19 +3760,19 @@
         </is>
       </c>
       <c r="B57" s="12" t="n">
-        <v>0.6177098330959241</v>
+        <v>0.6177106857573594</v>
       </c>
       <c r="C57" s="34" t="n">
-        <v>0.02355606716845942</v>
+        <v>0.02355604513159771</v>
       </c>
       <c r="D57" s="34" t="n">
-        <v>0.01455081431902545</v>
+        <v>0.01455082079197053</v>
       </c>
       <c r="E57" s="12" t="n">
-        <v>0.4944066713926716</v>
+        <v>0.4944072524560491</v>
       </c>
       <c r="F57" s="12" t="n">
-        <v>0.8261569337194916</v>
+        <v>0.8261549596926778</v>
       </c>
     </row>
     <row r="58">
@@ -3777,19 +3782,19 @@
         </is>
       </c>
       <c r="B58" s="9" t="n">
-        <v>0.1996560638318086</v>
+        <v>0.1996548712353037</v>
       </c>
       <c r="C58" s="33" t="n">
-        <v>0.03480302416962155</v>
+        <v>0.03480311487371655</v>
       </c>
       <c r="D58" s="33" t="n">
-        <v>0.006948634815149939</v>
+        <v>0.006948611418699359</v>
       </c>
       <c r="E58" s="9" t="n">
-        <v>0.2361002851359047</v>
+        <v>0.2360996626251926</v>
       </c>
       <c r="F58" s="9" t="n">
-        <v>0.6542475904087065</v>
+        <v>0.654246587683997</v>
       </c>
     </row>
     <row r="59">
@@ -3799,19 +3804,19 @@
         </is>
       </c>
       <c r="B59" s="12" t="n">
-        <v>0.02725816753926526</v>
+        <v>0.02725821573980387</v>
       </c>
       <c r="C59" s="34" t="n">
-        <v>0.05923205736966428</v>
+        <v>0.05923194708907975</v>
       </c>
       <c r="D59" s="34" t="n">
-        <v>0.001614557343477681</v>
+        <v>0.001614557192442783</v>
       </c>
       <c r="E59" s="12" t="n">
-        <v>0.05485932982580027</v>
+        <v>0.0548593647644455</v>
       </c>
       <c r="F59" s="12" t="n">
-        <v>0.6432518675233434</v>
+        <v>0.6432517319898794</v>
       </c>
     </row>
     <row r="60">
@@ -3821,19 +3826,19 @@
         </is>
       </c>
       <c r="B60" s="9" t="n">
-        <v>0.02103337525120018</v>
+        <v>0.02103339008584262</v>
       </c>
       <c r="C60" s="33" t="n">
-        <v>0.02252567322576673</v>
+        <v>0.02252548320671542</v>
       </c>
       <c r="D60" s="33" t="n">
-        <v>0.0004737909377434645</v>
+        <v>0.0004737872751589424</v>
       </c>
       <c r="E60" s="9" t="n">
-        <v>0.01609843925775884</v>
+        <v>0.0160983265692635</v>
       </c>
       <c r="F60" s="9" t="n">
-        <v>0.4913807456936256</v>
+        <v>0.4913808005382763</v>
       </c>
     </row>
   </sheetData>
@@ -4291,7 +4296,7 @@
         </is>
       </c>
       <c r="C15" s="33" t="n">
-        <v>0.96360466770692</v>
+        <v>0.963604579887064</v>
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
@@ -4316,7 +4321,7 @@
         </is>
       </c>
       <c r="C16" s="34" t="n">
-        <v>0.9585938725922083</v>
+        <v>0.9585938857673019</v>
       </c>
       <c r="D16" s="22" t="inlineStr">
         <is>
@@ -4341,7 +4346,7 @@
         </is>
       </c>
       <c r="C17" s="33" t="n">
-        <v>0.9351150389158752</v>
+        <v>0.9351150145885929</v>
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
@@ -4366,7 +4371,7 @@
         </is>
       </c>
       <c r="C18" s="34" t="n">
-        <v>0.8153011671069538</v>
+        <v>0.8153008916507385</v>
       </c>
       <c r="D18" s="22" t="inlineStr">
         <is>
@@ -4391,7 +4396,7 @@
         </is>
       </c>
       <c r="C19" s="33" t="n">
-        <v>0.7921833148274291</v>
+        <v>0.7921827030700286</v>
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
@@ -4416,7 +4421,7 @@
         </is>
       </c>
       <c r="C20" s="34" t="n">
-        <v>0.756686346400972</v>
+        <v>0.7566863410399924</v>
       </c>
       <c r="D20" s="22" t="inlineStr">
         <is>
@@ -4441,7 +4446,7 @@
         </is>
       </c>
       <c r="C21" s="33" t="n">
-        <v>0.7550181047695816</v>
+        <v>0.7550185248134618</v>
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
@@ -4466,7 +4471,7 @@
         </is>
       </c>
       <c r="C22" s="34" t="n">
-        <v>0.7503301762560417</v>
+        <v>0.7503296960631181</v>
       </c>
       <c r="D22" s="22" t="inlineStr">
         <is>
@@ -4491,7 +4496,7 @@
         </is>
       </c>
       <c r="C23" s="33" t="n">
-        <v>0.7467845731139183</v>
+        <v>0.746784625795175</v>
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
@@ -4516,7 +4521,7 @@
         </is>
       </c>
       <c r="C24" s="34" t="n">
-        <v>0.6253590242908137</v>
+        <v>0.6253586382631419</v>
       </c>
       <c r="D24" s="22" t="inlineStr">
         <is>
@@ -4541,7 +4546,7 @@
         </is>
       </c>
       <c r="C25" s="33" t="n">
-        <v>0.6118581657309232</v>
+        <v>0.6118588409428388</v>
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
@@ -4566,7 +4571,7 @@
         </is>
       </c>
       <c r="C26" s="34" t="n">
-        <v>0.5930083533390097</v>
+        <v>0.5930074609613168</v>
       </c>
       <c r="D26" s="22" t="inlineStr">
         <is>
@@ -4591,7 +4596,7 @@
         </is>
       </c>
       <c r="C27" s="33" t="n">
-        <v>0.5532735406938195</v>
+        <v>0.5532735481847542</v>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
@@ -4616,7 +4621,7 @@
         </is>
       </c>
       <c r="C28" s="34" t="n">
-        <v>-0.5361296218117397</v>
+        <v>-0.5361309580009153</v>
       </c>
       <c r="D28" s="22" t="inlineStr">
         <is>
@@ -4641,7 +4646,7 @@
         </is>
       </c>
       <c r="C29" s="33" t="n">
-        <v>0.528597871691144</v>
+        <v>0.5286001691139169</v>
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
@@ -4731,19 +4736,19 @@
         </is>
       </c>
       <c r="B3" s="33" t="n">
-        <v>0.5927324628348662</v>
+        <v>0.5927327150397735</v>
       </c>
       <c r="C3" s="33" t="n">
-        <v>0.2495525907280696</v>
+        <v>0.2495523098663607</v>
       </c>
       <c r="D3" s="33" t="n">
-        <v>2.460423059424298</v>
+        <v>2.460418985371243</v>
       </c>
       <c r="E3" s="33" t="n">
-        <v>1.997183727022387</v>
+        <v>1.997176760310123</v>
       </c>
       <c r="F3" s="33" t="n">
-        <v>-0.02007599367985166</v>
+        <v>-0.02007623701015466</v>
       </c>
     </row>
     <row r="4">
@@ -4753,19 +4758,19 @@
         </is>
       </c>
       <c r="B4" s="34" t="n">
-        <v>0.6313816852499345</v>
+        <v>0.6313820183962096</v>
       </c>
       <c r="C4" s="34" t="n">
-        <v>0.3361744377105355</v>
+        <v>0.3361740654264061</v>
       </c>
       <c r="D4" s="34" t="n">
-        <v>2.146979762765747</v>
+        <v>2.146974527988826</v>
       </c>
       <c r="E4" s="34" t="n">
-        <v>0.3615968606782248</v>
+        <v>0.3615875557444018</v>
       </c>
       <c r="F4" s="34" t="n">
-        <v>-0.0261846790514917</v>
+        <v>-0.02618494416133161</v>
       </c>
     </row>
     <row r="5">
@@ -4775,19 +4780,19 @@
         </is>
       </c>
       <c r="B5" s="33" t="n">
-        <v>0.4597385026027135</v>
+        <v>0.4597377893280422</v>
       </c>
       <c r="C5" s="33" t="n">
-        <v>0.5803733430961843</v>
+        <v>0.580372581560643</v>
       </c>
       <c r="D5" s="33" t="n">
-        <v>2.856649546801769</v>
+        <v>2.856638421555682</v>
       </c>
       <c r="E5" s="33" t="n">
-        <v>0.02930984789698554</v>
+        <v>0.02933521107835607</v>
       </c>
       <c r="F5" s="33" t="n">
-        <v>-0.04492216535560389</v>
+        <v>-0.04492263039729934</v>
       </c>
     </row>
     <row r="6">
@@ -4797,19 +4802,19 @@
         </is>
       </c>
       <c r="B6" s="34" t="n">
-        <v>0.359180629674831</v>
+        <v>0.3591806160720604</v>
       </c>
       <c r="C6" s="34" t="n">
-        <v>0.4308581354864889</v>
+        <v>0.4308574963426787</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>1.337789206419006</v>
+        <v>1.337783775943102</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>2.361603006797575</v>
+        <v>2.361591902067863</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>-0.009980878555596838</v>
+        <v>-0.009981127111012841</v>
       </c>
     </row>
     <row r="7">
@@ -4819,19 +4824,19 @@
         </is>
       </c>
       <c r="B7" s="33" t="n">
-        <v>0.1620839697497295</v>
+        <v>0.162083582947631</v>
       </c>
       <c r="C7" s="33" t="n">
-        <v>0.4610386885106495</v>
+        <v>0.4610383070351105</v>
       </c>
       <c r="D7" s="33" t="n">
-        <v>0.5164427744334301</v>
+        <v>0.5164422089887049</v>
       </c>
       <c r="E7" s="33" t="n">
-        <v>4.113333203526983</v>
+        <v>4.113308307736573</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>-0.007163486376460381</v>
+        <v>-0.007163543705210864</v>
       </c>
     </row>
   </sheetData>

</xml_diff>